<commit_message>
Add before/after photo attachment sheet for corrective actions
Adds 지적사항_조치전후사진대지 sheet to 경영책임자_현장순회점검표.xlsx with
3 finding blocks, each pairing a 조치 전(Before)/조치 후(After) photo
placeholder with 지적사항 내용, 조치내용, 조치일자, and 확인자 fields, to
document corrective action evidence for patrol inspection findings.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SqkinqfGqqfBrcHRBkScVm
</commit_message>
<xml_diff>
--- a/templates/경영책임자_현장순회점검표.xlsx
+++ b/templates/경영책임자_현장순회점검표.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현장순회점검표" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사진대지" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="지적사항_조치전후사진대지" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'현장순회점검표'!$A$1:$AB$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'사진대지'!$A$1:$AB$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'지적사항_조치전후사진대지'!$A$1:$AB$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -136,6 +138,24 @@
       <color rgb="FF000000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="FFC00000"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="FF2E7D32"/>
+      <sz val="10.5"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -170,7 +190,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -323,11 +343,80 @@
         <color rgb="FFA6A6A6"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </right>
+      <top style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </right>
+      <top/>
+      <bottom style="dashed">
+        <color rgb="FFA6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -409,6 +498,28 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2082,32 +2193,6 @@
           <t>현장순회점검 사진대지</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
-      <c r="V2" s="2" t="n"/>
-      <c r="W2" s="2" t="n"/>
-      <c r="X2" s="2" t="n"/>
-      <c r="Y2" s="2" t="n"/>
-      <c r="Z2" s="2" t="n"/>
-      <c r="AA2" s="2" t="n"/>
-      <c r="AB2" s="2" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
@@ -2131,315 +2216,117 @@
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="C7" s="35" t="n"/>
-      <c r="D7" s="35" t="n"/>
-      <c r="E7" s="35" t="n"/>
-      <c r="F7" s="35" t="n"/>
-      <c r="G7" s="35" t="n"/>
-      <c r="H7" s="35" t="n"/>
-      <c r="I7" s="35" t="n"/>
-      <c r="J7" s="35" t="n"/>
-      <c r="K7" s="35" t="n"/>
-      <c r="L7" s="35" t="n"/>
-      <c r="M7" s="35" t="n"/>
-      <c r="N7" s="35" t="n"/>
+      <c r="C7" s="40" t="n"/>
+      <c r="D7" s="40" t="n"/>
+      <c r="E7" s="40" t="n"/>
+      <c r="F7" s="40" t="n"/>
+      <c r="G7" s="40" t="n"/>
+      <c r="H7" s="40" t="n"/>
+      <c r="I7" s="40" t="n"/>
+      <c r="J7" s="40" t="n"/>
+      <c r="K7" s="40" t="n"/>
+      <c r="L7" s="40" t="n"/>
+      <c r="M7" s="40" t="n"/>
+      <c r="N7" s="41" t="n"/>
       <c r="P7" s="34" t="inlineStr">
         <is>
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="Q7" s="35" t="n"/>
-      <c r="R7" s="35" t="n"/>
-      <c r="S7" s="35" t="n"/>
-      <c r="T7" s="35" t="n"/>
-      <c r="U7" s="35" t="n"/>
-      <c r="V7" s="35" t="n"/>
-      <c r="W7" s="35" t="n"/>
-      <c r="X7" s="35" t="n"/>
-      <c r="Y7" s="35" t="n"/>
-      <c r="Z7" s="35" t="n"/>
-      <c r="AA7" s="35" t="n"/>
-      <c r="AB7" s="35" t="n"/>
+      <c r="Q7" s="40" t="n"/>
+      <c r="R7" s="40" t="n"/>
+      <c r="S7" s="40" t="n"/>
+      <c r="T7" s="40" t="n"/>
+      <c r="U7" s="40" t="n"/>
+      <c r="V7" s="40" t="n"/>
+      <c r="W7" s="40" t="n"/>
+      <c r="X7" s="40" t="n"/>
+      <c r="Y7" s="40" t="n"/>
+      <c r="Z7" s="40" t="n"/>
+      <c r="AA7" s="40" t="n"/>
+      <c r="AB7" s="41" t="n"/>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="B8" s="35" t="n"/>
-      <c r="C8" s="35" t="n"/>
-      <c r="D8" s="35" t="n"/>
-      <c r="E8" s="35" t="n"/>
-      <c r="F8" s="35" t="n"/>
-      <c r="G8" s="35" t="n"/>
-      <c r="H8" s="35" t="n"/>
-      <c r="I8" s="35" t="n"/>
-      <c r="J8" s="35" t="n"/>
-      <c r="K8" s="35" t="n"/>
-      <c r="L8" s="35" t="n"/>
-      <c r="M8" s="35" t="n"/>
-      <c r="N8" s="35" t="n"/>
-      <c r="P8" s="35" t="n"/>
-      <c r="Q8" s="35" t="n"/>
-      <c r="R8" s="35" t="n"/>
-      <c r="S8" s="35" t="n"/>
-      <c r="T8" s="35" t="n"/>
-      <c r="U8" s="35" t="n"/>
-      <c r="V8" s="35" t="n"/>
-      <c r="W8" s="35" t="n"/>
-      <c r="X8" s="35" t="n"/>
-      <c r="Y8" s="35" t="n"/>
-      <c r="Z8" s="35" t="n"/>
-      <c r="AA8" s="35" t="n"/>
-      <c r="AB8" s="35" t="n"/>
+      <c r="B8" s="42" t="n"/>
+      <c r="N8" s="43" t="n"/>
+      <c r="P8" s="42" t="n"/>
+      <c r="AB8" s="43" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="B9" s="35" t="n"/>
-      <c r="C9" s="35" t="n"/>
-      <c r="D9" s="35" t="n"/>
-      <c r="E9" s="35" t="n"/>
-      <c r="F9" s="35" t="n"/>
-      <c r="G9" s="35" t="n"/>
-      <c r="H9" s="35" t="n"/>
-      <c r="I9" s="35" t="n"/>
-      <c r="J9" s="35" t="n"/>
-      <c r="K9" s="35" t="n"/>
-      <c r="L9" s="35" t="n"/>
-      <c r="M9" s="35" t="n"/>
-      <c r="N9" s="35" t="n"/>
-      <c r="P9" s="35" t="n"/>
-      <c r="Q9" s="35" t="n"/>
-      <c r="R9" s="35" t="n"/>
-      <c r="S9" s="35" t="n"/>
-      <c r="T9" s="35" t="n"/>
-      <c r="U9" s="35" t="n"/>
-      <c r="V9" s="35" t="n"/>
-      <c r="W9" s="35" t="n"/>
-      <c r="X9" s="35" t="n"/>
-      <c r="Y9" s="35" t="n"/>
-      <c r="Z9" s="35" t="n"/>
-      <c r="AA9" s="35" t="n"/>
-      <c r="AB9" s="35" t="n"/>
+      <c r="B9" s="42" t="n"/>
+      <c r="N9" s="43" t="n"/>
+      <c r="P9" s="42" t="n"/>
+      <c r="AB9" s="43" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="B10" s="35" t="n"/>
-      <c r="C10" s="35" t="n"/>
-      <c r="D10" s="35" t="n"/>
-      <c r="E10" s="35" t="n"/>
-      <c r="F10" s="35" t="n"/>
-      <c r="G10" s="35" t="n"/>
-      <c r="H10" s="35" t="n"/>
-      <c r="I10" s="35" t="n"/>
-      <c r="J10" s="35" t="n"/>
-      <c r="K10" s="35" t="n"/>
-      <c r="L10" s="35" t="n"/>
-      <c r="M10" s="35" t="n"/>
-      <c r="N10" s="35" t="n"/>
-      <c r="P10" s="35" t="n"/>
-      <c r="Q10" s="35" t="n"/>
-      <c r="R10" s="35" t="n"/>
-      <c r="S10" s="35" t="n"/>
-      <c r="T10" s="35" t="n"/>
-      <c r="U10" s="35" t="n"/>
-      <c r="V10" s="35" t="n"/>
-      <c r="W10" s="35" t="n"/>
-      <c r="X10" s="35" t="n"/>
-      <c r="Y10" s="35" t="n"/>
-      <c r="Z10" s="35" t="n"/>
-      <c r="AA10" s="35" t="n"/>
-      <c r="AB10" s="35" t="n"/>
+      <c r="B10" s="42" t="n"/>
+      <c r="N10" s="43" t="n"/>
+      <c r="P10" s="42" t="n"/>
+      <c r="AB10" s="43" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="B11" s="35" t="n"/>
-      <c r="C11" s="35" t="n"/>
-      <c r="D11" s="35" t="n"/>
-      <c r="E11" s="35" t="n"/>
-      <c r="F11" s="35" t="n"/>
-      <c r="G11" s="35" t="n"/>
-      <c r="H11" s="35" t="n"/>
-      <c r="I11" s="35" t="n"/>
-      <c r="J11" s="35" t="n"/>
-      <c r="K11" s="35" t="n"/>
-      <c r="L11" s="35" t="n"/>
-      <c r="M11" s="35" t="n"/>
-      <c r="N11" s="35" t="n"/>
-      <c r="P11" s="35" t="n"/>
-      <c r="Q11" s="35" t="n"/>
-      <c r="R11" s="35" t="n"/>
-      <c r="S11" s="35" t="n"/>
-      <c r="T11" s="35" t="n"/>
-      <c r="U11" s="35" t="n"/>
-      <c r="V11" s="35" t="n"/>
-      <c r="W11" s="35" t="n"/>
-      <c r="X11" s="35" t="n"/>
-      <c r="Y11" s="35" t="n"/>
-      <c r="Z11" s="35" t="n"/>
-      <c r="AA11" s="35" t="n"/>
-      <c r="AB11" s="35" t="n"/>
+      <c r="B11" s="42" t="n"/>
+      <c r="N11" s="43" t="n"/>
+      <c r="P11" s="42" t="n"/>
+      <c r="AB11" s="43" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="B12" s="35" t="n"/>
-      <c r="C12" s="35" t="n"/>
-      <c r="D12" s="35" t="n"/>
-      <c r="E12" s="35" t="n"/>
-      <c r="F12" s="35" t="n"/>
-      <c r="G12" s="35" t="n"/>
-      <c r="H12" s="35" t="n"/>
-      <c r="I12" s="35" t="n"/>
-      <c r="J12" s="35" t="n"/>
-      <c r="K12" s="35" t="n"/>
-      <c r="L12" s="35" t="n"/>
-      <c r="M12" s="35" t="n"/>
-      <c r="N12" s="35" t="n"/>
-      <c r="P12" s="35" t="n"/>
-      <c r="Q12" s="35" t="n"/>
-      <c r="R12" s="35" t="n"/>
-      <c r="S12" s="35" t="n"/>
-      <c r="T12" s="35" t="n"/>
-      <c r="U12" s="35" t="n"/>
-      <c r="V12" s="35" t="n"/>
-      <c r="W12" s="35" t="n"/>
-      <c r="X12" s="35" t="n"/>
-      <c r="Y12" s="35" t="n"/>
-      <c r="Z12" s="35" t="n"/>
-      <c r="AA12" s="35" t="n"/>
-      <c r="AB12" s="35" t="n"/>
+      <c r="B12" s="42" t="n"/>
+      <c r="N12" s="43" t="n"/>
+      <c r="P12" s="42" t="n"/>
+      <c r="AB12" s="43" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="35" t="n"/>
-      <c r="C13" s="35" t="n"/>
-      <c r="D13" s="35" t="n"/>
-      <c r="E13" s="35" t="n"/>
-      <c r="F13" s="35" t="n"/>
-      <c r="G13" s="35" t="n"/>
-      <c r="H13" s="35" t="n"/>
-      <c r="I13" s="35" t="n"/>
-      <c r="J13" s="35" t="n"/>
-      <c r="K13" s="35" t="n"/>
-      <c r="L13" s="35" t="n"/>
-      <c r="M13" s="35" t="n"/>
-      <c r="N13" s="35" t="n"/>
-      <c r="P13" s="35" t="n"/>
-      <c r="Q13" s="35" t="n"/>
-      <c r="R13" s="35" t="n"/>
-      <c r="S13" s="35" t="n"/>
-      <c r="T13" s="35" t="n"/>
-      <c r="U13" s="35" t="n"/>
-      <c r="V13" s="35" t="n"/>
-      <c r="W13" s="35" t="n"/>
-      <c r="X13" s="35" t="n"/>
-      <c r="Y13" s="35" t="n"/>
-      <c r="Z13" s="35" t="n"/>
-      <c r="AA13" s="35" t="n"/>
-      <c r="AB13" s="35" t="n"/>
+      <c r="B13" s="42" t="n"/>
+      <c r="N13" s="43" t="n"/>
+      <c r="P13" s="42" t="n"/>
+      <c r="AB13" s="43" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="B14" s="35" t="n"/>
-      <c r="C14" s="35" t="n"/>
-      <c r="D14" s="35" t="n"/>
-      <c r="E14" s="35" t="n"/>
-      <c r="F14" s="35" t="n"/>
-      <c r="G14" s="35" t="n"/>
-      <c r="H14" s="35" t="n"/>
-      <c r="I14" s="35" t="n"/>
-      <c r="J14" s="35" t="n"/>
-      <c r="K14" s="35" t="n"/>
-      <c r="L14" s="35" t="n"/>
-      <c r="M14" s="35" t="n"/>
-      <c r="N14" s="35" t="n"/>
-      <c r="P14" s="35" t="n"/>
-      <c r="Q14" s="35" t="n"/>
-      <c r="R14" s="35" t="n"/>
-      <c r="S14" s="35" t="n"/>
-      <c r="T14" s="35" t="n"/>
-      <c r="U14" s="35" t="n"/>
-      <c r="V14" s="35" t="n"/>
-      <c r="W14" s="35" t="n"/>
-      <c r="X14" s="35" t="n"/>
-      <c r="Y14" s="35" t="n"/>
-      <c r="Z14" s="35" t="n"/>
-      <c r="AA14" s="35" t="n"/>
-      <c r="AB14" s="35" t="n"/>
+      <c r="B14" s="42" t="n"/>
+      <c r="N14" s="43" t="n"/>
+      <c r="P14" s="42" t="n"/>
+      <c r="AB14" s="43" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="B15" s="35" t="n"/>
-      <c r="C15" s="35" t="n"/>
-      <c r="D15" s="35" t="n"/>
-      <c r="E15" s="35" t="n"/>
-      <c r="F15" s="35" t="n"/>
-      <c r="G15" s="35" t="n"/>
-      <c r="H15" s="35" t="n"/>
-      <c r="I15" s="35" t="n"/>
-      <c r="J15" s="35" t="n"/>
-      <c r="K15" s="35" t="n"/>
-      <c r="L15" s="35" t="n"/>
-      <c r="M15" s="35" t="n"/>
-      <c r="N15" s="35" t="n"/>
-      <c r="P15" s="35" t="n"/>
-      <c r="Q15" s="35" t="n"/>
-      <c r="R15" s="35" t="n"/>
-      <c r="S15" s="35" t="n"/>
-      <c r="T15" s="35" t="n"/>
-      <c r="U15" s="35" t="n"/>
-      <c r="V15" s="35" t="n"/>
-      <c r="W15" s="35" t="n"/>
-      <c r="X15" s="35" t="n"/>
-      <c r="Y15" s="35" t="n"/>
-      <c r="Z15" s="35" t="n"/>
-      <c r="AA15" s="35" t="n"/>
-      <c r="AB15" s="35" t="n"/>
+      <c r="B15" s="42" t="n"/>
+      <c r="N15" s="43" t="n"/>
+      <c r="P15" s="42" t="n"/>
+      <c r="AB15" s="43" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="B16" s="35" t="n"/>
-      <c r="C16" s="35" t="n"/>
-      <c r="D16" s="35" t="n"/>
-      <c r="E16" s="35" t="n"/>
-      <c r="F16" s="35" t="n"/>
-      <c r="G16" s="35" t="n"/>
-      <c r="H16" s="35" t="n"/>
-      <c r="I16" s="35" t="n"/>
-      <c r="J16" s="35" t="n"/>
-      <c r="K16" s="35" t="n"/>
-      <c r="L16" s="35" t="n"/>
-      <c r="M16" s="35" t="n"/>
-      <c r="N16" s="35" t="n"/>
-      <c r="P16" s="35" t="n"/>
-      <c r="Q16" s="35" t="n"/>
-      <c r="R16" s="35" t="n"/>
-      <c r="S16" s="35" t="n"/>
-      <c r="T16" s="35" t="n"/>
-      <c r="U16" s="35" t="n"/>
-      <c r="V16" s="35" t="n"/>
-      <c r="W16" s="35" t="n"/>
-      <c r="X16" s="35" t="n"/>
-      <c r="Y16" s="35" t="n"/>
-      <c r="Z16" s="35" t="n"/>
-      <c r="AA16" s="35" t="n"/>
-      <c r="AB16" s="35" t="n"/>
+      <c r="B16" s="42" t="n"/>
+      <c r="N16" s="43" t="n"/>
+      <c r="P16" s="42" t="n"/>
+      <c r="AB16" s="43" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="B17" s="35" t="n"/>
-      <c r="C17" s="35" t="n"/>
-      <c r="D17" s="35" t="n"/>
-      <c r="E17" s="35" t="n"/>
-      <c r="F17" s="35" t="n"/>
-      <c r="G17" s="35" t="n"/>
-      <c r="H17" s="35" t="n"/>
-      <c r="I17" s="35" t="n"/>
-      <c r="J17" s="35" t="n"/>
-      <c r="K17" s="35" t="n"/>
-      <c r="L17" s="35" t="n"/>
-      <c r="M17" s="35" t="n"/>
-      <c r="N17" s="35" t="n"/>
-      <c r="P17" s="35" t="n"/>
-      <c r="Q17" s="35" t="n"/>
-      <c r="R17" s="35" t="n"/>
-      <c r="S17" s="35" t="n"/>
-      <c r="T17" s="35" t="n"/>
-      <c r="U17" s="35" t="n"/>
-      <c r="V17" s="35" t="n"/>
-      <c r="W17" s="35" t="n"/>
-      <c r="X17" s="35" t="n"/>
-      <c r="Y17" s="35" t="n"/>
-      <c r="Z17" s="35" t="n"/>
-      <c r="AA17" s="35" t="n"/>
-      <c r="AB17" s="35" t="n"/>
+      <c r="B17" s="44" t="n"/>
+      <c r="C17" s="45" t="n"/>
+      <c r="D17" s="45" t="n"/>
+      <c r="E17" s="45" t="n"/>
+      <c r="F17" s="45" t="n"/>
+      <c r="G17" s="45" t="n"/>
+      <c r="H17" s="45" t="n"/>
+      <c r="I17" s="45" t="n"/>
+      <c r="J17" s="45" t="n"/>
+      <c r="K17" s="45" t="n"/>
+      <c r="L17" s="45" t="n"/>
+      <c r="M17" s="45" t="n"/>
+      <c r="N17" s="46" t="n"/>
+      <c r="P17" s="44" t="n"/>
+      <c r="Q17" s="45" t="n"/>
+      <c r="R17" s="45" t="n"/>
+      <c r="S17" s="45" t="n"/>
+      <c r="T17" s="45" t="n"/>
+      <c r="U17" s="45" t="n"/>
+      <c r="V17" s="45" t="n"/>
+      <c r="W17" s="45" t="n"/>
+      <c r="X17" s="45" t="n"/>
+      <c r="Y17" s="45" t="n"/>
+      <c r="Z17" s="45" t="n"/>
+      <c r="AA17" s="45" t="n"/>
+      <c r="AB17" s="46" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="36" t="inlineStr">
@@ -2447,40 +2334,40 @@
           <t>사진 1</t>
         </is>
       </c>
-      <c r="C18" s="19" t="n"/>
-      <c r="D18" s="19" t="n"/>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="23" t="n"/>
       <c r="E18" s="37" t="inlineStr">
         <is>
           <t>위치</t>
         </is>
       </c>
-      <c r="F18" s="19" t="n"/>
-      <c r="G18" s="19" t="n"/>
+      <c r="F18" s="22" t="n"/>
+      <c r="G18" s="23" t="n"/>
       <c r="H18" s="38" t="inlineStr"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
+      <c r="I18" s="22" t="n"/>
+      <c r="J18" s="22" t="n"/>
+      <c r="K18" s="23" t="n"/>
       <c r="P18" s="36" t="inlineStr">
         <is>
           <t>사진 2</t>
         </is>
       </c>
-      <c r="Q18" s="19" t="n"/>
-      <c r="R18" s="19" t="n"/>
+      <c r="Q18" s="22" t="n"/>
+      <c r="R18" s="23" t="n"/>
       <c r="S18" s="37" t="inlineStr">
         <is>
           <t>위치</t>
         </is>
       </c>
-      <c r="T18" s="19" t="n"/>
-      <c r="U18" s="19" t="n"/>
+      <c r="T18" s="22" t="n"/>
+      <c r="U18" s="23" t="n"/>
       <c r="V18" s="38" t="inlineStr"/>
-      <c r="W18" s="7" t="n"/>
-      <c r="X18" s="7" t="n"/>
-      <c r="Y18" s="7" t="n"/>
-      <c r="Z18" s="7" t="n"/>
-      <c r="AA18" s="7" t="n"/>
-      <c r="AB18" s="7" t="n"/>
+      <c r="W18" s="22" t="n"/>
+      <c r="X18" s="22" t="n"/>
+      <c r="Y18" s="22" t="n"/>
+      <c r="Z18" s="22" t="n"/>
+      <c r="AA18" s="22" t="n"/>
+      <c r="AB18" s="23" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="B19" s="37" t="inlineStr">
@@ -2488,63 +2375,63 @@
           <t>내용</t>
         </is>
       </c>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="19" t="n"/>
+      <c r="C19" s="26" t="n"/>
+      <c r="D19" s="27" t="n"/>
       <c r="E19" s="39" t="inlineStr"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="7" t="n"/>
-      <c r="J19" s="7" t="n"/>
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
-      <c r="N19" s="7" t="n"/>
+      <c r="F19" s="26" t="n"/>
+      <c r="G19" s="26" t="n"/>
+      <c r="H19" s="26" t="n"/>
+      <c r="I19" s="26" t="n"/>
+      <c r="J19" s="26" t="n"/>
+      <c r="K19" s="26" t="n"/>
+      <c r="L19" s="26" t="n"/>
+      <c r="M19" s="26" t="n"/>
+      <c r="N19" s="27" t="n"/>
       <c r="P19" s="37" t="inlineStr">
         <is>
           <t>내용</t>
         </is>
       </c>
-      <c r="Q19" s="19" t="n"/>
-      <c r="R19" s="19" t="n"/>
+      <c r="Q19" s="26" t="n"/>
+      <c r="R19" s="27" t="n"/>
       <c r="S19" s="39" t="inlineStr"/>
-      <c r="T19" s="7" t="n"/>
-      <c r="U19" s="7" t="n"/>
-      <c r="V19" s="7" t="n"/>
-      <c r="W19" s="7" t="n"/>
-      <c r="X19" s="7" t="n"/>
-      <c r="Y19" s="7" t="n"/>
-      <c r="Z19" s="7" t="n"/>
-      <c r="AA19" s="7" t="n"/>
-      <c r="AB19" s="7" t="n"/>
+      <c r="T19" s="26" t="n"/>
+      <c r="U19" s="26" t="n"/>
+      <c r="V19" s="26" t="n"/>
+      <c r="W19" s="26" t="n"/>
+      <c r="X19" s="26" t="n"/>
+      <c r="Y19" s="26" t="n"/>
+      <c r="Z19" s="26" t="n"/>
+      <c r="AA19" s="26" t="n"/>
+      <c r="AB19" s="27" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="B20" s="19" t="n"/>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="n"/>
-      <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
-      <c r="P20" s="19" t="n"/>
-      <c r="Q20" s="19" t="n"/>
-      <c r="R20" s="19" t="n"/>
-      <c r="S20" s="7" t="n"/>
-      <c r="T20" s="7" t="n"/>
-      <c r="U20" s="7" t="n"/>
-      <c r="V20" s="7" t="n"/>
-      <c r="W20" s="7" t="n"/>
-      <c r="X20" s="7" t="n"/>
-      <c r="Y20" s="7" t="n"/>
-      <c r="Z20" s="7" t="n"/>
-      <c r="AA20" s="7" t="n"/>
-      <c r="AB20" s="7" t="n"/>
+      <c r="B20" s="30" t="n"/>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="30" t="n"/>
+      <c r="F20" s="31" t="n"/>
+      <c r="G20" s="31" t="n"/>
+      <c r="H20" s="31" t="n"/>
+      <c r="I20" s="31" t="n"/>
+      <c r="J20" s="31" t="n"/>
+      <c r="K20" s="31" t="n"/>
+      <c r="L20" s="31" t="n"/>
+      <c r="M20" s="31" t="n"/>
+      <c r="N20" s="32" t="n"/>
+      <c r="P20" s="30" t="n"/>
+      <c r="Q20" s="31" t="n"/>
+      <c r="R20" s="32" t="n"/>
+      <c r="S20" s="30" t="n"/>
+      <c r="T20" s="31" t="n"/>
+      <c r="U20" s="31" t="n"/>
+      <c r="V20" s="31" t="n"/>
+      <c r="W20" s="31" t="n"/>
+      <c r="X20" s="31" t="n"/>
+      <c r="Y20" s="31" t="n"/>
+      <c r="Z20" s="31" t="n"/>
+      <c r="AA20" s="31" t="n"/>
+      <c r="AB20" s="32" t="n"/>
     </row>
     <row r="21" ht="10" customHeight="1"/>
     <row r="22" ht="16" customHeight="1">
@@ -2553,315 +2440,117 @@
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="C22" s="35" t="n"/>
-      <c r="D22" s="35" t="n"/>
-      <c r="E22" s="35" t="n"/>
-      <c r="F22" s="35" t="n"/>
-      <c r="G22" s="35" t="n"/>
-      <c r="H22" s="35" t="n"/>
-      <c r="I22" s="35" t="n"/>
-      <c r="J22" s="35" t="n"/>
-      <c r="K22" s="35" t="n"/>
-      <c r="L22" s="35" t="n"/>
-      <c r="M22" s="35" t="n"/>
-      <c r="N22" s="35" t="n"/>
+      <c r="C22" s="40" t="n"/>
+      <c r="D22" s="40" t="n"/>
+      <c r="E22" s="40" t="n"/>
+      <c r="F22" s="40" t="n"/>
+      <c r="G22" s="40" t="n"/>
+      <c r="H22" s="40" t="n"/>
+      <c r="I22" s="40" t="n"/>
+      <c r="J22" s="40" t="n"/>
+      <c r="K22" s="40" t="n"/>
+      <c r="L22" s="40" t="n"/>
+      <c r="M22" s="40" t="n"/>
+      <c r="N22" s="41" t="n"/>
       <c r="P22" s="34" t="inlineStr">
         <is>
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="Q22" s="35" t="n"/>
-      <c r="R22" s="35" t="n"/>
-      <c r="S22" s="35" t="n"/>
-      <c r="T22" s="35" t="n"/>
-      <c r="U22" s="35" t="n"/>
-      <c r="V22" s="35" t="n"/>
-      <c r="W22" s="35" t="n"/>
-      <c r="X22" s="35" t="n"/>
-      <c r="Y22" s="35" t="n"/>
-      <c r="Z22" s="35" t="n"/>
-      <c r="AA22" s="35" t="n"/>
-      <c r="AB22" s="35" t="n"/>
+      <c r="Q22" s="40" t="n"/>
+      <c r="R22" s="40" t="n"/>
+      <c r="S22" s="40" t="n"/>
+      <c r="T22" s="40" t="n"/>
+      <c r="U22" s="40" t="n"/>
+      <c r="V22" s="40" t="n"/>
+      <c r="W22" s="40" t="n"/>
+      <c r="X22" s="40" t="n"/>
+      <c r="Y22" s="40" t="n"/>
+      <c r="Z22" s="40" t="n"/>
+      <c r="AA22" s="40" t="n"/>
+      <c r="AB22" s="41" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="B23" s="35" t="n"/>
-      <c r="C23" s="35" t="n"/>
-      <c r="D23" s="35" t="n"/>
-      <c r="E23" s="35" t="n"/>
-      <c r="F23" s="35" t="n"/>
-      <c r="G23" s="35" t="n"/>
-      <c r="H23" s="35" t="n"/>
-      <c r="I23" s="35" t="n"/>
-      <c r="J23" s="35" t="n"/>
-      <c r="K23" s="35" t="n"/>
-      <c r="L23" s="35" t="n"/>
-      <c r="M23" s="35" t="n"/>
-      <c r="N23" s="35" t="n"/>
-      <c r="P23" s="35" t="n"/>
-      <c r="Q23" s="35" t="n"/>
-      <c r="R23" s="35" t="n"/>
-      <c r="S23" s="35" t="n"/>
-      <c r="T23" s="35" t="n"/>
-      <c r="U23" s="35" t="n"/>
-      <c r="V23" s="35" t="n"/>
-      <c r="W23" s="35" t="n"/>
-      <c r="X23" s="35" t="n"/>
-      <c r="Y23" s="35" t="n"/>
-      <c r="Z23" s="35" t="n"/>
-      <c r="AA23" s="35" t="n"/>
-      <c r="AB23" s="35" t="n"/>
+      <c r="B23" s="42" t="n"/>
+      <c r="N23" s="43" t="n"/>
+      <c r="P23" s="42" t="n"/>
+      <c r="AB23" s="43" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="B24" s="35" t="n"/>
-      <c r="C24" s="35" t="n"/>
-      <c r="D24" s="35" t="n"/>
-      <c r="E24" s="35" t="n"/>
-      <c r="F24" s="35" t="n"/>
-      <c r="G24" s="35" t="n"/>
-      <c r="H24" s="35" t="n"/>
-      <c r="I24" s="35" t="n"/>
-      <c r="J24" s="35" t="n"/>
-      <c r="K24" s="35" t="n"/>
-      <c r="L24" s="35" t="n"/>
-      <c r="M24" s="35" t="n"/>
-      <c r="N24" s="35" t="n"/>
-      <c r="P24" s="35" t="n"/>
-      <c r="Q24" s="35" t="n"/>
-      <c r="R24" s="35" t="n"/>
-      <c r="S24" s="35" t="n"/>
-      <c r="T24" s="35" t="n"/>
-      <c r="U24" s="35" t="n"/>
-      <c r="V24" s="35" t="n"/>
-      <c r="W24" s="35" t="n"/>
-      <c r="X24" s="35" t="n"/>
-      <c r="Y24" s="35" t="n"/>
-      <c r="Z24" s="35" t="n"/>
-      <c r="AA24" s="35" t="n"/>
-      <c r="AB24" s="35" t="n"/>
+      <c r="B24" s="42" t="n"/>
+      <c r="N24" s="43" t="n"/>
+      <c r="P24" s="42" t="n"/>
+      <c r="AB24" s="43" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="B25" s="35" t="n"/>
-      <c r="C25" s="35" t="n"/>
-      <c r="D25" s="35" t="n"/>
-      <c r="E25" s="35" t="n"/>
-      <c r="F25" s="35" t="n"/>
-      <c r="G25" s="35" t="n"/>
-      <c r="H25" s="35" t="n"/>
-      <c r="I25" s="35" t="n"/>
-      <c r="J25" s="35" t="n"/>
-      <c r="K25" s="35" t="n"/>
-      <c r="L25" s="35" t="n"/>
-      <c r="M25" s="35" t="n"/>
-      <c r="N25" s="35" t="n"/>
-      <c r="P25" s="35" t="n"/>
-      <c r="Q25" s="35" t="n"/>
-      <c r="R25" s="35" t="n"/>
-      <c r="S25" s="35" t="n"/>
-      <c r="T25" s="35" t="n"/>
-      <c r="U25" s="35" t="n"/>
-      <c r="V25" s="35" t="n"/>
-      <c r="W25" s="35" t="n"/>
-      <c r="X25" s="35" t="n"/>
-      <c r="Y25" s="35" t="n"/>
-      <c r="Z25" s="35" t="n"/>
-      <c r="AA25" s="35" t="n"/>
-      <c r="AB25" s="35" t="n"/>
+      <c r="B25" s="42" t="n"/>
+      <c r="N25" s="43" t="n"/>
+      <c r="P25" s="42" t="n"/>
+      <c r="AB25" s="43" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="B26" s="35" t="n"/>
-      <c r="C26" s="35" t="n"/>
-      <c r="D26" s="35" t="n"/>
-      <c r="E26" s="35" t="n"/>
-      <c r="F26" s="35" t="n"/>
-      <c r="G26" s="35" t="n"/>
-      <c r="H26" s="35" t="n"/>
-      <c r="I26" s="35" t="n"/>
-      <c r="J26" s="35" t="n"/>
-      <c r="K26" s="35" t="n"/>
-      <c r="L26" s="35" t="n"/>
-      <c r="M26" s="35" t="n"/>
-      <c r="N26" s="35" t="n"/>
-      <c r="P26" s="35" t="n"/>
-      <c r="Q26" s="35" t="n"/>
-      <c r="R26" s="35" t="n"/>
-      <c r="S26" s="35" t="n"/>
-      <c r="T26" s="35" t="n"/>
-      <c r="U26" s="35" t="n"/>
-      <c r="V26" s="35" t="n"/>
-      <c r="W26" s="35" t="n"/>
-      <c r="X26" s="35" t="n"/>
-      <c r="Y26" s="35" t="n"/>
-      <c r="Z26" s="35" t="n"/>
-      <c r="AA26" s="35" t="n"/>
-      <c r="AB26" s="35" t="n"/>
+      <c r="B26" s="42" t="n"/>
+      <c r="N26" s="43" t="n"/>
+      <c r="P26" s="42" t="n"/>
+      <c r="AB26" s="43" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="B27" s="35" t="n"/>
-      <c r="C27" s="35" t="n"/>
-      <c r="D27" s="35" t="n"/>
-      <c r="E27" s="35" t="n"/>
-      <c r="F27" s="35" t="n"/>
-      <c r="G27" s="35" t="n"/>
-      <c r="H27" s="35" t="n"/>
-      <c r="I27" s="35" t="n"/>
-      <c r="J27" s="35" t="n"/>
-      <c r="K27" s="35" t="n"/>
-      <c r="L27" s="35" t="n"/>
-      <c r="M27" s="35" t="n"/>
-      <c r="N27" s="35" t="n"/>
-      <c r="P27" s="35" t="n"/>
-      <c r="Q27" s="35" t="n"/>
-      <c r="R27" s="35" t="n"/>
-      <c r="S27" s="35" t="n"/>
-      <c r="T27" s="35" t="n"/>
-      <c r="U27" s="35" t="n"/>
-      <c r="V27" s="35" t="n"/>
-      <c r="W27" s="35" t="n"/>
-      <c r="X27" s="35" t="n"/>
-      <c r="Y27" s="35" t="n"/>
-      <c r="Z27" s="35" t="n"/>
-      <c r="AA27" s="35" t="n"/>
-      <c r="AB27" s="35" t="n"/>
+      <c r="B27" s="42" t="n"/>
+      <c r="N27" s="43" t="n"/>
+      <c r="P27" s="42" t="n"/>
+      <c r="AB27" s="43" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="35" t="n"/>
-      <c r="C28" s="35" t="n"/>
-      <c r="D28" s="35" t="n"/>
-      <c r="E28" s="35" t="n"/>
-      <c r="F28" s="35" t="n"/>
-      <c r="G28" s="35" t="n"/>
-      <c r="H28" s="35" t="n"/>
-      <c r="I28" s="35" t="n"/>
-      <c r="J28" s="35" t="n"/>
-      <c r="K28" s="35" t="n"/>
-      <c r="L28" s="35" t="n"/>
-      <c r="M28" s="35" t="n"/>
-      <c r="N28" s="35" t="n"/>
-      <c r="P28" s="35" t="n"/>
-      <c r="Q28" s="35" t="n"/>
-      <c r="R28" s="35" t="n"/>
-      <c r="S28" s="35" t="n"/>
-      <c r="T28" s="35" t="n"/>
-      <c r="U28" s="35" t="n"/>
-      <c r="V28" s="35" t="n"/>
-      <c r="W28" s="35" t="n"/>
-      <c r="X28" s="35" t="n"/>
-      <c r="Y28" s="35" t="n"/>
-      <c r="Z28" s="35" t="n"/>
-      <c r="AA28" s="35" t="n"/>
-      <c r="AB28" s="35" t="n"/>
+      <c r="B28" s="42" t="n"/>
+      <c r="N28" s="43" t="n"/>
+      <c r="P28" s="42" t="n"/>
+      <c r="AB28" s="43" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="B29" s="35" t="n"/>
-      <c r="C29" s="35" t="n"/>
-      <c r="D29" s="35" t="n"/>
-      <c r="E29" s="35" t="n"/>
-      <c r="F29" s="35" t="n"/>
-      <c r="G29" s="35" t="n"/>
-      <c r="H29" s="35" t="n"/>
-      <c r="I29" s="35" t="n"/>
-      <c r="J29" s="35" t="n"/>
-      <c r="K29" s="35" t="n"/>
-      <c r="L29" s="35" t="n"/>
-      <c r="M29" s="35" t="n"/>
-      <c r="N29" s="35" t="n"/>
-      <c r="P29" s="35" t="n"/>
-      <c r="Q29" s="35" t="n"/>
-      <c r="R29" s="35" t="n"/>
-      <c r="S29" s="35" t="n"/>
-      <c r="T29" s="35" t="n"/>
-      <c r="U29" s="35" t="n"/>
-      <c r="V29" s="35" t="n"/>
-      <c r="W29" s="35" t="n"/>
-      <c r="X29" s="35" t="n"/>
-      <c r="Y29" s="35" t="n"/>
-      <c r="Z29" s="35" t="n"/>
-      <c r="AA29" s="35" t="n"/>
-      <c r="AB29" s="35" t="n"/>
+      <c r="B29" s="42" t="n"/>
+      <c r="N29" s="43" t="n"/>
+      <c r="P29" s="42" t="n"/>
+      <c r="AB29" s="43" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="B30" s="35" t="n"/>
-      <c r="C30" s="35" t="n"/>
-      <c r="D30" s="35" t="n"/>
-      <c r="E30" s="35" t="n"/>
-      <c r="F30" s="35" t="n"/>
-      <c r="G30" s="35" t="n"/>
-      <c r="H30" s="35" t="n"/>
-      <c r="I30" s="35" t="n"/>
-      <c r="J30" s="35" t="n"/>
-      <c r="K30" s="35" t="n"/>
-      <c r="L30" s="35" t="n"/>
-      <c r="M30" s="35" t="n"/>
-      <c r="N30" s="35" t="n"/>
-      <c r="P30" s="35" t="n"/>
-      <c r="Q30" s="35" t="n"/>
-      <c r="R30" s="35" t="n"/>
-      <c r="S30" s="35" t="n"/>
-      <c r="T30" s="35" t="n"/>
-      <c r="U30" s="35" t="n"/>
-      <c r="V30" s="35" t="n"/>
-      <c r="W30" s="35" t="n"/>
-      <c r="X30" s="35" t="n"/>
-      <c r="Y30" s="35" t="n"/>
-      <c r="Z30" s="35" t="n"/>
-      <c r="AA30" s="35" t="n"/>
-      <c r="AB30" s="35" t="n"/>
+      <c r="B30" s="42" t="n"/>
+      <c r="N30" s="43" t="n"/>
+      <c r="P30" s="42" t="n"/>
+      <c r="AB30" s="43" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="B31" s="35" t="n"/>
-      <c r="C31" s="35" t="n"/>
-      <c r="D31" s="35" t="n"/>
-      <c r="E31" s="35" t="n"/>
-      <c r="F31" s="35" t="n"/>
-      <c r="G31" s="35" t="n"/>
-      <c r="H31" s="35" t="n"/>
-      <c r="I31" s="35" t="n"/>
-      <c r="J31" s="35" t="n"/>
-      <c r="K31" s="35" t="n"/>
-      <c r="L31" s="35" t="n"/>
-      <c r="M31" s="35" t="n"/>
-      <c r="N31" s="35" t="n"/>
-      <c r="P31" s="35" t="n"/>
-      <c r="Q31" s="35" t="n"/>
-      <c r="R31" s="35" t="n"/>
-      <c r="S31" s="35" t="n"/>
-      <c r="T31" s="35" t="n"/>
-      <c r="U31" s="35" t="n"/>
-      <c r="V31" s="35" t="n"/>
-      <c r="W31" s="35" t="n"/>
-      <c r="X31" s="35" t="n"/>
-      <c r="Y31" s="35" t="n"/>
-      <c r="Z31" s="35" t="n"/>
-      <c r="AA31" s="35" t="n"/>
-      <c r="AB31" s="35" t="n"/>
+      <c r="B31" s="42" t="n"/>
+      <c r="N31" s="43" t="n"/>
+      <c r="P31" s="42" t="n"/>
+      <c r="AB31" s="43" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="35" t="n"/>
-      <c r="C32" s="35" t="n"/>
-      <c r="D32" s="35" t="n"/>
-      <c r="E32" s="35" t="n"/>
-      <c r="F32" s="35" t="n"/>
-      <c r="G32" s="35" t="n"/>
-      <c r="H32" s="35" t="n"/>
-      <c r="I32" s="35" t="n"/>
-      <c r="J32" s="35" t="n"/>
-      <c r="K32" s="35" t="n"/>
-      <c r="L32" s="35" t="n"/>
-      <c r="M32" s="35" t="n"/>
-      <c r="N32" s="35" t="n"/>
-      <c r="P32" s="35" t="n"/>
-      <c r="Q32" s="35" t="n"/>
-      <c r="R32" s="35" t="n"/>
-      <c r="S32" s="35" t="n"/>
-      <c r="T32" s="35" t="n"/>
-      <c r="U32" s="35" t="n"/>
-      <c r="V32" s="35" t="n"/>
-      <c r="W32" s="35" t="n"/>
-      <c r="X32" s="35" t="n"/>
-      <c r="Y32" s="35" t="n"/>
-      <c r="Z32" s="35" t="n"/>
-      <c r="AA32" s="35" t="n"/>
-      <c r="AB32" s="35" t="n"/>
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="45" t="n"/>
+      <c r="I32" s="45" t="n"/>
+      <c r="J32" s="45" t="n"/>
+      <c r="K32" s="45" t="n"/>
+      <c r="L32" s="45" t="n"/>
+      <c r="M32" s="45" t="n"/>
+      <c r="N32" s="46" t="n"/>
+      <c r="P32" s="44" t="n"/>
+      <c r="Q32" s="45" t="n"/>
+      <c r="R32" s="45" t="n"/>
+      <c r="S32" s="45" t="n"/>
+      <c r="T32" s="45" t="n"/>
+      <c r="U32" s="45" t="n"/>
+      <c r="V32" s="45" t="n"/>
+      <c r="W32" s="45" t="n"/>
+      <c r="X32" s="45" t="n"/>
+      <c r="Y32" s="45" t="n"/>
+      <c r="Z32" s="45" t="n"/>
+      <c r="AA32" s="45" t="n"/>
+      <c r="AB32" s="46" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="36" t="inlineStr">
@@ -2869,40 +2558,40 @@
           <t>사진 3</t>
         </is>
       </c>
-      <c r="C33" s="19" t="n"/>
-      <c r="D33" s="19" t="n"/>
+      <c r="C33" s="22" t="n"/>
+      <c r="D33" s="23" t="n"/>
       <c r="E33" s="37" t="inlineStr">
         <is>
           <t>위치</t>
         </is>
       </c>
-      <c r="F33" s="19" t="n"/>
-      <c r="G33" s="19" t="n"/>
+      <c r="F33" s="22" t="n"/>
+      <c r="G33" s="23" t="n"/>
       <c r="H33" s="38" t="inlineStr"/>
-      <c r="I33" s="7" t="n"/>
-      <c r="J33" s="7" t="n"/>
-      <c r="K33" s="7" t="n"/>
+      <c r="I33" s="22" t="n"/>
+      <c r="J33" s="22" t="n"/>
+      <c r="K33" s="23" t="n"/>
       <c r="P33" s="36" t="inlineStr">
         <is>
           <t>사진 4</t>
         </is>
       </c>
-      <c r="Q33" s="19" t="n"/>
-      <c r="R33" s="19" t="n"/>
+      <c r="Q33" s="22" t="n"/>
+      <c r="R33" s="23" t="n"/>
       <c r="S33" s="37" t="inlineStr">
         <is>
           <t>위치</t>
         </is>
       </c>
-      <c r="T33" s="19" t="n"/>
-      <c r="U33" s="19" t="n"/>
+      <c r="T33" s="22" t="n"/>
+      <c r="U33" s="23" t="n"/>
       <c r="V33" s="38" t="inlineStr"/>
-      <c r="W33" s="7" t="n"/>
-      <c r="X33" s="7" t="n"/>
-      <c r="Y33" s="7" t="n"/>
-      <c r="Z33" s="7" t="n"/>
-      <c r="AA33" s="7" t="n"/>
-      <c r="AB33" s="7" t="n"/>
+      <c r="W33" s="22" t="n"/>
+      <c r="X33" s="22" t="n"/>
+      <c r="Y33" s="22" t="n"/>
+      <c r="Z33" s="22" t="n"/>
+      <c r="AA33" s="22" t="n"/>
+      <c r="AB33" s="23" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="B34" s="37" t="inlineStr">
@@ -2910,63 +2599,63 @@
           <t>내용</t>
         </is>
       </c>
-      <c r="C34" s="19" t="n"/>
-      <c r="D34" s="19" t="n"/>
+      <c r="C34" s="26" t="n"/>
+      <c r="D34" s="27" t="n"/>
       <c r="E34" s="39" t="inlineStr"/>
-      <c r="F34" s="7" t="n"/>
-      <c r="G34" s="7" t="n"/>
-      <c r="H34" s="7" t="n"/>
-      <c r="I34" s="7" t="n"/>
-      <c r="J34" s="7" t="n"/>
-      <c r="K34" s="7" t="n"/>
-      <c r="L34" s="7" t="n"/>
-      <c r="M34" s="7" t="n"/>
-      <c r="N34" s="7" t="n"/>
+      <c r="F34" s="26" t="n"/>
+      <c r="G34" s="26" t="n"/>
+      <c r="H34" s="26" t="n"/>
+      <c r="I34" s="26" t="n"/>
+      <c r="J34" s="26" t="n"/>
+      <c r="K34" s="26" t="n"/>
+      <c r="L34" s="26" t="n"/>
+      <c r="M34" s="26" t="n"/>
+      <c r="N34" s="27" t="n"/>
       <c r="P34" s="37" t="inlineStr">
         <is>
           <t>내용</t>
         </is>
       </c>
-      <c r="Q34" s="19" t="n"/>
-      <c r="R34" s="19" t="n"/>
+      <c r="Q34" s="26" t="n"/>
+      <c r="R34" s="27" t="n"/>
       <c r="S34" s="39" t="inlineStr"/>
-      <c r="T34" s="7" t="n"/>
-      <c r="U34" s="7" t="n"/>
-      <c r="V34" s="7" t="n"/>
-      <c r="W34" s="7" t="n"/>
-      <c r="X34" s="7" t="n"/>
-      <c r="Y34" s="7" t="n"/>
-      <c r="Z34" s="7" t="n"/>
-      <c r="AA34" s="7" t="n"/>
-      <c r="AB34" s="7" t="n"/>
+      <c r="T34" s="26" t="n"/>
+      <c r="U34" s="26" t="n"/>
+      <c r="V34" s="26" t="n"/>
+      <c r="W34" s="26" t="n"/>
+      <c r="X34" s="26" t="n"/>
+      <c r="Y34" s="26" t="n"/>
+      <c r="Z34" s="26" t="n"/>
+      <c r="AA34" s="26" t="n"/>
+      <c r="AB34" s="27" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="B35" s="19" t="n"/>
-      <c r="C35" s="19" t="n"/>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="n"/>
-      <c r="G35" s="7" t="n"/>
-      <c r="H35" s="7" t="n"/>
-      <c r="I35" s="7" t="n"/>
-      <c r="J35" s="7" t="n"/>
-      <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="n"/>
-      <c r="M35" s="7" t="n"/>
-      <c r="N35" s="7" t="n"/>
-      <c r="P35" s="19" t="n"/>
-      <c r="Q35" s="19" t="n"/>
-      <c r="R35" s="19" t="n"/>
-      <c r="S35" s="7" t="n"/>
-      <c r="T35" s="7" t="n"/>
-      <c r="U35" s="7" t="n"/>
-      <c r="V35" s="7" t="n"/>
-      <c r="W35" s="7" t="n"/>
-      <c r="X35" s="7" t="n"/>
-      <c r="Y35" s="7" t="n"/>
-      <c r="Z35" s="7" t="n"/>
-      <c r="AA35" s="7" t="n"/>
-      <c r="AB35" s="7" t="n"/>
+      <c r="B35" s="30" t="n"/>
+      <c r="C35" s="31" t="n"/>
+      <c r="D35" s="32" t="n"/>
+      <c r="E35" s="30" t="n"/>
+      <c r="F35" s="31" t="n"/>
+      <c r="G35" s="31" t="n"/>
+      <c r="H35" s="31" t="n"/>
+      <c r="I35" s="31" t="n"/>
+      <c r="J35" s="31" t="n"/>
+      <c r="K35" s="31" t="n"/>
+      <c r="L35" s="31" t="n"/>
+      <c r="M35" s="31" t="n"/>
+      <c r="N35" s="32" t="n"/>
+      <c r="P35" s="30" t="n"/>
+      <c r="Q35" s="31" t="n"/>
+      <c r="R35" s="32" t="n"/>
+      <c r="S35" s="30" t="n"/>
+      <c r="T35" s="31" t="n"/>
+      <c r="U35" s="31" t="n"/>
+      <c r="V35" s="31" t="n"/>
+      <c r="W35" s="31" t="n"/>
+      <c r="X35" s="31" t="n"/>
+      <c r="Y35" s="31" t="n"/>
+      <c r="Z35" s="31" t="n"/>
+      <c r="AA35" s="31" t="n"/>
+      <c r="AB35" s="32" t="n"/>
     </row>
     <row r="36" ht="10" customHeight="1"/>
     <row r="37" ht="16" customHeight="1">
@@ -2975,315 +2664,117 @@
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="C37" s="35" t="n"/>
-      <c r="D37" s="35" t="n"/>
-      <c r="E37" s="35" t="n"/>
-      <c r="F37" s="35" t="n"/>
-      <c r="G37" s="35" t="n"/>
-      <c r="H37" s="35" t="n"/>
-      <c r="I37" s="35" t="n"/>
-      <c r="J37" s="35" t="n"/>
-      <c r="K37" s="35" t="n"/>
-      <c r="L37" s="35" t="n"/>
-      <c r="M37" s="35" t="n"/>
-      <c r="N37" s="35" t="n"/>
+      <c r="C37" s="40" t="n"/>
+      <c r="D37" s="40" t="n"/>
+      <c r="E37" s="40" t="n"/>
+      <c r="F37" s="40" t="n"/>
+      <c r="G37" s="40" t="n"/>
+      <c r="H37" s="40" t="n"/>
+      <c r="I37" s="40" t="n"/>
+      <c r="J37" s="40" t="n"/>
+      <c r="K37" s="40" t="n"/>
+      <c r="L37" s="40" t="n"/>
+      <c r="M37" s="40" t="n"/>
+      <c r="N37" s="41" t="n"/>
       <c r="P37" s="34" t="inlineStr">
         <is>
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="Q37" s="35" t="n"/>
-      <c r="R37" s="35" t="n"/>
-      <c r="S37" s="35" t="n"/>
-      <c r="T37" s="35" t="n"/>
-      <c r="U37" s="35" t="n"/>
-      <c r="V37" s="35" t="n"/>
-      <c r="W37" s="35" t="n"/>
-      <c r="X37" s="35" t="n"/>
-      <c r="Y37" s="35" t="n"/>
-      <c r="Z37" s="35" t="n"/>
-      <c r="AA37" s="35" t="n"/>
-      <c r="AB37" s="35" t="n"/>
+      <c r="Q37" s="40" t="n"/>
+      <c r="R37" s="40" t="n"/>
+      <c r="S37" s="40" t="n"/>
+      <c r="T37" s="40" t="n"/>
+      <c r="U37" s="40" t="n"/>
+      <c r="V37" s="40" t="n"/>
+      <c r="W37" s="40" t="n"/>
+      <c r="X37" s="40" t="n"/>
+      <c r="Y37" s="40" t="n"/>
+      <c r="Z37" s="40" t="n"/>
+      <c r="AA37" s="40" t="n"/>
+      <c r="AB37" s="41" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="B38" s="35" t="n"/>
-      <c r="C38" s="35" t="n"/>
-      <c r="D38" s="35" t="n"/>
-      <c r="E38" s="35" t="n"/>
-      <c r="F38" s="35" t="n"/>
-      <c r="G38" s="35" t="n"/>
-      <c r="H38" s="35" t="n"/>
-      <c r="I38" s="35" t="n"/>
-      <c r="J38" s="35" t="n"/>
-      <c r="K38" s="35" t="n"/>
-      <c r="L38" s="35" t="n"/>
-      <c r="M38" s="35" t="n"/>
-      <c r="N38" s="35" t="n"/>
-      <c r="P38" s="35" t="n"/>
-      <c r="Q38" s="35" t="n"/>
-      <c r="R38" s="35" t="n"/>
-      <c r="S38" s="35" t="n"/>
-      <c r="T38" s="35" t="n"/>
-      <c r="U38" s="35" t="n"/>
-      <c r="V38" s="35" t="n"/>
-      <c r="W38" s="35" t="n"/>
-      <c r="X38" s="35" t="n"/>
-      <c r="Y38" s="35" t="n"/>
-      <c r="Z38" s="35" t="n"/>
-      <c r="AA38" s="35" t="n"/>
-      <c r="AB38" s="35" t="n"/>
+      <c r="B38" s="42" t="n"/>
+      <c r="N38" s="43" t="n"/>
+      <c r="P38" s="42" t="n"/>
+      <c r="AB38" s="43" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="B39" s="35" t="n"/>
-      <c r="C39" s="35" t="n"/>
-      <c r="D39" s="35" t="n"/>
-      <c r="E39" s="35" t="n"/>
-      <c r="F39" s="35" t="n"/>
-      <c r="G39" s="35" t="n"/>
-      <c r="H39" s="35" t="n"/>
-      <c r="I39" s="35" t="n"/>
-      <c r="J39" s="35" t="n"/>
-      <c r="K39" s="35" t="n"/>
-      <c r="L39" s="35" t="n"/>
-      <c r="M39" s="35" t="n"/>
-      <c r="N39" s="35" t="n"/>
-      <c r="P39" s="35" t="n"/>
-      <c r="Q39" s="35" t="n"/>
-      <c r="R39" s="35" t="n"/>
-      <c r="S39" s="35" t="n"/>
-      <c r="T39" s="35" t="n"/>
-      <c r="U39" s="35" t="n"/>
-      <c r="V39" s="35" t="n"/>
-      <c r="W39" s="35" t="n"/>
-      <c r="X39" s="35" t="n"/>
-      <c r="Y39" s="35" t="n"/>
-      <c r="Z39" s="35" t="n"/>
-      <c r="AA39" s="35" t="n"/>
-      <c r="AB39" s="35" t="n"/>
+      <c r="B39" s="42" t="n"/>
+      <c r="N39" s="43" t="n"/>
+      <c r="P39" s="42" t="n"/>
+      <c r="AB39" s="43" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="B40" s="35" t="n"/>
-      <c r="C40" s="35" t="n"/>
-      <c r="D40" s="35" t="n"/>
-      <c r="E40" s="35" t="n"/>
-      <c r="F40" s="35" t="n"/>
-      <c r="G40" s="35" t="n"/>
-      <c r="H40" s="35" t="n"/>
-      <c r="I40" s="35" t="n"/>
-      <c r="J40" s="35" t="n"/>
-      <c r="K40" s="35" t="n"/>
-      <c r="L40" s="35" t="n"/>
-      <c r="M40" s="35" t="n"/>
-      <c r="N40" s="35" t="n"/>
-      <c r="P40" s="35" t="n"/>
-      <c r="Q40" s="35" t="n"/>
-      <c r="R40" s="35" t="n"/>
-      <c r="S40" s="35" t="n"/>
-      <c r="T40" s="35" t="n"/>
-      <c r="U40" s="35" t="n"/>
-      <c r="V40" s="35" t="n"/>
-      <c r="W40" s="35" t="n"/>
-      <c r="X40" s="35" t="n"/>
-      <c r="Y40" s="35" t="n"/>
-      <c r="Z40" s="35" t="n"/>
-      <c r="AA40" s="35" t="n"/>
-      <c r="AB40" s="35" t="n"/>
+      <c r="B40" s="42" t="n"/>
+      <c r="N40" s="43" t="n"/>
+      <c r="P40" s="42" t="n"/>
+      <c r="AB40" s="43" t="n"/>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="B41" s="35" t="n"/>
-      <c r="C41" s="35" t="n"/>
-      <c r="D41" s="35" t="n"/>
-      <c r="E41" s="35" t="n"/>
-      <c r="F41" s="35" t="n"/>
-      <c r="G41" s="35" t="n"/>
-      <c r="H41" s="35" t="n"/>
-      <c r="I41" s="35" t="n"/>
-      <c r="J41" s="35" t="n"/>
-      <c r="K41" s="35" t="n"/>
-      <c r="L41" s="35" t="n"/>
-      <c r="M41" s="35" t="n"/>
-      <c r="N41" s="35" t="n"/>
-      <c r="P41" s="35" t="n"/>
-      <c r="Q41" s="35" t="n"/>
-      <c r="R41" s="35" t="n"/>
-      <c r="S41" s="35" t="n"/>
-      <c r="T41" s="35" t="n"/>
-      <c r="U41" s="35" t="n"/>
-      <c r="V41" s="35" t="n"/>
-      <c r="W41" s="35" t="n"/>
-      <c r="X41" s="35" t="n"/>
-      <c r="Y41" s="35" t="n"/>
-      <c r="Z41" s="35" t="n"/>
-      <c r="AA41" s="35" t="n"/>
-      <c r="AB41" s="35" t="n"/>
+      <c r="B41" s="42" t="n"/>
+      <c r="N41" s="43" t="n"/>
+      <c r="P41" s="42" t="n"/>
+      <c r="AB41" s="43" t="n"/>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="B42" s="35" t="n"/>
-      <c r="C42" s="35" t="n"/>
-      <c r="D42" s="35" t="n"/>
-      <c r="E42" s="35" t="n"/>
-      <c r="F42" s="35" t="n"/>
-      <c r="G42" s="35" t="n"/>
-      <c r="H42" s="35" t="n"/>
-      <c r="I42" s="35" t="n"/>
-      <c r="J42" s="35" t="n"/>
-      <c r="K42" s="35" t="n"/>
-      <c r="L42" s="35" t="n"/>
-      <c r="M42" s="35" t="n"/>
-      <c r="N42" s="35" t="n"/>
-      <c r="P42" s="35" t="n"/>
-      <c r="Q42" s="35" t="n"/>
-      <c r="R42" s="35" t="n"/>
-      <c r="S42" s="35" t="n"/>
-      <c r="T42" s="35" t="n"/>
-      <c r="U42" s="35" t="n"/>
-      <c r="V42" s="35" t="n"/>
-      <c r="W42" s="35" t="n"/>
-      <c r="X42" s="35" t="n"/>
-      <c r="Y42" s="35" t="n"/>
-      <c r="Z42" s="35" t="n"/>
-      <c r="AA42" s="35" t="n"/>
-      <c r="AB42" s="35" t="n"/>
+      <c r="B42" s="42" t="n"/>
+      <c r="N42" s="43" t="n"/>
+      <c r="P42" s="42" t="n"/>
+      <c r="AB42" s="43" t="n"/>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="B43" s="35" t="n"/>
-      <c r="C43" s="35" t="n"/>
-      <c r="D43" s="35" t="n"/>
-      <c r="E43" s="35" t="n"/>
-      <c r="F43" s="35" t="n"/>
-      <c r="G43" s="35" t="n"/>
-      <c r="H43" s="35" t="n"/>
-      <c r="I43" s="35" t="n"/>
-      <c r="J43" s="35" t="n"/>
-      <c r="K43" s="35" t="n"/>
-      <c r="L43" s="35" t="n"/>
-      <c r="M43" s="35" t="n"/>
-      <c r="N43" s="35" t="n"/>
-      <c r="P43" s="35" t="n"/>
-      <c r="Q43" s="35" t="n"/>
-      <c r="R43" s="35" t="n"/>
-      <c r="S43" s="35" t="n"/>
-      <c r="T43" s="35" t="n"/>
-      <c r="U43" s="35" t="n"/>
-      <c r="V43" s="35" t="n"/>
-      <c r="W43" s="35" t="n"/>
-      <c r="X43" s="35" t="n"/>
-      <c r="Y43" s="35" t="n"/>
-      <c r="Z43" s="35" t="n"/>
-      <c r="AA43" s="35" t="n"/>
-      <c r="AB43" s="35" t="n"/>
+      <c r="B43" s="42" t="n"/>
+      <c r="N43" s="43" t="n"/>
+      <c r="P43" s="42" t="n"/>
+      <c r="AB43" s="43" t="n"/>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="B44" s="35" t="n"/>
-      <c r="C44" s="35" t="n"/>
-      <c r="D44" s="35" t="n"/>
-      <c r="E44" s="35" t="n"/>
-      <c r="F44" s="35" t="n"/>
-      <c r="G44" s="35" t="n"/>
-      <c r="H44" s="35" t="n"/>
-      <c r="I44" s="35" t="n"/>
-      <c r="J44" s="35" t="n"/>
-      <c r="K44" s="35" t="n"/>
-      <c r="L44" s="35" t="n"/>
-      <c r="M44" s="35" t="n"/>
-      <c r="N44" s="35" t="n"/>
-      <c r="P44" s="35" t="n"/>
-      <c r="Q44" s="35" t="n"/>
-      <c r="R44" s="35" t="n"/>
-      <c r="S44" s="35" t="n"/>
-      <c r="T44" s="35" t="n"/>
-      <c r="U44" s="35" t="n"/>
-      <c r="V44" s="35" t="n"/>
-      <c r="W44" s="35" t="n"/>
-      <c r="X44" s="35" t="n"/>
-      <c r="Y44" s="35" t="n"/>
-      <c r="Z44" s="35" t="n"/>
-      <c r="AA44" s="35" t="n"/>
-      <c r="AB44" s="35" t="n"/>
+      <c r="B44" s="42" t="n"/>
+      <c r="N44" s="43" t="n"/>
+      <c r="P44" s="42" t="n"/>
+      <c r="AB44" s="43" t="n"/>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="B45" s="35" t="n"/>
-      <c r="C45" s="35" t="n"/>
-      <c r="D45" s="35" t="n"/>
-      <c r="E45" s="35" t="n"/>
-      <c r="F45" s="35" t="n"/>
-      <c r="G45" s="35" t="n"/>
-      <c r="H45" s="35" t="n"/>
-      <c r="I45" s="35" t="n"/>
-      <c r="J45" s="35" t="n"/>
-      <c r="K45" s="35" t="n"/>
-      <c r="L45" s="35" t="n"/>
-      <c r="M45" s="35" t="n"/>
-      <c r="N45" s="35" t="n"/>
-      <c r="P45" s="35" t="n"/>
-      <c r="Q45" s="35" t="n"/>
-      <c r="R45" s="35" t="n"/>
-      <c r="S45" s="35" t="n"/>
-      <c r="T45" s="35" t="n"/>
-      <c r="U45" s="35" t="n"/>
-      <c r="V45" s="35" t="n"/>
-      <c r="W45" s="35" t="n"/>
-      <c r="X45" s="35" t="n"/>
-      <c r="Y45" s="35" t="n"/>
-      <c r="Z45" s="35" t="n"/>
-      <c r="AA45" s="35" t="n"/>
-      <c r="AB45" s="35" t="n"/>
+      <c r="B45" s="42" t="n"/>
+      <c r="N45" s="43" t="n"/>
+      <c r="P45" s="42" t="n"/>
+      <c r="AB45" s="43" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="B46" s="35" t="n"/>
-      <c r="C46" s="35" t="n"/>
-      <c r="D46" s="35" t="n"/>
-      <c r="E46" s="35" t="n"/>
-      <c r="F46" s="35" t="n"/>
-      <c r="G46" s="35" t="n"/>
-      <c r="H46" s="35" t="n"/>
-      <c r="I46" s="35" t="n"/>
-      <c r="J46" s="35" t="n"/>
-      <c r="K46" s="35" t="n"/>
-      <c r="L46" s="35" t="n"/>
-      <c r="M46" s="35" t="n"/>
-      <c r="N46" s="35" t="n"/>
-      <c r="P46" s="35" t="n"/>
-      <c r="Q46" s="35" t="n"/>
-      <c r="R46" s="35" t="n"/>
-      <c r="S46" s="35" t="n"/>
-      <c r="T46" s="35" t="n"/>
-      <c r="U46" s="35" t="n"/>
-      <c r="V46" s="35" t="n"/>
-      <c r="W46" s="35" t="n"/>
-      <c r="X46" s="35" t="n"/>
-      <c r="Y46" s="35" t="n"/>
-      <c r="Z46" s="35" t="n"/>
-      <c r="AA46" s="35" t="n"/>
-      <c r="AB46" s="35" t="n"/>
+      <c r="B46" s="42" t="n"/>
+      <c r="N46" s="43" t="n"/>
+      <c r="P46" s="42" t="n"/>
+      <c r="AB46" s="43" t="n"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="B47" s="35" t="n"/>
-      <c r="C47" s="35" t="n"/>
-      <c r="D47" s="35" t="n"/>
-      <c r="E47" s="35" t="n"/>
-      <c r="F47" s="35" t="n"/>
-      <c r="G47" s="35" t="n"/>
-      <c r="H47" s="35" t="n"/>
-      <c r="I47" s="35" t="n"/>
-      <c r="J47" s="35" t="n"/>
-      <c r="K47" s="35" t="n"/>
-      <c r="L47" s="35" t="n"/>
-      <c r="M47" s="35" t="n"/>
-      <c r="N47" s="35" t="n"/>
-      <c r="P47" s="35" t="n"/>
-      <c r="Q47" s="35" t="n"/>
-      <c r="R47" s="35" t="n"/>
-      <c r="S47" s="35" t="n"/>
-      <c r="T47" s="35" t="n"/>
-      <c r="U47" s="35" t="n"/>
-      <c r="V47" s="35" t="n"/>
-      <c r="W47" s="35" t="n"/>
-      <c r="X47" s="35" t="n"/>
-      <c r="Y47" s="35" t="n"/>
-      <c r="Z47" s="35" t="n"/>
-      <c r="AA47" s="35" t="n"/>
-      <c r="AB47" s="35" t="n"/>
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="45" t="n"/>
+      <c r="I47" s="45" t="n"/>
+      <c r="J47" s="45" t="n"/>
+      <c r="K47" s="45" t="n"/>
+      <c r="L47" s="45" t="n"/>
+      <c r="M47" s="45" t="n"/>
+      <c r="N47" s="46" t="n"/>
+      <c r="P47" s="44" t="n"/>
+      <c r="Q47" s="45" t="n"/>
+      <c r="R47" s="45" t="n"/>
+      <c r="S47" s="45" t="n"/>
+      <c r="T47" s="45" t="n"/>
+      <c r="U47" s="45" t="n"/>
+      <c r="V47" s="45" t="n"/>
+      <c r="W47" s="45" t="n"/>
+      <c r="X47" s="45" t="n"/>
+      <c r="Y47" s="45" t="n"/>
+      <c r="Z47" s="45" t="n"/>
+      <c r="AA47" s="45" t="n"/>
+      <c r="AB47" s="46" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="36" t="inlineStr">
@@ -3291,40 +2782,40 @@
           <t>사진 5</t>
         </is>
       </c>
-      <c r="C48" s="19" t="n"/>
-      <c r="D48" s="19" t="n"/>
+      <c r="C48" s="22" t="n"/>
+      <c r="D48" s="23" t="n"/>
       <c r="E48" s="37" t="inlineStr">
         <is>
           <t>위치</t>
         </is>
       </c>
-      <c r="F48" s="19" t="n"/>
-      <c r="G48" s="19" t="n"/>
+      <c r="F48" s="22" t="n"/>
+      <c r="G48" s="23" t="n"/>
       <c r="H48" s="38" t="inlineStr"/>
-      <c r="I48" s="7" t="n"/>
-      <c r="J48" s="7" t="n"/>
-      <c r="K48" s="7" t="n"/>
+      <c r="I48" s="22" t="n"/>
+      <c r="J48" s="22" t="n"/>
+      <c r="K48" s="23" t="n"/>
       <c r="P48" s="36" t="inlineStr">
         <is>
           <t>사진 6</t>
         </is>
       </c>
-      <c r="Q48" s="19" t="n"/>
-      <c r="R48" s="19" t="n"/>
+      <c r="Q48" s="22" t="n"/>
+      <c r="R48" s="23" t="n"/>
       <c r="S48" s="37" t="inlineStr">
         <is>
           <t>위치</t>
         </is>
       </c>
-      <c r="T48" s="19" t="n"/>
-      <c r="U48" s="19" t="n"/>
+      <c r="T48" s="22" t="n"/>
+      <c r="U48" s="23" t="n"/>
       <c r="V48" s="38" t="inlineStr"/>
-      <c r="W48" s="7" t="n"/>
-      <c r="X48" s="7" t="n"/>
-      <c r="Y48" s="7" t="n"/>
-      <c r="Z48" s="7" t="n"/>
-      <c r="AA48" s="7" t="n"/>
-      <c r="AB48" s="7" t="n"/>
+      <c r="W48" s="22" t="n"/>
+      <c r="X48" s="22" t="n"/>
+      <c r="Y48" s="22" t="n"/>
+      <c r="Z48" s="22" t="n"/>
+      <c r="AA48" s="22" t="n"/>
+      <c r="AB48" s="23" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="B49" s="37" t="inlineStr">
@@ -3332,63 +2823,63 @@
           <t>내용</t>
         </is>
       </c>
-      <c r="C49" s="19" t="n"/>
-      <c r="D49" s="19" t="n"/>
+      <c r="C49" s="26" t="n"/>
+      <c r="D49" s="27" t="n"/>
       <c r="E49" s="39" t="inlineStr"/>
-      <c r="F49" s="7" t="n"/>
-      <c r="G49" s="7" t="n"/>
-      <c r="H49" s="7" t="n"/>
-      <c r="I49" s="7" t="n"/>
-      <c r="J49" s="7" t="n"/>
-      <c r="K49" s="7" t="n"/>
-      <c r="L49" s="7" t="n"/>
-      <c r="M49" s="7" t="n"/>
-      <c r="N49" s="7" t="n"/>
+      <c r="F49" s="26" t="n"/>
+      <c r="G49" s="26" t="n"/>
+      <c r="H49" s="26" t="n"/>
+      <c r="I49" s="26" t="n"/>
+      <c r="J49" s="26" t="n"/>
+      <c r="K49" s="26" t="n"/>
+      <c r="L49" s="26" t="n"/>
+      <c r="M49" s="26" t="n"/>
+      <c r="N49" s="27" t="n"/>
       <c r="P49" s="37" t="inlineStr">
         <is>
           <t>내용</t>
         </is>
       </c>
-      <c r="Q49" s="19" t="n"/>
-      <c r="R49" s="19" t="n"/>
+      <c r="Q49" s="26" t="n"/>
+      <c r="R49" s="27" t="n"/>
       <c r="S49" s="39" t="inlineStr"/>
-      <c r="T49" s="7" t="n"/>
-      <c r="U49" s="7" t="n"/>
-      <c r="V49" s="7" t="n"/>
-      <c r="W49" s="7" t="n"/>
-      <c r="X49" s="7" t="n"/>
-      <c r="Y49" s="7" t="n"/>
-      <c r="Z49" s="7" t="n"/>
-      <c r="AA49" s="7" t="n"/>
-      <c r="AB49" s="7" t="n"/>
+      <c r="T49" s="26" t="n"/>
+      <c r="U49" s="26" t="n"/>
+      <c r="V49" s="26" t="n"/>
+      <c r="W49" s="26" t="n"/>
+      <c r="X49" s="26" t="n"/>
+      <c r="Y49" s="26" t="n"/>
+      <c r="Z49" s="26" t="n"/>
+      <c r="AA49" s="26" t="n"/>
+      <c r="AB49" s="27" t="n"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="B50" s="19" t="n"/>
-      <c r="C50" s="19" t="n"/>
-      <c r="D50" s="19" t="n"/>
-      <c r="E50" s="7" t="n"/>
-      <c r="F50" s="7" t="n"/>
-      <c r="G50" s="7" t="n"/>
-      <c r="H50" s="7" t="n"/>
-      <c r="I50" s="7" t="n"/>
-      <c r="J50" s="7" t="n"/>
-      <c r="K50" s="7" t="n"/>
-      <c r="L50" s="7" t="n"/>
-      <c r="M50" s="7" t="n"/>
-      <c r="N50" s="7" t="n"/>
-      <c r="P50" s="19" t="n"/>
-      <c r="Q50" s="19" t="n"/>
-      <c r="R50" s="19" t="n"/>
-      <c r="S50" s="7" t="n"/>
-      <c r="T50" s="7" t="n"/>
-      <c r="U50" s="7" t="n"/>
-      <c r="V50" s="7" t="n"/>
-      <c r="W50" s="7" t="n"/>
-      <c r="X50" s="7" t="n"/>
-      <c r="Y50" s="7" t="n"/>
-      <c r="Z50" s="7" t="n"/>
-      <c r="AA50" s="7" t="n"/>
-      <c r="AB50" s="7" t="n"/>
+      <c r="B50" s="30" t="n"/>
+      <c r="C50" s="31" t="n"/>
+      <c r="D50" s="32" t="n"/>
+      <c r="E50" s="30" t="n"/>
+      <c r="F50" s="31" t="n"/>
+      <c r="G50" s="31" t="n"/>
+      <c r="H50" s="31" t="n"/>
+      <c r="I50" s="31" t="n"/>
+      <c r="J50" s="31" t="n"/>
+      <c r="K50" s="31" t="n"/>
+      <c r="L50" s="31" t="n"/>
+      <c r="M50" s="31" t="n"/>
+      <c r="N50" s="32" t="n"/>
+      <c r="P50" s="30" t="n"/>
+      <c r="Q50" s="31" t="n"/>
+      <c r="R50" s="32" t="n"/>
+      <c r="S50" s="30" t="n"/>
+      <c r="T50" s="31" t="n"/>
+      <c r="U50" s="31" t="n"/>
+      <c r="V50" s="31" t="n"/>
+      <c r="W50" s="31" t="n"/>
+      <c r="X50" s="31" t="n"/>
+      <c r="Y50" s="31" t="n"/>
+      <c r="Z50" s="31" t="n"/>
+      <c r="AA50" s="31" t="n"/>
+      <c r="AB50" s="32" t="n"/>
     </row>
     <row r="51" ht="10" customHeight="1"/>
   </sheetData>
@@ -3436,4 +2927,1539 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF305496"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:AB56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4.6" customWidth="1" min="2" max="2"/>
+    <col width="4.6" customWidth="1" min="3" max="3"/>
+    <col width="4.6" customWidth="1" min="4" max="4"/>
+    <col width="4.6" customWidth="1" min="5" max="5"/>
+    <col width="4.6" customWidth="1" min="6" max="6"/>
+    <col width="4.6" customWidth="1" min="7" max="7"/>
+    <col width="4.6" customWidth="1" min="8" max="8"/>
+    <col width="4.6" customWidth="1" min="9" max="9"/>
+    <col width="4.6" customWidth="1" min="10" max="10"/>
+    <col width="4.6" customWidth="1" min="11" max="11"/>
+    <col width="4.6" customWidth="1" min="12" max="12"/>
+    <col width="4.6" customWidth="1" min="13" max="13"/>
+    <col width="4.6" customWidth="1" min="14" max="14"/>
+    <col width="4.6" customWidth="1" min="15" max="15"/>
+    <col width="4.6" customWidth="1" min="16" max="16"/>
+    <col width="4.6" customWidth="1" min="17" max="17"/>
+    <col width="4.6" customWidth="1" min="18" max="18"/>
+    <col width="4.6" customWidth="1" min="19" max="19"/>
+    <col width="4.6" customWidth="1" min="20" max="20"/>
+    <col width="4.6" customWidth="1" min="21" max="21"/>
+    <col width="4.6" customWidth="1" min="22" max="22"/>
+    <col width="4.6" customWidth="1" min="23" max="23"/>
+    <col width="4.6" customWidth="1" min="24" max="24"/>
+    <col width="4.6" customWidth="1" min="25" max="25"/>
+    <col width="4.6" customWidth="1" min="26" max="26"/>
+    <col width="4.6" customWidth="1" min="27" max="27"/>
+    <col width="4.6" customWidth="1" min="28" max="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="6" customHeight="1"/>
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>지적사항 조치 전·후 사진대지</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+      <c r="Z2" s="2" t="n"/>
+      <c r="AA2" s="2" t="n"/>
+      <c r="AB2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>(경영책임자 현장순회점검표 첨부자료 - 지적사항별 개선 전/후 비교)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1"/>
+    <row r="5" ht="16" customHeight="1">
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>※ 사진 삽입 방법: 아래 점선 박스를 클릭한 후 [삽입] → [그림]으로 조치 전/후 사진을 각각 첨부하세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="6" customHeight="1"/>
+    <row r="7" ht="20" customHeight="1">
+      <c r="B7" s="47" t="inlineStr">
+        <is>
+          <t>No.1</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="36" t="inlineStr">
+        <is>
+          <t>지적사항 내용</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="19" t="n"/>
+      <c r="H7" s="19" t="n"/>
+      <c r="I7" s="48" t="inlineStr"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
+      <c r="O7" s="7" t="n"/>
+      <c r="P7" s="7" t="n"/>
+      <c r="Q7" s="7" t="n"/>
+      <c r="R7" s="7" t="n"/>
+      <c r="S7" s="7" t="n"/>
+      <c r="T7" s="7" t="n"/>
+      <c r="U7" s="7" t="n"/>
+      <c r="V7" s="7" t="n"/>
+      <c r="W7" s="7" t="n"/>
+      <c r="X7" s="7" t="n"/>
+      <c r="Y7" s="7" t="n"/>
+      <c r="Z7" s="7" t="n"/>
+      <c r="AA7" s="7" t="n"/>
+      <c r="AB7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>▼ 조치 전 (Before)</t>
+        </is>
+      </c>
+      <c r="P8" s="50" t="inlineStr">
+        <is>
+          <t>▼ 조치 후 (After)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="B9" s="34" t="inlineStr">
+        <is>
+          <t>사진 삽입 영역</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="n"/>
+      <c r="D9" s="35" t="n"/>
+      <c r="E9" s="35" t="n"/>
+      <c r="F9" s="35" t="n"/>
+      <c r="G9" s="35" t="n"/>
+      <c r="H9" s="35" t="n"/>
+      <c r="I9" s="35" t="n"/>
+      <c r="J9" s="35" t="n"/>
+      <c r="K9" s="35" t="n"/>
+      <c r="L9" s="35" t="n"/>
+      <c r="M9" s="35" t="n"/>
+      <c r="N9" s="35" t="n"/>
+      <c r="P9" s="34" t="inlineStr">
+        <is>
+          <t>사진 삽입 영역</t>
+        </is>
+      </c>
+      <c r="Q9" s="35" t="n"/>
+      <c r="R9" s="35" t="n"/>
+      <c r="S9" s="35" t="n"/>
+      <c r="T9" s="35" t="n"/>
+      <c r="U9" s="35" t="n"/>
+      <c r="V9" s="35" t="n"/>
+      <c r="W9" s="35" t="n"/>
+      <c r="X9" s="35" t="n"/>
+      <c r="Y9" s="35" t="n"/>
+      <c r="Z9" s="35" t="n"/>
+      <c r="AA9" s="35" t="n"/>
+      <c r="AB9" s="35" t="n"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="B10" s="35" t="n"/>
+      <c r="C10" s="35" t="n"/>
+      <c r="D10" s="35" t="n"/>
+      <c r="E10" s="35" t="n"/>
+      <c r="F10" s="35" t="n"/>
+      <c r="G10" s="35" t="n"/>
+      <c r="H10" s="35" t="n"/>
+      <c r="I10" s="35" t="n"/>
+      <c r="J10" s="35" t="n"/>
+      <c r="K10" s="35" t="n"/>
+      <c r="L10" s="35" t="n"/>
+      <c r="M10" s="35" t="n"/>
+      <c r="N10" s="35" t="n"/>
+      <c r="P10" s="35" t="n"/>
+      <c r="Q10" s="35" t="n"/>
+      <c r="R10" s="35" t="n"/>
+      <c r="S10" s="35" t="n"/>
+      <c r="T10" s="35" t="n"/>
+      <c r="U10" s="35" t="n"/>
+      <c r="V10" s="35" t="n"/>
+      <c r="W10" s="35" t="n"/>
+      <c r="X10" s="35" t="n"/>
+      <c r="Y10" s="35" t="n"/>
+      <c r="Z10" s="35" t="n"/>
+      <c r="AA10" s="35" t="n"/>
+      <c r="AB10" s="35" t="n"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="B11" s="35" t="n"/>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="35" t="n"/>
+      <c r="E11" s="35" t="n"/>
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="35" t="n"/>
+      <c r="H11" s="35" t="n"/>
+      <c r="I11" s="35" t="n"/>
+      <c r="J11" s="35" t="n"/>
+      <c r="K11" s="35" t="n"/>
+      <c r="L11" s="35" t="n"/>
+      <c r="M11" s="35" t="n"/>
+      <c r="N11" s="35" t="n"/>
+      <c r="P11" s="35" t="n"/>
+      <c r="Q11" s="35" t="n"/>
+      <c r="R11" s="35" t="n"/>
+      <c r="S11" s="35" t="n"/>
+      <c r="T11" s="35" t="n"/>
+      <c r="U11" s="35" t="n"/>
+      <c r="V11" s="35" t="n"/>
+      <c r="W11" s="35" t="n"/>
+      <c r="X11" s="35" t="n"/>
+      <c r="Y11" s="35" t="n"/>
+      <c r="Z11" s="35" t="n"/>
+      <c r="AA11" s="35" t="n"/>
+      <c r="AB11" s="35" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="B12" s="35" t="n"/>
+      <c r="C12" s="35" t="n"/>
+      <c r="D12" s="35" t="n"/>
+      <c r="E12" s="35" t="n"/>
+      <c r="F12" s="35" t="n"/>
+      <c r="G12" s="35" t="n"/>
+      <c r="H12" s="35" t="n"/>
+      <c r="I12" s="35" t="n"/>
+      <c r="J12" s="35" t="n"/>
+      <c r="K12" s="35" t="n"/>
+      <c r="L12" s="35" t="n"/>
+      <c r="M12" s="35" t="n"/>
+      <c r="N12" s="35" t="n"/>
+      <c r="P12" s="35" t="n"/>
+      <c r="Q12" s="35" t="n"/>
+      <c r="R12" s="35" t="n"/>
+      <c r="S12" s="35" t="n"/>
+      <c r="T12" s="35" t="n"/>
+      <c r="U12" s="35" t="n"/>
+      <c r="V12" s="35" t="n"/>
+      <c r="W12" s="35" t="n"/>
+      <c r="X12" s="35" t="n"/>
+      <c r="Y12" s="35" t="n"/>
+      <c r="Z12" s="35" t="n"/>
+      <c r="AA12" s="35" t="n"/>
+      <c r="AB12" s="35" t="n"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="35" t="n"/>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="35" t="n"/>
+      <c r="H13" s="35" t="n"/>
+      <c r="I13" s="35" t="n"/>
+      <c r="J13" s="35" t="n"/>
+      <c r="K13" s="35" t="n"/>
+      <c r="L13" s="35" t="n"/>
+      <c r="M13" s="35" t="n"/>
+      <c r="N13" s="35" t="n"/>
+      <c r="P13" s="35" t="n"/>
+      <c r="Q13" s="35" t="n"/>
+      <c r="R13" s="35" t="n"/>
+      <c r="S13" s="35" t="n"/>
+      <c r="T13" s="35" t="n"/>
+      <c r="U13" s="35" t="n"/>
+      <c r="V13" s="35" t="n"/>
+      <c r="W13" s="35" t="n"/>
+      <c r="X13" s="35" t="n"/>
+      <c r="Y13" s="35" t="n"/>
+      <c r="Z13" s="35" t="n"/>
+      <c r="AA13" s="35" t="n"/>
+      <c r="AB13" s="35" t="n"/>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="B14" s="35" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="35" t="n"/>
+      <c r="E14" s="35" t="n"/>
+      <c r="F14" s="35" t="n"/>
+      <c r="G14" s="35" t="n"/>
+      <c r="H14" s="35" t="n"/>
+      <c r="I14" s="35" t="n"/>
+      <c r="J14" s="35" t="n"/>
+      <c r="K14" s="35" t="n"/>
+      <c r="L14" s="35" t="n"/>
+      <c r="M14" s="35" t="n"/>
+      <c r="N14" s="35" t="n"/>
+      <c r="P14" s="35" t="n"/>
+      <c r="Q14" s="35" t="n"/>
+      <c r="R14" s="35" t="n"/>
+      <c r="S14" s="35" t="n"/>
+      <c r="T14" s="35" t="n"/>
+      <c r="U14" s="35" t="n"/>
+      <c r="V14" s="35" t="n"/>
+      <c r="W14" s="35" t="n"/>
+      <c r="X14" s="35" t="n"/>
+      <c r="Y14" s="35" t="n"/>
+      <c r="Z14" s="35" t="n"/>
+      <c r="AA14" s="35" t="n"/>
+      <c r="AB14" s="35" t="n"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="B15" s="35" t="n"/>
+      <c r="C15" s="35" t="n"/>
+      <c r="D15" s="35" t="n"/>
+      <c r="E15" s="35" t="n"/>
+      <c r="F15" s="35" t="n"/>
+      <c r="G15" s="35" t="n"/>
+      <c r="H15" s="35" t="n"/>
+      <c r="I15" s="35" t="n"/>
+      <c r="J15" s="35" t="n"/>
+      <c r="K15" s="35" t="n"/>
+      <c r="L15" s="35" t="n"/>
+      <c r="M15" s="35" t="n"/>
+      <c r="N15" s="35" t="n"/>
+      <c r="P15" s="35" t="n"/>
+      <c r="Q15" s="35" t="n"/>
+      <c r="R15" s="35" t="n"/>
+      <c r="S15" s="35" t="n"/>
+      <c r="T15" s="35" t="n"/>
+      <c r="U15" s="35" t="n"/>
+      <c r="V15" s="35" t="n"/>
+      <c r="W15" s="35" t="n"/>
+      <c r="X15" s="35" t="n"/>
+      <c r="Y15" s="35" t="n"/>
+      <c r="Z15" s="35" t="n"/>
+      <c r="AA15" s="35" t="n"/>
+      <c r="AB15" s="35" t="n"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="35" t="n"/>
+      <c r="E16" s="35" t="n"/>
+      <c r="F16" s="35" t="n"/>
+      <c r="G16" s="35" t="n"/>
+      <c r="H16" s="35" t="n"/>
+      <c r="I16" s="35" t="n"/>
+      <c r="J16" s="35" t="n"/>
+      <c r="K16" s="35" t="n"/>
+      <c r="L16" s="35" t="n"/>
+      <c r="M16" s="35" t="n"/>
+      <c r="N16" s="35" t="n"/>
+      <c r="P16" s="35" t="n"/>
+      <c r="Q16" s="35" t="n"/>
+      <c r="R16" s="35" t="n"/>
+      <c r="S16" s="35" t="n"/>
+      <c r="T16" s="35" t="n"/>
+      <c r="U16" s="35" t="n"/>
+      <c r="V16" s="35" t="n"/>
+      <c r="W16" s="35" t="n"/>
+      <c r="X16" s="35" t="n"/>
+      <c r="Y16" s="35" t="n"/>
+      <c r="Z16" s="35" t="n"/>
+      <c r="AA16" s="35" t="n"/>
+      <c r="AB16" s="35" t="n"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="B17" s="35" t="n"/>
+      <c r="C17" s="35" t="n"/>
+      <c r="D17" s="35" t="n"/>
+      <c r="E17" s="35" t="n"/>
+      <c r="F17" s="35" t="n"/>
+      <c r="G17" s="35" t="n"/>
+      <c r="H17" s="35" t="n"/>
+      <c r="I17" s="35" t="n"/>
+      <c r="J17" s="35" t="n"/>
+      <c r="K17" s="35" t="n"/>
+      <c r="L17" s="35" t="n"/>
+      <c r="M17" s="35" t="n"/>
+      <c r="N17" s="35" t="n"/>
+      <c r="P17" s="35" t="n"/>
+      <c r="Q17" s="35" t="n"/>
+      <c r="R17" s="35" t="n"/>
+      <c r="S17" s="35" t="n"/>
+      <c r="T17" s="35" t="n"/>
+      <c r="U17" s="35" t="n"/>
+      <c r="V17" s="35" t="n"/>
+      <c r="W17" s="35" t="n"/>
+      <c r="X17" s="35" t="n"/>
+      <c r="Y17" s="35" t="n"/>
+      <c r="Z17" s="35" t="n"/>
+      <c r="AA17" s="35" t="n"/>
+      <c r="AB17" s="35" t="n"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="35" t="n"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="35" t="n"/>
+      <c r="H18" s="35" t="n"/>
+      <c r="I18" s="35" t="n"/>
+      <c r="J18" s="35" t="n"/>
+      <c r="K18" s="35" t="n"/>
+      <c r="L18" s="35" t="n"/>
+      <c r="M18" s="35" t="n"/>
+      <c r="N18" s="35" t="n"/>
+      <c r="P18" s="35" t="n"/>
+      <c r="Q18" s="35" t="n"/>
+      <c r="R18" s="35" t="n"/>
+      <c r="S18" s="35" t="n"/>
+      <c r="T18" s="35" t="n"/>
+      <c r="U18" s="35" t="n"/>
+      <c r="V18" s="35" t="n"/>
+      <c r="W18" s="35" t="n"/>
+      <c r="X18" s="35" t="n"/>
+      <c r="Y18" s="35" t="n"/>
+      <c r="Z18" s="35" t="n"/>
+      <c r="AA18" s="35" t="n"/>
+      <c r="AB18" s="35" t="n"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="B19" s="35" t="n"/>
+      <c r="C19" s="35" t="n"/>
+      <c r="D19" s="35" t="n"/>
+      <c r="E19" s="35" t="n"/>
+      <c r="F19" s="35" t="n"/>
+      <c r="G19" s="35" t="n"/>
+      <c r="H19" s="35" t="n"/>
+      <c r="I19" s="35" t="n"/>
+      <c r="J19" s="35" t="n"/>
+      <c r="K19" s="35" t="n"/>
+      <c r="L19" s="35" t="n"/>
+      <c r="M19" s="35" t="n"/>
+      <c r="N19" s="35" t="n"/>
+      <c r="P19" s="35" t="n"/>
+      <c r="Q19" s="35" t="n"/>
+      <c r="R19" s="35" t="n"/>
+      <c r="S19" s="35" t="n"/>
+      <c r="T19" s="35" t="n"/>
+      <c r="U19" s="35" t="n"/>
+      <c r="V19" s="35" t="n"/>
+      <c r="W19" s="35" t="n"/>
+      <c r="X19" s="35" t="n"/>
+      <c r="Y19" s="35" t="n"/>
+      <c r="Z19" s="35" t="n"/>
+      <c r="AA19" s="35" t="n"/>
+      <c r="AB19" s="35" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>조치내용</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="51" t="inlineStr"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="7" t="n"/>
+      <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
+      <c r="N20" s="7" t="n"/>
+      <c r="O20" s="7" t="n"/>
+      <c r="P20" s="7" t="n"/>
+      <c r="Q20" s="7" t="n"/>
+      <c r="R20" s="7" t="n"/>
+      <c r="S20" s="7" t="n"/>
+      <c r="T20" s="7" t="n"/>
+      <c r="U20" s="7" t="n"/>
+      <c r="V20" s="7" t="n"/>
+      <c r="W20" s="7" t="n"/>
+      <c r="X20" s="7" t="n"/>
+      <c r="Y20" s="7" t="n"/>
+      <c r="Z20" s="7" t="n"/>
+      <c r="AA20" s="7" t="n"/>
+      <c r="AB20" s="7" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="19" t="n"/>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="7" t="n"/>
+      <c r="K21" s="7" t="n"/>
+      <c r="L21" s="7" t="n"/>
+      <c r="M21" s="7" t="n"/>
+      <c r="N21" s="7" t="n"/>
+      <c r="O21" s="7" t="n"/>
+      <c r="P21" s="7" t="n"/>
+      <c r="Q21" s="7" t="n"/>
+      <c r="R21" s="7" t="n"/>
+      <c r="S21" s="7" t="n"/>
+      <c r="T21" s="7" t="n"/>
+      <c r="U21" s="7" t="n"/>
+      <c r="V21" s="7" t="n"/>
+      <c r="W21" s="7" t="n"/>
+      <c r="X21" s="7" t="n"/>
+      <c r="Y21" s="7" t="n"/>
+      <c r="Z21" s="7" t="n"/>
+      <c r="AA21" s="7" t="n"/>
+      <c r="AB21" s="7" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>조치일자</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="12" t="inlineStr"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="36" t="inlineStr">
+        <is>
+          <t>확인자</t>
+        </is>
+      </c>
+      <c r="K22" s="19" t="n"/>
+      <c r="L22" s="19" t="n"/>
+      <c r="M22" s="12" t="inlineStr"/>
+      <c r="N22" s="7" t="n"/>
+      <c r="O22" s="7" t="n"/>
+      <c r="P22" s="7" t="n"/>
+      <c r="Q22" s="7" t="n"/>
+      <c r="R22" s="7" t="n"/>
+      <c r="S22" s="7" t="n"/>
+      <c r="T22" s="7" t="n"/>
+      <c r="U22" s="7" t="n"/>
+      <c r="V22" s="7" t="n"/>
+      <c r="W22" s="7" t="n"/>
+      <c r="X22" s="7" t="n"/>
+      <c r="Y22" s="7" t="n"/>
+      <c r="Z22" s="7" t="n"/>
+      <c r="AA22" s="7" t="n"/>
+      <c r="AB22" s="7" t="n"/>
+    </row>
+    <row r="23" ht="14" customHeight="1"/>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="47" t="inlineStr">
+        <is>
+          <t>No.2</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="36" t="inlineStr">
+        <is>
+          <t>지적사항 내용</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="19" t="n"/>
+      <c r="H24" s="19" t="n"/>
+      <c r="I24" s="48" t="inlineStr"/>
+      <c r="J24" s="7" t="n"/>
+      <c r="K24" s="7" t="n"/>
+      <c r="L24" s="7" t="n"/>
+      <c r="M24" s="7" t="n"/>
+      <c r="N24" s="7" t="n"/>
+      <c r="O24" s="7" t="n"/>
+      <c r="P24" s="7" t="n"/>
+      <c r="Q24" s="7" t="n"/>
+      <c r="R24" s="7" t="n"/>
+      <c r="S24" s="7" t="n"/>
+      <c r="T24" s="7" t="n"/>
+      <c r="U24" s="7" t="n"/>
+      <c r="V24" s="7" t="n"/>
+      <c r="W24" s="7" t="n"/>
+      <c r="X24" s="7" t="n"/>
+      <c r="Y24" s="7" t="n"/>
+      <c r="Z24" s="7" t="n"/>
+      <c r="AA24" s="7" t="n"/>
+      <c r="AB24" s="7" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>▼ 조치 전 (Before)</t>
+        </is>
+      </c>
+      <c r="P25" s="50" t="inlineStr">
+        <is>
+          <t>▼ 조치 후 (After)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="B26" s="34" t="inlineStr">
+        <is>
+          <t>사진 삽입 영역</t>
+        </is>
+      </c>
+      <c r="C26" s="35" t="n"/>
+      <c r="D26" s="35" t="n"/>
+      <c r="E26" s="35" t="n"/>
+      <c r="F26" s="35" t="n"/>
+      <c r="G26" s="35" t="n"/>
+      <c r="H26" s="35" t="n"/>
+      <c r="I26" s="35" t="n"/>
+      <c r="J26" s="35" t="n"/>
+      <c r="K26" s="35" t="n"/>
+      <c r="L26" s="35" t="n"/>
+      <c r="M26" s="35" t="n"/>
+      <c r="N26" s="35" t="n"/>
+      <c r="P26" s="34" t="inlineStr">
+        <is>
+          <t>사진 삽입 영역</t>
+        </is>
+      </c>
+      <c r="Q26" s="35" t="n"/>
+      <c r="R26" s="35" t="n"/>
+      <c r="S26" s="35" t="n"/>
+      <c r="T26" s="35" t="n"/>
+      <c r="U26" s="35" t="n"/>
+      <c r="V26" s="35" t="n"/>
+      <c r="W26" s="35" t="n"/>
+      <c r="X26" s="35" t="n"/>
+      <c r="Y26" s="35" t="n"/>
+      <c r="Z26" s="35" t="n"/>
+      <c r="AA26" s="35" t="n"/>
+      <c r="AB26" s="35" t="n"/>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="B27" s="35" t="n"/>
+      <c r="C27" s="35" t="n"/>
+      <c r="D27" s="35" t="n"/>
+      <c r="E27" s="35" t="n"/>
+      <c r="F27" s="35" t="n"/>
+      <c r="G27" s="35" t="n"/>
+      <c r="H27" s="35" t="n"/>
+      <c r="I27" s="35" t="n"/>
+      <c r="J27" s="35" t="n"/>
+      <c r="K27" s="35" t="n"/>
+      <c r="L27" s="35" t="n"/>
+      <c r="M27" s="35" t="n"/>
+      <c r="N27" s="35" t="n"/>
+      <c r="P27" s="35" t="n"/>
+      <c r="Q27" s="35" t="n"/>
+      <c r="R27" s="35" t="n"/>
+      <c r="S27" s="35" t="n"/>
+      <c r="T27" s="35" t="n"/>
+      <c r="U27" s="35" t="n"/>
+      <c r="V27" s="35" t="n"/>
+      <c r="W27" s="35" t="n"/>
+      <c r="X27" s="35" t="n"/>
+      <c r="Y27" s="35" t="n"/>
+      <c r="Z27" s="35" t="n"/>
+      <c r="AA27" s="35" t="n"/>
+      <c r="AB27" s="35" t="n"/>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="B28" s="35" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="35" t="n"/>
+      <c r="G28" s="35" t="n"/>
+      <c r="H28" s="35" t="n"/>
+      <c r="I28" s="35" t="n"/>
+      <c r="J28" s="35" t="n"/>
+      <c r="K28" s="35" t="n"/>
+      <c r="L28" s="35" t="n"/>
+      <c r="M28" s="35" t="n"/>
+      <c r="N28" s="35" t="n"/>
+      <c r="P28" s="35" t="n"/>
+      <c r="Q28" s="35" t="n"/>
+      <c r="R28" s="35" t="n"/>
+      <c r="S28" s="35" t="n"/>
+      <c r="T28" s="35" t="n"/>
+      <c r="U28" s="35" t="n"/>
+      <c r="V28" s="35" t="n"/>
+      <c r="W28" s="35" t="n"/>
+      <c r="X28" s="35" t="n"/>
+      <c r="Y28" s="35" t="n"/>
+      <c r="Z28" s="35" t="n"/>
+      <c r="AA28" s="35" t="n"/>
+      <c r="AB28" s="35" t="n"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="B29" s="35" t="n"/>
+      <c r="C29" s="35" t="n"/>
+      <c r="D29" s="35" t="n"/>
+      <c r="E29" s="35" t="n"/>
+      <c r="F29" s="35" t="n"/>
+      <c r="G29" s="35" t="n"/>
+      <c r="H29" s="35" t="n"/>
+      <c r="I29" s="35" t="n"/>
+      <c r="J29" s="35" t="n"/>
+      <c r="K29" s="35" t="n"/>
+      <c r="L29" s="35" t="n"/>
+      <c r="M29" s="35" t="n"/>
+      <c r="N29" s="35" t="n"/>
+      <c r="P29" s="35" t="n"/>
+      <c r="Q29" s="35" t="n"/>
+      <c r="R29" s="35" t="n"/>
+      <c r="S29" s="35" t="n"/>
+      <c r="T29" s="35" t="n"/>
+      <c r="U29" s="35" t="n"/>
+      <c r="V29" s="35" t="n"/>
+      <c r="W29" s="35" t="n"/>
+      <c r="X29" s="35" t="n"/>
+      <c r="Y29" s="35" t="n"/>
+      <c r="Z29" s="35" t="n"/>
+      <c r="AA29" s="35" t="n"/>
+      <c r="AB29" s="35" t="n"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="B30" s="35" t="n"/>
+      <c r="C30" s="35" t="n"/>
+      <c r="D30" s="35" t="n"/>
+      <c r="E30" s="35" t="n"/>
+      <c r="F30" s="35" t="n"/>
+      <c r="G30" s="35" t="n"/>
+      <c r="H30" s="35" t="n"/>
+      <c r="I30" s="35" t="n"/>
+      <c r="J30" s="35" t="n"/>
+      <c r="K30" s="35" t="n"/>
+      <c r="L30" s="35" t="n"/>
+      <c r="M30" s="35" t="n"/>
+      <c r="N30" s="35" t="n"/>
+      <c r="P30" s="35" t="n"/>
+      <c r="Q30" s="35" t="n"/>
+      <c r="R30" s="35" t="n"/>
+      <c r="S30" s="35" t="n"/>
+      <c r="T30" s="35" t="n"/>
+      <c r="U30" s="35" t="n"/>
+      <c r="V30" s="35" t="n"/>
+      <c r="W30" s="35" t="n"/>
+      <c r="X30" s="35" t="n"/>
+      <c r="Y30" s="35" t="n"/>
+      <c r="Z30" s="35" t="n"/>
+      <c r="AA30" s="35" t="n"/>
+      <c r="AB30" s="35" t="n"/>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="B31" s="35" t="n"/>
+      <c r="C31" s="35" t="n"/>
+      <c r="D31" s="35" t="n"/>
+      <c r="E31" s="35" t="n"/>
+      <c r="F31" s="35" t="n"/>
+      <c r="G31" s="35" t="n"/>
+      <c r="H31" s="35" t="n"/>
+      <c r="I31" s="35" t="n"/>
+      <c r="J31" s="35" t="n"/>
+      <c r="K31" s="35" t="n"/>
+      <c r="L31" s="35" t="n"/>
+      <c r="M31" s="35" t="n"/>
+      <c r="N31" s="35" t="n"/>
+      <c r="P31" s="35" t="n"/>
+      <c r="Q31" s="35" t="n"/>
+      <c r="R31" s="35" t="n"/>
+      <c r="S31" s="35" t="n"/>
+      <c r="T31" s="35" t="n"/>
+      <c r="U31" s="35" t="n"/>
+      <c r="V31" s="35" t="n"/>
+      <c r="W31" s="35" t="n"/>
+      <c r="X31" s="35" t="n"/>
+      <c r="Y31" s="35" t="n"/>
+      <c r="Z31" s="35" t="n"/>
+      <c r="AA31" s="35" t="n"/>
+      <c r="AB31" s="35" t="n"/>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="B32" s="35" t="n"/>
+      <c r="C32" s="35" t="n"/>
+      <c r="D32" s="35" t="n"/>
+      <c r="E32" s="35" t="n"/>
+      <c r="F32" s="35" t="n"/>
+      <c r="G32" s="35" t="n"/>
+      <c r="H32" s="35" t="n"/>
+      <c r="I32" s="35" t="n"/>
+      <c r="J32" s="35" t="n"/>
+      <c r="K32" s="35" t="n"/>
+      <c r="L32" s="35" t="n"/>
+      <c r="M32" s="35" t="n"/>
+      <c r="N32" s="35" t="n"/>
+      <c r="P32" s="35" t="n"/>
+      <c r="Q32" s="35" t="n"/>
+      <c r="R32" s="35" t="n"/>
+      <c r="S32" s="35" t="n"/>
+      <c r="T32" s="35" t="n"/>
+      <c r="U32" s="35" t="n"/>
+      <c r="V32" s="35" t="n"/>
+      <c r="W32" s="35" t="n"/>
+      <c r="X32" s="35" t="n"/>
+      <c r="Y32" s="35" t="n"/>
+      <c r="Z32" s="35" t="n"/>
+      <c r="AA32" s="35" t="n"/>
+      <c r="AB32" s="35" t="n"/>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="B33" s="35" t="n"/>
+      <c r="C33" s="35" t="n"/>
+      <c r="D33" s="35" t="n"/>
+      <c r="E33" s="35" t="n"/>
+      <c r="F33" s="35" t="n"/>
+      <c r="G33" s="35" t="n"/>
+      <c r="H33" s="35" t="n"/>
+      <c r="I33" s="35" t="n"/>
+      <c r="J33" s="35" t="n"/>
+      <c r="K33" s="35" t="n"/>
+      <c r="L33" s="35" t="n"/>
+      <c r="M33" s="35" t="n"/>
+      <c r="N33" s="35" t="n"/>
+      <c r="P33" s="35" t="n"/>
+      <c r="Q33" s="35" t="n"/>
+      <c r="R33" s="35" t="n"/>
+      <c r="S33" s="35" t="n"/>
+      <c r="T33" s="35" t="n"/>
+      <c r="U33" s="35" t="n"/>
+      <c r="V33" s="35" t="n"/>
+      <c r="W33" s="35" t="n"/>
+      <c r="X33" s="35" t="n"/>
+      <c r="Y33" s="35" t="n"/>
+      <c r="Z33" s="35" t="n"/>
+      <c r="AA33" s="35" t="n"/>
+      <c r="AB33" s="35" t="n"/>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="B34" s="35" t="n"/>
+      <c r="C34" s="35" t="n"/>
+      <c r="D34" s="35" t="n"/>
+      <c r="E34" s="35" t="n"/>
+      <c r="F34" s="35" t="n"/>
+      <c r="G34" s="35" t="n"/>
+      <c r="H34" s="35" t="n"/>
+      <c r="I34" s="35" t="n"/>
+      <c r="J34" s="35" t="n"/>
+      <c r="K34" s="35" t="n"/>
+      <c r="L34" s="35" t="n"/>
+      <c r="M34" s="35" t="n"/>
+      <c r="N34" s="35" t="n"/>
+      <c r="P34" s="35" t="n"/>
+      <c r="Q34" s="35" t="n"/>
+      <c r="R34" s="35" t="n"/>
+      <c r="S34" s="35" t="n"/>
+      <c r="T34" s="35" t="n"/>
+      <c r="U34" s="35" t="n"/>
+      <c r="V34" s="35" t="n"/>
+      <c r="W34" s="35" t="n"/>
+      <c r="X34" s="35" t="n"/>
+      <c r="Y34" s="35" t="n"/>
+      <c r="Z34" s="35" t="n"/>
+      <c r="AA34" s="35" t="n"/>
+      <c r="AB34" s="35" t="n"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="B35" s="35" t="n"/>
+      <c r="C35" s="35" t="n"/>
+      <c r="D35" s="35" t="n"/>
+      <c r="E35" s="35" t="n"/>
+      <c r="F35" s="35" t="n"/>
+      <c r="G35" s="35" t="n"/>
+      <c r="H35" s="35" t="n"/>
+      <c r="I35" s="35" t="n"/>
+      <c r="J35" s="35" t="n"/>
+      <c r="K35" s="35" t="n"/>
+      <c r="L35" s="35" t="n"/>
+      <c r="M35" s="35" t="n"/>
+      <c r="N35" s="35" t="n"/>
+      <c r="P35" s="35" t="n"/>
+      <c r="Q35" s="35" t="n"/>
+      <c r="R35" s="35" t="n"/>
+      <c r="S35" s="35" t="n"/>
+      <c r="T35" s="35" t="n"/>
+      <c r="U35" s="35" t="n"/>
+      <c r="V35" s="35" t="n"/>
+      <c r="W35" s="35" t="n"/>
+      <c r="X35" s="35" t="n"/>
+      <c r="Y35" s="35" t="n"/>
+      <c r="Z35" s="35" t="n"/>
+      <c r="AA35" s="35" t="n"/>
+      <c r="AB35" s="35" t="n"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="B36" s="35" t="n"/>
+      <c r="C36" s="35" t="n"/>
+      <c r="D36" s="35" t="n"/>
+      <c r="E36" s="35" t="n"/>
+      <c r="F36" s="35" t="n"/>
+      <c r="G36" s="35" t="n"/>
+      <c r="H36" s="35" t="n"/>
+      <c r="I36" s="35" t="n"/>
+      <c r="J36" s="35" t="n"/>
+      <c r="K36" s="35" t="n"/>
+      <c r="L36" s="35" t="n"/>
+      <c r="M36" s="35" t="n"/>
+      <c r="N36" s="35" t="n"/>
+      <c r="P36" s="35" t="n"/>
+      <c r="Q36" s="35" t="n"/>
+      <c r="R36" s="35" t="n"/>
+      <c r="S36" s="35" t="n"/>
+      <c r="T36" s="35" t="n"/>
+      <c r="U36" s="35" t="n"/>
+      <c r="V36" s="35" t="n"/>
+      <c r="W36" s="35" t="n"/>
+      <c r="X36" s="35" t="n"/>
+      <c r="Y36" s="35" t="n"/>
+      <c r="Z36" s="35" t="n"/>
+      <c r="AA36" s="35" t="n"/>
+      <c r="AB36" s="35" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="B37" s="36" t="inlineStr">
+        <is>
+          <t>조치내용</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="51" t="inlineStr"/>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="7" t="n"/>
+      <c r="I37" s="7" t="n"/>
+      <c r="J37" s="7" t="n"/>
+      <c r="K37" s="7" t="n"/>
+      <c r="L37" s="7" t="n"/>
+      <c r="M37" s="7" t="n"/>
+      <c r="N37" s="7" t="n"/>
+      <c r="O37" s="7" t="n"/>
+      <c r="P37" s="7" t="n"/>
+      <c r="Q37" s="7" t="n"/>
+      <c r="R37" s="7" t="n"/>
+      <c r="S37" s="7" t="n"/>
+      <c r="T37" s="7" t="n"/>
+      <c r="U37" s="7" t="n"/>
+      <c r="V37" s="7" t="n"/>
+      <c r="W37" s="7" t="n"/>
+      <c r="X37" s="7" t="n"/>
+      <c r="Y37" s="7" t="n"/>
+      <c r="Z37" s="7" t="n"/>
+      <c r="AA37" s="7" t="n"/>
+      <c r="AB37" s="7" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="B38" s="19" t="n"/>
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="7" t="n"/>
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="n"/>
+      <c r="H38" s="7" t="n"/>
+      <c r="I38" s="7" t="n"/>
+      <c r="J38" s="7" t="n"/>
+      <c r="K38" s="7" t="n"/>
+      <c r="L38" s="7" t="n"/>
+      <c r="M38" s="7" t="n"/>
+      <c r="N38" s="7" t="n"/>
+      <c r="O38" s="7" t="n"/>
+      <c r="P38" s="7" t="n"/>
+      <c r="Q38" s="7" t="n"/>
+      <c r="R38" s="7" t="n"/>
+      <c r="S38" s="7" t="n"/>
+      <c r="T38" s="7" t="n"/>
+      <c r="U38" s="7" t="n"/>
+      <c r="V38" s="7" t="n"/>
+      <c r="W38" s="7" t="n"/>
+      <c r="X38" s="7" t="n"/>
+      <c r="Y38" s="7" t="n"/>
+      <c r="Z38" s="7" t="n"/>
+      <c r="AA38" s="7" t="n"/>
+      <c r="AB38" s="7" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="B39" s="36" t="inlineStr">
+        <is>
+          <t>조치일자</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="12" t="inlineStr"/>
+      <c r="E39" s="7" t="n"/>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="7" t="n"/>
+      <c r="H39" s="7" t="n"/>
+      <c r="I39" s="7" t="n"/>
+      <c r="J39" s="36" t="inlineStr">
+        <is>
+          <t>확인자</t>
+        </is>
+      </c>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="12" t="inlineStr"/>
+      <c r="N39" s="7" t="n"/>
+      <c r="O39" s="7" t="n"/>
+      <c r="P39" s="7" t="n"/>
+      <c r="Q39" s="7" t="n"/>
+      <c r="R39" s="7" t="n"/>
+      <c r="S39" s="7" t="n"/>
+      <c r="T39" s="7" t="n"/>
+      <c r="U39" s="7" t="n"/>
+      <c r="V39" s="7" t="n"/>
+      <c r="W39" s="7" t="n"/>
+      <c r="X39" s="7" t="n"/>
+      <c r="Y39" s="7" t="n"/>
+      <c r="Z39" s="7" t="n"/>
+      <c r="AA39" s="7" t="n"/>
+      <c r="AB39" s="7" t="n"/>
+    </row>
+    <row r="40" ht="14" customHeight="1"/>
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="47" t="inlineStr">
+        <is>
+          <t>No.3</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="36" t="inlineStr">
+        <is>
+          <t>지적사항 내용</t>
+        </is>
+      </c>
+      <c r="E41" s="19" t="n"/>
+      <c r="F41" s="19" t="n"/>
+      <c r="G41" s="19" t="n"/>
+      <c r="H41" s="19" t="n"/>
+      <c r="I41" s="48" t="inlineStr"/>
+      <c r="J41" s="7" t="n"/>
+      <c r="K41" s="7" t="n"/>
+      <c r="L41" s="7" t="n"/>
+      <c r="M41" s="7" t="n"/>
+      <c r="N41" s="7" t="n"/>
+      <c r="O41" s="7" t="n"/>
+      <c r="P41" s="7" t="n"/>
+      <c r="Q41" s="7" t="n"/>
+      <c r="R41" s="7" t="n"/>
+      <c r="S41" s="7" t="n"/>
+      <c r="T41" s="7" t="n"/>
+      <c r="U41" s="7" t="n"/>
+      <c r="V41" s="7" t="n"/>
+      <c r="W41" s="7" t="n"/>
+      <c r="X41" s="7" t="n"/>
+      <c r="Y41" s="7" t="n"/>
+      <c r="Z41" s="7" t="n"/>
+      <c r="AA41" s="7" t="n"/>
+      <c r="AB41" s="7" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>▼ 조치 전 (Before)</t>
+        </is>
+      </c>
+      <c r="P42" s="50" t="inlineStr">
+        <is>
+          <t>▼ 조치 후 (After)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="B43" s="34" t="inlineStr">
+        <is>
+          <t>사진 삽입 영역</t>
+        </is>
+      </c>
+      <c r="C43" s="35" t="n"/>
+      <c r="D43" s="35" t="n"/>
+      <c r="E43" s="35" t="n"/>
+      <c r="F43" s="35" t="n"/>
+      <c r="G43" s="35" t="n"/>
+      <c r="H43" s="35" t="n"/>
+      <c r="I43" s="35" t="n"/>
+      <c r="J43" s="35" t="n"/>
+      <c r="K43" s="35" t="n"/>
+      <c r="L43" s="35" t="n"/>
+      <c r="M43" s="35" t="n"/>
+      <c r="N43" s="35" t="n"/>
+      <c r="P43" s="34" t="inlineStr">
+        <is>
+          <t>사진 삽입 영역</t>
+        </is>
+      </c>
+      <c r="Q43" s="35" t="n"/>
+      <c r="R43" s="35" t="n"/>
+      <c r="S43" s="35" t="n"/>
+      <c r="T43" s="35" t="n"/>
+      <c r="U43" s="35" t="n"/>
+      <c r="V43" s="35" t="n"/>
+      <c r="W43" s="35" t="n"/>
+      <c r="X43" s="35" t="n"/>
+      <c r="Y43" s="35" t="n"/>
+      <c r="Z43" s="35" t="n"/>
+      <c r="AA43" s="35" t="n"/>
+      <c r="AB43" s="35" t="n"/>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="B44" s="35" t="n"/>
+      <c r="C44" s="35" t="n"/>
+      <c r="D44" s="35" t="n"/>
+      <c r="E44" s="35" t="n"/>
+      <c r="F44" s="35" t="n"/>
+      <c r="G44" s="35" t="n"/>
+      <c r="H44" s="35" t="n"/>
+      <c r="I44" s="35" t="n"/>
+      <c r="J44" s="35" t="n"/>
+      <c r="K44" s="35" t="n"/>
+      <c r="L44" s="35" t="n"/>
+      <c r="M44" s="35" t="n"/>
+      <c r="N44" s="35" t="n"/>
+      <c r="P44" s="35" t="n"/>
+      <c r="Q44" s="35" t="n"/>
+      <c r="R44" s="35" t="n"/>
+      <c r="S44" s="35" t="n"/>
+      <c r="T44" s="35" t="n"/>
+      <c r="U44" s="35" t="n"/>
+      <c r="V44" s="35" t="n"/>
+      <c r="W44" s="35" t="n"/>
+      <c r="X44" s="35" t="n"/>
+      <c r="Y44" s="35" t="n"/>
+      <c r="Z44" s="35" t="n"/>
+      <c r="AA44" s="35" t="n"/>
+      <c r="AB44" s="35" t="n"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="B45" s="35" t="n"/>
+      <c r="C45" s="35" t="n"/>
+      <c r="D45" s="35" t="n"/>
+      <c r="E45" s="35" t="n"/>
+      <c r="F45" s="35" t="n"/>
+      <c r="G45" s="35" t="n"/>
+      <c r="H45" s="35" t="n"/>
+      <c r="I45" s="35" t="n"/>
+      <c r="J45" s="35" t="n"/>
+      <c r="K45" s="35" t="n"/>
+      <c r="L45" s="35" t="n"/>
+      <c r="M45" s="35" t="n"/>
+      <c r="N45" s="35" t="n"/>
+      <c r="P45" s="35" t="n"/>
+      <c r="Q45" s="35" t="n"/>
+      <c r="R45" s="35" t="n"/>
+      <c r="S45" s="35" t="n"/>
+      <c r="T45" s="35" t="n"/>
+      <c r="U45" s="35" t="n"/>
+      <c r="V45" s="35" t="n"/>
+      <c r="W45" s="35" t="n"/>
+      <c r="X45" s="35" t="n"/>
+      <c r="Y45" s="35" t="n"/>
+      <c r="Z45" s="35" t="n"/>
+      <c r="AA45" s="35" t="n"/>
+      <c r="AB45" s="35" t="n"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="B46" s="35" t="n"/>
+      <c r="C46" s="35" t="n"/>
+      <c r="D46" s="35" t="n"/>
+      <c r="E46" s="35" t="n"/>
+      <c r="F46" s="35" t="n"/>
+      <c r="G46" s="35" t="n"/>
+      <c r="H46" s="35" t="n"/>
+      <c r="I46" s="35" t="n"/>
+      <c r="J46" s="35" t="n"/>
+      <c r="K46" s="35" t="n"/>
+      <c r="L46" s="35" t="n"/>
+      <c r="M46" s="35" t="n"/>
+      <c r="N46" s="35" t="n"/>
+      <c r="P46" s="35" t="n"/>
+      <c r="Q46" s="35" t="n"/>
+      <c r="R46" s="35" t="n"/>
+      <c r="S46" s="35" t="n"/>
+      <c r="T46" s="35" t="n"/>
+      <c r="U46" s="35" t="n"/>
+      <c r="V46" s="35" t="n"/>
+      <c r="W46" s="35" t="n"/>
+      <c r="X46" s="35" t="n"/>
+      <c r="Y46" s="35" t="n"/>
+      <c r="Z46" s="35" t="n"/>
+      <c r="AA46" s="35" t="n"/>
+      <c r="AB46" s="35" t="n"/>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="B47" s="35" t="n"/>
+      <c r="C47" s="35" t="n"/>
+      <c r="D47" s="35" t="n"/>
+      <c r="E47" s="35" t="n"/>
+      <c r="F47" s="35" t="n"/>
+      <c r="G47" s="35" t="n"/>
+      <c r="H47" s="35" t="n"/>
+      <c r="I47" s="35" t="n"/>
+      <c r="J47" s="35" t="n"/>
+      <c r="K47" s="35" t="n"/>
+      <c r="L47" s="35" t="n"/>
+      <c r="M47" s="35" t="n"/>
+      <c r="N47" s="35" t="n"/>
+      <c r="P47" s="35" t="n"/>
+      <c r="Q47" s="35" t="n"/>
+      <c r="R47" s="35" t="n"/>
+      <c r="S47" s="35" t="n"/>
+      <c r="T47" s="35" t="n"/>
+      <c r="U47" s="35" t="n"/>
+      <c r="V47" s="35" t="n"/>
+      <c r="W47" s="35" t="n"/>
+      <c r="X47" s="35" t="n"/>
+      <c r="Y47" s="35" t="n"/>
+      <c r="Z47" s="35" t="n"/>
+      <c r="AA47" s="35" t="n"/>
+      <c r="AB47" s="35" t="n"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="B48" s="35" t="n"/>
+      <c r="C48" s="35" t="n"/>
+      <c r="D48" s="35" t="n"/>
+      <c r="E48" s="35" t="n"/>
+      <c r="F48" s="35" t="n"/>
+      <c r="G48" s="35" t="n"/>
+      <c r="H48" s="35" t="n"/>
+      <c r="I48" s="35" t="n"/>
+      <c r="J48" s="35" t="n"/>
+      <c r="K48" s="35" t="n"/>
+      <c r="L48" s="35" t="n"/>
+      <c r="M48" s="35" t="n"/>
+      <c r="N48" s="35" t="n"/>
+      <c r="P48" s="35" t="n"/>
+      <c r="Q48" s="35" t="n"/>
+      <c r="R48" s="35" t="n"/>
+      <c r="S48" s="35" t="n"/>
+      <c r="T48" s="35" t="n"/>
+      <c r="U48" s="35" t="n"/>
+      <c r="V48" s="35" t="n"/>
+      <c r="W48" s="35" t="n"/>
+      <c r="X48" s="35" t="n"/>
+      <c r="Y48" s="35" t="n"/>
+      <c r="Z48" s="35" t="n"/>
+      <c r="AA48" s="35" t="n"/>
+      <c r="AB48" s="35" t="n"/>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="B49" s="35" t="n"/>
+      <c r="C49" s="35" t="n"/>
+      <c r="D49" s="35" t="n"/>
+      <c r="E49" s="35" t="n"/>
+      <c r="F49" s="35" t="n"/>
+      <c r="G49" s="35" t="n"/>
+      <c r="H49" s="35" t="n"/>
+      <c r="I49" s="35" t="n"/>
+      <c r="J49" s="35" t="n"/>
+      <c r="K49" s="35" t="n"/>
+      <c r="L49" s="35" t="n"/>
+      <c r="M49" s="35" t="n"/>
+      <c r="N49" s="35" t="n"/>
+      <c r="P49" s="35" t="n"/>
+      <c r="Q49" s="35" t="n"/>
+      <c r="R49" s="35" t="n"/>
+      <c r="S49" s="35" t="n"/>
+      <c r="T49" s="35" t="n"/>
+      <c r="U49" s="35" t="n"/>
+      <c r="V49" s="35" t="n"/>
+      <c r="W49" s="35" t="n"/>
+      <c r="X49" s="35" t="n"/>
+      <c r="Y49" s="35" t="n"/>
+      <c r="Z49" s="35" t="n"/>
+      <c r="AA49" s="35" t="n"/>
+      <c r="AB49" s="35" t="n"/>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="B50" s="35" t="n"/>
+      <c r="C50" s="35" t="n"/>
+      <c r="D50" s="35" t="n"/>
+      <c r="E50" s="35" t="n"/>
+      <c r="F50" s="35" t="n"/>
+      <c r="G50" s="35" t="n"/>
+      <c r="H50" s="35" t="n"/>
+      <c r="I50" s="35" t="n"/>
+      <c r="J50" s="35" t="n"/>
+      <c r="K50" s="35" t="n"/>
+      <c r="L50" s="35" t="n"/>
+      <c r="M50" s="35" t="n"/>
+      <c r="N50" s="35" t="n"/>
+      <c r="P50" s="35" t="n"/>
+      <c r="Q50" s="35" t="n"/>
+      <c r="R50" s="35" t="n"/>
+      <c r="S50" s="35" t="n"/>
+      <c r="T50" s="35" t="n"/>
+      <c r="U50" s="35" t="n"/>
+      <c r="V50" s="35" t="n"/>
+      <c r="W50" s="35" t="n"/>
+      <c r="X50" s="35" t="n"/>
+      <c r="Y50" s="35" t="n"/>
+      <c r="Z50" s="35" t="n"/>
+      <c r="AA50" s="35" t="n"/>
+      <c r="AB50" s="35" t="n"/>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="B51" s="35" t="n"/>
+      <c r="C51" s="35" t="n"/>
+      <c r="D51" s="35" t="n"/>
+      <c r="E51" s="35" t="n"/>
+      <c r="F51" s="35" t="n"/>
+      <c r="G51" s="35" t="n"/>
+      <c r="H51" s="35" t="n"/>
+      <c r="I51" s="35" t="n"/>
+      <c r="J51" s="35" t="n"/>
+      <c r="K51" s="35" t="n"/>
+      <c r="L51" s="35" t="n"/>
+      <c r="M51" s="35" t="n"/>
+      <c r="N51" s="35" t="n"/>
+      <c r="P51" s="35" t="n"/>
+      <c r="Q51" s="35" t="n"/>
+      <c r="R51" s="35" t="n"/>
+      <c r="S51" s="35" t="n"/>
+      <c r="T51" s="35" t="n"/>
+      <c r="U51" s="35" t="n"/>
+      <c r="V51" s="35" t="n"/>
+      <c r="W51" s="35" t="n"/>
+      <c r="X51" s="35" t="n"/>
+      <c r="Y51" s="35" t="n"/>
+      <c r="Z51" s="35" t="n"/>
+      <c r="AA51" s="35" t="n"/>
+      <c r="AB51" s="35" t="n"/>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="B52" s="35" t="n"/>
+      <c r="C52" s="35" t="n"/>
+      <c r="D52" s="35" t="n"/>
+      <c r="E52" s="35" t="n"/>
+      <c r="F52" s="35" t="n"/>
+      <c r="G52" s="35" t="n"/>
+      <c r="H52" s="35" t="n"/>
+      <c r="I52" s="35" t="n"/>
+      <c r="J52" s="35" t="n"/>
+      <c r="K52" s="35" t="n"/>
+      <c r="L52" s="35" t="n"/>
+      <c r="M52" s="35" t="n"/>
+      <c r="N52" s="35" t="n"/>
+      <c r="P52" s="35" t="n"/>
+      <c r="Q52" s="35" t="n"/>
+      <c r="R52" s="35" t="n"/>
+      <c r="S52" s="35" t="n"/>
+      <c r="T52" s="35" t="n"/>
+      <c r="U52" s="35" t="n"/>
+      <c r="V52" s="35" t="n"/>
+      <c r="W52" s="35" t="n"/>
+      <c r="X52" s="35" t="n"/>
+      <c r="Y52" s="35" t="n"/>
+      <c r="Z52" s="35" t="n"/>
+      <c r="AA52" s="35" t="n"/>
+      <c r="AB52" s="35" t="n"/>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="B53" s="35" t="n"/>
+      <c r="C53" s="35" t="n"/>
+      <c r="D53" s="35" t="n"/>
+      <c r="E53" s="35" t="n"/>
+      <c r="F53" s="35" t="n"/>
+      <c r="G53" s="35" t="n"/>
+      <c r="H53" s="35" t="n"/>
+      <c r="I53" s="35" t="n"/>
+      <c r="J53" s="35" t="n"/>
+      <c r="K53" s="35" t="n"/>
+      <c r="L53" s="35" t="n"/>
+      <c r="M53" s="35" t="n"/>
+      <c r="N53" s="35" t="n"/>
+      <c r="P53" s="35" t="n"/>
+      <c r="Q53" s="35" t="n"/>
+      <c r="R53" s="35" t="n"/>
+      <c r="S53" s="35" t="n"/>
+      <c r="T53" s="35" t="n"/>
+      <c r="U53" s="35" t="n"/>
+      <c r="V53" s="35" t="n"/>
+      <c r="W53" s="35" t="n"/>
+      <c r="X53" s="35" t="n"/>
+      <c r="Y53" s="35" t="n"/>
+      <c r="Z53" s="35" t="n"/>
+      <c r="AA53" s="35" t="n"/>
+      <c r="AB53" s="35" t="n"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="B54" s="36" t="inlineStr">
+        <is>
+          <t>조치내용</t>
+        </is>
+      </c>
+      <c r="C54" s="19" t="n"/>
+      <c r="D54" s="51" t="inlineStr"/>
+      <c r="E54" s="7" t="n"/>
+      <c r="F54" s="7" t="n"/>
+      <c r="G54" s="7" t="n"/>
+      <c r="H54" s="7" t="n"/>
+      <c r="I54" s="7" t="n"/>
+      <c r="J54" s="7" t="n"/>
+      <c r="K54" s="7" t="n"/>
+      <c r="L54" s="7" t="n"/>
+      <c r="M54" s="7" t="n"/>
+      <c r="N54" s="7" t="n"/>
+      <c r="O54" s="7" t="n"/>
+      <c r="P54" s="7" t="n"/>
+      <c r="Q54" s="7" t="n"/>
+      <c r="R54" s="7" t="n"/>
+      <c r="S54" s="7" t="n"/>
+      <c r="T54" s="7" t="n"/>
+      <c r="U54" s="7" t="n"/>
+      <c r="V54" s="7" t="n"/>
+      <c r="W54" s="7" t="n"/>
+      <c r="X54" s="7" t="n"/>
+      <c r="Y54" s="7" t="n"/>
+      <c r="Z54" s="7" t="n"/>
+      <c r="AA54" s="7" t="n"/>
+      <c r="AB54" s="7" t="n"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="B55" s="19" t="n"/>
+      <c r="C55" s="19" t="n"/>
+      <c r="D55" s="7" t="n"/>
+      <c r="E55" s="7" t="n"/>
+      <c r="F55" s="7" t="n"/>
+      <c r="G55" s="7" t="n"/>
+      <c r="H55" s="7" t="n"/>
+      <c r="I55" s="7" t="n"/>
+      <c r="J55" s="7" t="n"/>
+      <c r="K55" s="7" t="n"/>
+      <c r="L55" s="7" t="n"/>
+      <c r="M55" s="7" t="n"/>
+      <c r="N55" s="7" t="n"/>
+      <c r="O55" s="7" t="n"/>
+      <c r="P55" s="7" t="n"/>
+      <c r="Q55" s="7" t="n"/>
+      <c r="R55" s="7" t="n"/>
+      <c r="S55" s="7" t="n"/>
+      <c r="T55" s="7" t="n"/>
+      <c r="U55" s="7" t="n"/>
+      <c r="V55" s="7" t="n"/>
+      <c r="W55" s="7" t="n"/>
+      <c r="X55" s="7" t="n"/>
+      <c r="Y55" s="7" t="n"/>
+      <c r="Z55" s="7" t="n"/>
+      <c r="AA55" s="7" t="n"/>
+      <c r="AB55" s="7" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="36" t="inlineStr">
+        <is>
+          <t>조치일자</t>
+        </is>
+      </c>
+      <c r="C56" s="19" t="n"/>
+      <c r="D56" s="12" t="inlineStr"/>
+      <c r="E56" s="7" t="n"/>
+      <c r="F56" s="7" t="n"/>
+      <c r="G56" s="7" t="n"/>
+      <c r="H56" s="7" t="n"/>
+      <c r="I56" s="7" t="n"/>
+      <c r="J56" s="36" t="inlineStr">
+        <is>
+          <t>확인자</t>
+        </is>
+      </c>
+      <c r="K56" s="19" t="n"/>
+      <c r="L56" s="19" t="n"/>
+      <c r="M56" s="12" t="inlineStr"/>
+      <c r="N56" s="7" t="n"/>
+      <c r="O56" s="7" t="n"/>
+      <c r="P56" s="7" t="n"/>
+      <c r="Q56" s="7" t="n"/>
+      <c r="R56" s="7" t="n"/>
+      <c r="S56" s="7" t="n"/>
+      <c r="T56" s="7" t="n"/>
+      <c r="U56" s="7" t="n"/>
+      <c r="V56" s="7" t="n"/>
+      <c r="W56" s="7" t="n"/>
+      <c r="X56" s="7" t="n"/>
+      <c r="Y56" s="7" t="n"/>
+      <c r="Z56" s="7" t="n"/>
+      <c r="AA56" s="7" t="n"/>
+      <c r="AB56" s="7" t="n"/>
+    </row>
+    <row r="57" ht="14" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="42">
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="P9:AB19"/>
+    <mergeCell ref="B2:AB2"/>
+    <mergeCell ref="B37:C38"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="P42:AB42"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="D56:I56"/>
+    <mergeCell ref="B20:C21"/>
+    <mergeCell ref="M56:AB56"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="I7:AB7"/>
+    <mergeCell ref="B54:C55"/>
+    <mergeCell ref="B25:N25"/>
+    <mergeCell ref="I41:AB41"/>
+    <mergeCell ref="J56:L56"/>
+    <mergeCell ref="D39:I39"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="P25:AB25"/>
+    <mergeCell ref="B9:N19"/>
+    <mergeCell ref="M39:AB39"/>
+    <mergeCell ref="J39:L39"/>
+    <mergeCell ref="B26:N36"/>
+    <mergeCell ref="B5:AB5"/>
+    <mergeCell ref="I24:AB24"/>
+    <mergeCell ref="P8:AB8"/>
+    <mergeCell ref="B42:N42"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D37:AB38"/>
+    <mergeCell ref="P43:AB53"/>
+    <mergeCell ref="B8:N8"/>
+    <mergeCell ref="D20:AB21"/>
+    <mergeCell ref="D22:I22"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="M22:AB22"/>
+    <mergeCell ref="P26:AB36"/>
+    <mergeCell ref="D54:AB55"/>
+    <mergeCell ref="B3:AB3"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B43:N53"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add result report and action plan sheets to management-responsible person's site patrol workbook
Adds 결과보고서 and 조치계획서 sheets to 경영책임자_현장순회점검표.xlsx:
- 결과보고서: findings summary by the 6 checklist categories (auto-summed
  good/poor/N-A counts), a major-findings list, overall comments, and a
  sign-off block for 경영책임자/현장소장/안전관리자
- 조치계획서: per-finding corrective action plan (cause analysis, action,
  owner, due date, budget, status, completion, confirmation)

Both sheets pull site name/date/inspector from the 현장순회점검표 sheet via
formulas, so the workbook now covers checklist -> photos -> before/after
evidence -> result report -> action plan end to end.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SqkinqfGqqfBrcHRBkScVm
</commit_message>
<xml_diff>
--- a/templates/경영책임자_현장순회점검표.xlsx
+++ b/templates/경영책임자_현장순회점검표.xlsx
@@ -10,11 +10,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현장순회점검표" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사진대지" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="지적사항_조치전후사진대지" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="결과보고서" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="조치계획서" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'현장순회점검표'!$A$1:$AB$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'사진대지'!$A$1:$AB$52</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'지적사항_조치전후사진대지'!$A$1:$AB$58</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'결과보고서'!$A$1:$AB$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'조치계획서'!$A$1:$AB$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -155,6 +159,16 @@
       <b val="1"/>
       <color rgb="FF2E7D32"/>
       <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="7">
@@ -416,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -519,6 +533,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -2976,32 +3008,6 @@
           <t>지적사항 조치 전·후 사진대지</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
-      <c r="V2" s="2" t="n"/>
-      <c r="W2" s="2" t="n"/>
-      <c r="X2" s="2" t="n"/>
-      <c r="Y2" s="2" t="n"/>
-      <c r="Z2" s="2" t="n"/>
-      <c r="AA2" s="2" t="n"/>
-      <c r="AB2" s="2" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
@@ -3025,36 +3031,36 @@
           <t>No.1</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n"/>
+      <c r="C7" s="23" t="n"/>
       <c r="D7" s="36" t="inlineStr">
         <is>
           <t>지적사항 내용</t>
         </is>
       </c>
-      <c r="E7" s="19" t="n"/>
-      <c r="F7" s="19" t="n"/>
-      <c r="G7" s="19" t="n"/>
-      <c r="H7" s="19" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="22" t="n"/>
+      <c r="H7" s="23" t="n"/>
       <c r="I7" s="48" t="inlineStr"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="n"/>
-      <c r="Q7" s="7" t="n"/>
-      <c r="R7" s="7" t="n"/>
-      <c r="S7" s="7" t="n"/>
-      <c r="T7" s="7" t="n"/>
-      <c r="U7" s="7" t="n"/>
-      <c r="V7" s="7" t="n"/>
-      <c r="W7" s="7" t="n"/>
-      <c r="X7" s="7" t="n"/>
-      <c r="Y7" s="7" t="n"/>
-      <c r="Z7" s="7" t="n"/>
-      <c r="AA7" s="7" t="n"/>
-      <c r="AB7" s="7" t="n"/>
+      <c r="J7" s="22" t="n"/>
+      <c r="K7" s="22" t="n"/>
+      <c r="L7" s="22" t="n"/>
+      <c r="M7" s="22" t="n"/>
+      <c r="N7" s="22" t="n"/>
+      <c r="O7" s="22" t="n"/>
+      <c r="P7" s="22" t="n"/>
+      <c r="Q7" s="22" t="n"/>
+      <c r="R7" s="22" t="n"/>
+      <c r="S7" s="22" t="n"/>
+      <c r="T7" s="22" t="n"/>
+      <c r="U7" s="22" t="n"/>
+      <c r="V7" s="22" t="n"/>
+      <c r="W7" s="22" t="n"/>
+      <c r="X7" s="22" t="n"/>
+      <c r="Y7" s="22" t="n"/>
+      <c r="Z7" s="22" t="n"/>
+      <c r="AA7" s="22" t="n"/>
+      <c r="AB7" s="23" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="49" t="inlineStr">
@@ -3074,315 +3080,117 @@
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="C9" s="35" t="n"/>
-      <c r="D9" s="35" t="n"/>
-      <c r="E9" s="35" t="n"/>
-      <c r="F9" s="35" t="n"/>
-      <c r="G9" s="35" t="n"/>
-      <c r="H9" s="35" t="n"/>
-      <c r="I9" s="35" t="n"/>
-      <c r="J9" s="35" t="n"/>
-      <c r="K9" s="35" t="n"/>
-      <c r="L9" s="35" t="n"/>
-      <c r="M9" s="35" t="n"/>
-      <c r="N9" s="35" t="n"/>
+      <c r="C9" s="40" t="n"/>
+      <c r="D9" s="40" t="n"/>
+      <c r="E9" s="40" t="n"/>
+      <c r="F9" s="40" t="n"/>
+      <c r="G9" s="40" t="n"/>
+      <c r="H9" s="40" t="n"/>
+      <c r="I9" s="40" t="n"/>
+      <c r="J9" s="40" t="n"/>
+      <c r="K9" s="40" t="n"/>
+      <c r="L9" s="40" t="n"/>
+      <c r="M9" s="40" t="n"/>
+      <c r="N9" s="41" t="n"/>
       <c r="P9" s="34" t="inlineStr">
         <is>
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="Q9" s="35" t="n"/>
-      <c r="R9" s="35" t="n"/>
-      <c r="S9" s="35" t="n"/>
-      <c r="T9" s="35" t="n"/>
-      <c r="U9" s="35" t="n"/>
-      <c r="V9" s="35" t="n"/>
-      <c r="W9" s="35" t="n"/>
-      <c r="X9" s="35" t="n"/>
-      <c r="Y9" s="35" t="n"/>
-      <c r="Z9" s="35" t="n"/>
-      <c r="AA9" s="35" t="n"/>
-      <c r="AB9" s="35" t="n"/>
+      <c r="Q9" s="40" t="n"/>
+      <c r="R9" s="40" t="n"/>
+      <c r="S9" s="40" t="n"/>
+      <c r="T9" s="40" t="n"/>
+      <c r="U9" s="40" t="n"/>
+      <c r="V9" s="40" t="n"/>
+      <c r="W9" s="40" t="n"/>
+      <c r="X9" s="40" t="n"/>
+      <c r="Y9" s="40" t="n"/>
+      <c r="Z9" s="40" t="n"/>
+      <c r="AA9" s="40" t="n"/>
+      <c r="AB9" s="41" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="B10" s="35" t="n"/>
-      <c r="C10" s="35" t="n"/>
-      <c r="D10" s="35" t="n"/>
-      <c r="E10" s="35" t="n"/>
-      <c r="F10" s="35" t="n"/>
-      <c r="G10" s="35" t="n"/>
-      <c r="H10" s="35" t="n"/>
-      <c r="I10" s="35" t="n"/>
-      <c r="J10" s="35" t="n"/>
-      <c r="K10" s="35" t="n"/>
-      <c r="L10" s="35" t="n"/>
-      <c r="M10" s="35" t="n"/>
-      <c r="N10" s="35" t="n"/>
-      <c r="P10" s="35" t="n"/>
-      <c r="Q10" s="35" t="n"/>
-      <c r="R10" s="35" t="n"/>
-      <c r="S10" s="35" t="n"/>
-      <c r="T10" s="35" t="n"/>
-      <c r="U10" s="35" t="n"/>
-      <c r="V10" s="35" t="n"/>
-      <c r="W10" s="35" t="n"/>
-      <c r="X10" s="35" t="n"/>
-      <c r="Y10" s="35" t="n"/>
-      <c r="Z10" s="35" t="n"/>
-      <c r="AA10" s="35" t="n"/>
-      <c r="AB10" s="35" t="n"/>
+      <c r="B10" s="42" t="n"/>
+      <c r="N10" s="43" t="n"/>
+      <c r="P10" s="42" t="n"/>
+      <c r="AB10" s="43" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="B11" s="35" t="n"/>
-      <c r="C11" s="35" t="n"/>
-      <c r="D11" s="35" t="n"/>
-      <c r="E11" s="35" t="n"/>
-      <c r="F11" s="35" t="n"/>
-      <c r="G11" s="35" t="n"/>
-      <c r="H11" s="35" t="n"/>
-      <c r="I11" s="35" t="n"/>
-      <c r="J11" s="35" t="n"/>
-      <c r="K11" s="35" t="n"/>
-      <c r="L11" s="35" t="n"/>
-      <c r="M11" s="35" t="n"/>
-      <c r="N11" s="35" t="n"/>
-      <c r="P11" s="35" t="n"/>
-      <c r="Q11" s="35" t="n"/>
-      <c r="R11" s="35" t="n"/>
-      <c r="S11" s="35" t="n"/>
-      <c r="T11" s="35" t="n"/>
-      <c r="U11" s="35" t="n"/>
-      <c r="V11" s="35" t="n"/>
-      <c r="W11" s="35" t="n"/>
-      <c r="X11" s="35" t="n"/>
-      <c r="Y11" s="35" t="n"/>
-      <c r="Z11" s="35" t="n"/>
-      <c r="AA11" s="35" t="n"/>
-      <c r="AB11" s="35" t="n"/>
+      <c r="B11" s="42" t="n"/>
+      <c r="N11" s="43" t="n"/>
+      <c r="P11" s="42" t="n"/>
+      <c r="AB11" s="43" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="B12" s="35" t="n"/>
-      <c r="C12" s="35" t="n"/>
-      <c r="D12" s="35" t="n"/>
-      <c r="E12" s="35" t="n"/>
-      <c r="F12" s="35" t="n"/>
-      <c r="G12" s="35" t="n"/>
-      <c r="H12" s="35" t="n"/>
-      <c r="I12" s="35" t="n"/>
-      <c r="J12" s="35" t="n"/>
-      <c r="K12" s="35" t="n"/>
-      <c r="L12" s="35" t="n"/>
-      <c r="M12" s="35" t="n"/>
-      <c r="N12" s="35" t="n"/>
-      <c r="P12" s="35" t="n"/>
-      <c r="Q12" s="35" t="n"/>
-      <c r="R12" s="35" t="n"/>
-      <c r="S12" s="35" t="n"/>
-      <c r="T12" s="35" t="n"/>
-      <c r="U12" s="35" t="n"/>
-      <c r="V12" s="35" t="n"/>
-      <c r="W12" s="35" t="n"/>
-      <c r="X12" s="35" t="n"/>
-      <c r="Y12" s="35" t="n"/>
-      <c r="Z12" s="35" t="n"/>
-      <c r="AA12" s="35" t="n"/>
-      <c r="AB12" s="35" t="n"/>
+      <c r="B12" s="42" t="n"/>
+      <c r="N12" s="43" t="n"/>
+      <c r="P12" s="42" t="n"/>
+      <c r="AB12" s="43" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="35" t="n"/>
-      <c r="C13" s="35" t="n"/>
-      <c r="D13" s="35" t="n"/>
-      <c r="E13" s="35" t="n"/>
-      <c r="F13" s="35" t="n"/>
-      <c r="G13" s="35" t="n"/>
-      <c r="H13" s="35" t="n"/>
-      <c r="I13" s="35" t="n"/>
-      <c r="J13" s="35" t="n"/>
-      <c r="K13" s="35" t="n"/>
-      <c r="L13" s="35" t="n"/>
-      <c r="M13" s="35" t="n"/>
-      <c r="N13" s="35" t="n"/>
-      <c r="P13" s="35" t="n"/>
-      <c r="Q13" s="35" t="n"/>
-      <c r="R13" s="35" t="n"/>
-      <c r="S13" s="35" t="n"/>
-      <c r="T13" s="35" t="n"/>
-      <c r="U13" s="35" t="n"/>
-      <c r="V13" s="35" t="n"/>
-      <c r="W13" s="35" t="n"/>
-      <c r="X13" s="35" t="n"/>
-      <c r="Y13" s="35" t="n"/>
-      <c r="Z13" s="35" t="n"/>
-      <c r="AA13" s="35" t="n"/>
-      <c r="AB13" s="35" t="n"/>
+      <c r="B13" s="42" t="n"/>
+      <c r="N13" s="43" t="n"/>
+      <c r="P13" s="42" t="n"/>
+      <c r="AB13" s="43" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="B14" s="35" t="n"/>
-      <c r="C14" s="35" t="n"/>
-      <c r="D14" s="35" t="n"/>
-      <c r="E14" s="35" t="n"/>
-      <c r="F14" s="35" t="n"/>
-      <c r="G14" s="35" t="n"/>
-      <c r="H14" s="35" t="n"/>
-      <c r="I14" s="35" t="n"/>
-      <c r="J14" s="35" t="n"/>
-      <c r="K14" s="35" t="n"/>
-      <c r="L14" s="35" t="n"/>
-      <c r="M14" s="35" t="n"/>
-      <c r="N14" s="35" t="n"/>
-      <c r="P14" s="35" t="n"/>
-      <c r="Q14" s="35" t="n"/>
-      <c r="R14" s="35" t="n"/>
-      <c r="S14" s="35" t="n"/>
-      <c r="T14" s="35" t="n"/>
-      <c r="U14" s="35" t="n"/>
-      <c r="V14" s="35" t="n"/>
-      <c r="W14" s="35" t="n"/>
-      <c r="X14" s="35" t="n"/>
-      <c r="Y14" s="35" t="n"/>
-      <c r="Z14" s="35" t="n"/>
-      <c r="AA14" s="35" t="n"/>
-      <c r="AB14" s="35" t="n"/>
+      <c r="B14" s="42" t="n"/>
+      <c r="N14" s="43" t="n"/>
+      <c r="P14" s="42" t="n"/>
+      <c r="AB14" s="43" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="B15" s="35" t="n"/>
-      <c r="C15" s="35" t="n"/>
-      <c r="D15" s="35" t="n"/>
-      <c r="E15" s="35" t="n"/>
-      <c r="F15" s="35" t="n"/>
-      <c r="G15" s="35" t="n"/>
-      <c r="H15" s="35" t="n"/>
-      <c r="I15" s="35" t="n"/>
-      <c r="J15" s="35" t="n"/>
-      <c r="K15" s="35" t="n"/>
-      <c r="L15" s="35" t="n"/>
-      <c r="M15" s="35" t="n"/>
-      <c r="N15" s="35" t="n"/>
-      <c r="P15" s="35" t="n"/>
-      <c r="Q15" s="35" t="n"/>
-      <c r="R15" s="35" t="n"/>
-      <c r="S15" s="35" t="n"/>
-      <c r="T15" s="35" t="n"/>
-      <c r="U15" s="35" t="n"/>
-      <c r="V15" s="35" t="n"/>
-      <c r="W15" s="35" t="n"/>
-      <c r="X15" s="35" t="n"/>
-      <c r="Y15" s="35" t="n"/>
-      <c r="Z15" s="35" t="n"/>
-      <c r="AA15" s="35" t="n"/>
-      <c r="AB15" s="35" t="n"/>
+      <c r="B15" s="42" t="n"/>
+      <c r="N15" s="43" t="n"/>
+      <c r="P15" s="42" t="n"/>
+      <c r="AB15" s="43" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="B16" s="35" t="n"/>
-      <c r="C16" s="35" t="n"/>
-      <c r="D16" s="35" t="n"/>
-      <c r="E16" s="35" t="n"/>
-      <c r="F16" s="35" t="n"/>
-      <c r="G16" s="35" t="n"/>
-      <c r="H16" s="35" t="n"/>
-      <c r="I16" s="35" t="n"/>
-      <c r="J16" s="35" t="n"/>
-      <c r="K16" s="35" t="n"/>
-      <c r="L16" s="35" t="n"/>
-      <c r="M16" s="35" t="n"/>
-      <c r="N16" s="35" t="n"/>
-      <c r="P16" s="35" t="n"/>
-      <c r="Q16" s="35" t="n"/>
-      <c r="R16" s="35" t="n"/>
-      <c r="S16" s="35" t="n"/>
-      <c r="T16" s="35" t="n"/>
-      <c r="U16" s="35" t="n"/>
-      <c r="V16" s="35" t="n"/>
-      <c r="W16" s="35" t="n"/>
-      <c r="X16" s="35" t="n"/>
-      <c r="Y16" s="35" t="n"/>
-      <c r="Z16" s="35" t="n"/>
-      <c r="AA16" s="35" t="n"/>
-      <c r="AB16" s="35" t="n"/>
+      <c r="B16" s="42" t="n"/>
+      <c r="N16" s="43" t="n"/>
+      <c r="P16" s="42" t="n"/>
+      <c r="AB16" s="43" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="B17" s="35" t="n"/>
-      <c r="C17" s="35" t="n"/>
-      <c r="D17" s="35" t="n"/>
-      <c r="E17" s="35" t="n"/>
-      <c r="F17" s="35" t="n"/>
-      <c r="G17" s="35" t="n"/>
-      <c r="H17" s="35" t="n"/>
-      <c r="I17" s="35" t="n"/>
-      <c r="J17" s="35" t="n"/>
-      <c r="K17" s="35" t="n"/>
-      <c r="L17" s="35" t="n"/>
-      <c r="M17" s="35" t="n"/>
-      <c r="N17" s="35" t="n"/>
-      <c r="P17" s="35" t="n"/>
-      <c r="Q17" s="35" t="n"/>
-      <c r="R17" s="35" t="n"/>
-      <c r="S17" s="35" t="n"/>
-      <c r="T17" s="35" t="n"/>
-      <c r="U17" s="35" t="n"/>
-      <c r="V17" s="35" t="n"/>
-      <c r="W17" s="35" t="n"/>
-      <c r="X17" s="35" t="n"/>
-      <c r="Y17" s="35" t="n"/>
-      <c r="Z17" s="35" t="n"/>
-      <c r="AA17" s="35" t="n"/>
-      <c r="AB17" s="35" t="n"/>
+      <c r="B17" s="42" t="n"/>
+      <c r="N17" s="43" t="n"/>
+      <c r="P17" s="42" t="n"/>
+      <c r="AB17" s="43" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="B18" s="35" t="n"/>
-      <c r="C18" s="35" t="n"/>
-      <c r="D18" s="35" t="n"/>
-      <c r="E18" s="35" t="n"/>
-      <c r="F18" s="35" t="n"/>
-      <c r="G18" s="35" t="n"/>
-      <c r="H18" s="35" t="n"/>
-      <c r="I18" s="35" t="n"/>
-      <c r="J18" s="35" t="n"/>
-      <c r="K18" s="35" t="n"/>
-      <c r="L18" s="35" t="n"/>
-      <c r="M18" s="35" t="n"/>
-      <c r="N18" s="35" t="n"/>
-      <c r="P18" s="35" t="n"/>
-      <c r="Q18" s="35" t="n"/>
-      <c r="R18" s="35" t="n"/>
-      <c r="S18" s="35" t="n"/>
-      <c r="T18" s="35" t="n"/>
-      <c r="U18" s="35" t="n"/>
-      <c r="V18" s="35" t="n"/>
-      <c r="W18" s="35" t="n"/>
-      <c r="X18" s="35" t="n"/>
-      <c r="Y18" s="35" t="n"/>
-      <c r="Z18" s="35" t="n"/>
-      <c r="AA18" s="35" t="n"/>
-      <c r="AB18" s="35" t="n"/>
+      <c r="B18" s="42" t="n"/>
+      <c r="N18" s="43" t="n"/>
+      <c r="P18" s="42" t="n"/>
+      <c r="AB18" s="43" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="B19" s="35" t="n"/>
-      <c r="C19" s="35" t="n"/>
-      <c r="D19" s="35" t="n"/>
-      <c r="E19" s="35" t="n"/>
-      <c r="F19" s="35" t="n"/>
-      <c r="G19" s="35" t="n"/>
-      <c r="H19" s="35" t="n"/>
-      <c r="I19" s="35" t="n"/>
-      <c r="J19" s="35" t="n"/>
-      <c r="K19" s="35" t="n"/>
-      <c r="L19" s="35" t="n"/>
-      <c r="M19" s="35" t="n"/>
-      <c r="N19" s="35" t="n"/>
-      <c r="P19" s="35" t="n"/>
-      <c r="Q19" s="35" t="n"/>
-      <c r="R19" s="35" t="n"/>
-      <c r="S19" s="35" t="n"/>
-      <c r="T19" s="35" t="n"/>
-      <c r="U19" s="35" t="n"/>
-      <c r="V19" s="35" t="n"/>
-      <c r="W19" s="35" t="n"/>
-      <c r="X19" s="35" t="n"/>
-      <c r="Y19" s="35" t="n"/>
-      <c r="Z19" s="35" t="n"/>
-      <c r="AA19" s="35" t="n"/>
-      <c r="AB19" s="35" t="n"/>
+      <c r="B19" s="44" t="n"/>
+      <c r="C19" s="45" t="n"/>
+      <c r="D19" s="45" t="n"/>
+      <c r="E19" s="45" t="n"/>
+      <c r="F19" s="45" t="n"/>
+      <c r="G19" s="45" t="n"/>
+      <c r="H19" s="45" t="n"/>
+      <c r="I19" s="45" t="n"/>
+      <c r="J19" s="45" t="n"/>
+      <c r="K19" s="45" t="n"/>
+      <c r="L19" s="45" t="n"/>
+      <c r="M19" s="45" t="n"/>
+      <c r="N19" s="46" t="n"/>
+      <c r="P19" s="44" t="n"/>
+      <c r="Q19" s="45" t="n"/>
+      <c r="R19" s="45" t="n"/>
+      <c r="S19" s="45" t="n"/>
+      <c r="T19" s="45" t="n"/>
+      <c r="U19" s="45" t="n"/>
+      <c r="V19" s="45" t="n"/>
+      <c r="W19" s="45" t="n"/>
+      <c r="X19" s="45" t="n"/>
+      <c r="Y19" s="45" t="n"/>
+      <c r="Z19" s="45" t="n"/>
+      <c r="AA19" s="45" t="n"/>
+      <c r="AB19" s="46" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="36" t="inlineStr">
@@ -3390,61 +3198,61 @@
           <t>조치내용</t>
         </is>
       </c>
-      <c r="C20" s="19" t="n"/>
+      <c r="C20" s="27" t="n"/>
       <c r="D20" s="51" t="inlineStr"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="n"/>
-      <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
-      <c r="O20" s="7" t="n"/>
-      <c r="P20" s="7" t="n"/>
-      <c r="Q20" s="7" t="n"/>
-      <c r="R20" s="7" t="n"/>
-      <c r="S20" s="7" t="n"/>
-      <c r="T20" s="7" t="n"/>
-      <c r="U20" s="7" t="n"/>
-      <c r="V20" s="7" t="n"/>
-      <c r="W20" s="7" t="n"/>
-      <c r="X20" s="7" t="n"/>
-      <c r="Y20" s="7" t="n"/>
-      <c r="Z20" s="7" t="n"/>
-      <c r="AA20" s="7" t="n"/>
-      <c r="AB20" s="7" t="n"/>
+      <c r="E20" s="26" t="n"/>
+      <c r="F20" s="26" t="n"/>
+      <c r="G20" s="26" t="n"/>
+      <c r="H20" s="26" t="n"/>
+      <c r="I20" s="26" t="n"/>
+      <c r="J20" s="26" t="n"/>
+      <c r="K20" s="26" t="n"/>
+      <c r="L20" s="26" t="n"/>
+      <c r="M20" s="26" t="n"/>
+      <c r="N20" s="26" t="n"/>
+      <c r="O20" s="26" t="n"/>
+      <c r="P20" s="26" t="n"/>
+      <c r="Q20" s="26" t="n"/>
+      <c r="R20" s="26" t="n"/>
+      <c r="S20" s="26" t="n"/>
+      <c r="T20" s="26" t="n"/>
+      <c r="U20" s="26" t="n"/>
+      <c r="V20" s="26" t="n"/>
+      <c r="W20" s="26" t="n"/>
+      <c r="X20" s="26" t="n"/>
+      <c r="Y20" s="26" t="n"/>
+      <c r="Z20" s="26" t="n"/>
+      <c r="AA20" s="26" t="n"/>
+      <c r="AB20" s="27" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
-      <c r="I21" s="7" t="n"/>
-      <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
-      <c r="P21" s="7" t="n"/>
-      <c r="Q21" s="7" t="n"/>
-      <c r="R21" s="7" t="n"/>
-      <c r="S21" s="7" t="n"/>
-      <c r="T21" s="7" t="n"/>
-      <c r="U21" s="7" t="n"/>
-      <c r="V21" s="7" t="n"/>
-      <c r="W21" s="7" t="n"/>
-      <c r="X21" s="7" t="n"/>
-      <c r="Y21" s="7" t="n"/>
-      <c r="Z21" s="7" t="n"/>
-      <c r="AA21" s="7" t="n"/>
-      <c r="AB21" s="7" t="n"/>
+      <c r="B21" s="30" t="n"/>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="30" t="n"/>
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="31" t="n"/>
+      <c r="G21" s="31" t="n"/>
+      <c r="H21" s="31" t="n"/>
+      <c r="I21" s="31" t="n"/>
+      <c r="J21" s="31" t="n"/>
+      <c r="K21" s="31" t="n"/>
+      <c r="L21" s="31" t="n"/>
+      <c r="M21" s="31" t="n"/>
+      <c r="N21" s="31" t="n"/>
+      <c r="O21" s="31" t="n"/>
+      <c r="P21" s="31" t="n"/>
+      <c r="Q21" s="31" t="n"/>
+      <c r="R21" s="31" t="n"/>
+      <c r="S21" s="31" t="n"/>
+      <c r="T21" s="31" t="n"/>
+      <c r="U21" s="31" t="n"/>
+      <c r="V21" s="31" t="n"/>
+      <c r="W21" s="31" t="n"/>
+      <c r="X21" s="31" t="n"/>
+      <c r="Y21" s="31" t="n"/>
+      <c r="Z21" s="31" t="n"/>
+      <c r="AA21" s="31" t="n"/>
+      <c r="AB21" s="32" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="36" t="inlineStr">
@@ -3452,36 +3260,36 @@
           <t>조치일자</t>
         </is>
       </c>
-      <c r="C22" s="19" t="n"/>
+      <c r="C22" s="23" t="n"/>
       <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
+      <c r="E22" s="22" t="n"/>
+      <c r="F22" s="22" t="n"/>
+      <c r="G22" s="22" t="n"/>
+      <c r="H22" s="22" t="n"/>
+      <c r="I22" s="23" t="n"/>
       <c r="J22" s="36" t="inlineStr">
         <is>
           <t>확인자</t>
         </is>
       </c>
-      <c r="K22" s="19" t="n"/>
-      <c r="L22" s="19" t="n"/>
+      <c r="K22" s="22" t="n"/>
+      <c r="L22" s="23" t="n"/>
       <c r="M22" s="12" t="inlineStr"/>
-      <c r="N22" s="7" t="n"/>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="7" t="n"/>
-      <c r="Q22" s="7" t="n"/>
-      <c r="R22" s="7" t="n"/>
-      <c r="S22" s="7" t="n"/>
-      <c r="T22" s="7" t="n"/>
-      <c r="U22" s="7" t="n"/>
-      <c r="V22" s="7" t="n"/>
-      <c r="W22" s="7" t="n"/>
-      <c r="X22" s="7" t="n"/>
-      <c r="Y22" s="7" t="n"/>
-      <c r="Z22" s="7" t="n"/>
-      <c r="AA22" s="7" t="n"/>
-      <c r="AB22" s="7" t="n"/>
+      <c r="N22" s="22" t="n"/>
+      <c r="O22" s="22" t="n"/>
+      <c r="P22" s="22" t="n"/>
+      <c r="Q22" s="22" t="n"/>
+      <c r="R22" s="22" t="n"/>
+      <c r="S22" s="22" t="n"/>
+      <c r="T22" s="22" t="n"/>
+      <c r="U22" s="22" t="n"/>
+      <c r="V22" s="22" t="n"/>
+      <c r="W22" s="22" t="n"/>
+      <c r="X22" s="22" t="n"/>
+      <c r="Y22" s="22" t="n"/>
+      <c r="Z22" s="22" t="n"/>
+      <c r="AA22" s="22" t="n"/>
+      <c r="AB22" s="23" t="n"/>
     </row>
     <row r="23" ht="14" customHeight="1"/>
     <row r="24" ht="20" customHeight="1">
@@ -3490,36 +3298,36 @@
           <t>No.2</t>
         </is>
       </c>
-      <c r="C24" s="10" t="n"/>
+      <c r="C24" s="23" t="n"/>
       <c r="D24" s="36" t="inlineStr">
         <is>
           <t>지적사항 내용</t>
         </is>
       </c>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="19" t="n"/>
-      <c r="G24" s="19" t="n"/>
-      <c r="H24" s="19" t="n"/>
+      <c r="E24" s="22" t="n"/>
+      <c r="F24" s="22" t="n"/>
+      <c r="G24" s="22" t="n"/>
+      <c r="H24" s="23" t="n"/>
       <c r="I24" s="48" t="inlineStr"/>
-      <c r="J24" s="7" t="n"/>
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
-      <c r="M24" s="7" t="n"/>
-      <c r="N24" s="7" t="n"/>
-      <c r="O24" s="7" t="n"/>
-      <c r="P24" s="7" t="n"/>
-      <c r="Q24" s="7" t="n"/>
-      <c r="R24" s="7" t="n"/>
-      <c r="S24" s="7" t="n"/>
-      <c r="T24" s="7" t="n"/>
-      <c r="U24" s="7" t="n"/>
-      <c r="V24" s="7" t="n"/>
-      <c r="W24" s="7" t="n"/>
-      <c r="X24" s="7" t="n"/>
-      <c r="Y24" s="7" t="n"/>
-      <c r="Z24" s="7" t="n"/>
-      <c r="AA24" s="7" t="n"/>
-      <c r="AB24" s="7" t="n"/>
+      <c r="J24" s="22" t="n"/>
+      <c r="K24" s="22" t="n"/>
+      <c r="L24" s="22" t="n"/>
+      <c r="M24" s="22" t="n"/>
+      <c r="N24" s="22" t="n"/>
+      <c r="O24" s="22" t="n"/>
+      <c r="P24" s="22" t="n"/>
+      <c r="Q24" s="22" t="n"/>
+      <c r="R24" s="22" t="n"/>
+      <c r="S24" s="22" t="n"/>
+      <c r="T24" s="22" t="n"/>
+      <c r="U24" s="22" t="n"/>
+      <c r="V24" s="22" t="n"/>
+      <c r="W24" s="22" t="n"/>
+      <c r="X24" s="22" t="n"/>
+      <c r="Y24" s="22" t="n"/>
+      <c r="Z24" s="22" t="n"/>
+      <c r="AA24" s="22" t="n"/>
+      <c r="AB24" s="23" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="49" t="inlineStr">
@@ -3539,315 +3347,117 @@
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="C26" s="35" t="n"/>
-      <c r="D26" s="35" t="n"/>
-      <c r="E26" s="35" t="n"/>
-      <c r="F26" s="35" t="n"/>
-      <c r="G26" s="35" t="n"/>
-      <c r="H26" s="35" t="n"/>
-      <c r="I26" s="35" t="n"/>
-      <c r="J26" s="35" t="n"/>
-      <c r="K26" s="35" t="n"/>
-      <c r="L26" s="35" t="n"/>
-      <c r="M26" s="35" t="n"/>
-      <c r="N26" s="35" t="n"/>
+      <c r="C26" s="40" t="n"/>
+      <c r="D26" s="40" t="n"/>
+      <c r="E26" s="40" t="n"/>
+      <c r="F26" s="40" t="n"/>
+      <c r="G26" s="40" t="n"/>
+      <c r="H26" s="40" t="n"/>
+      <c r="I26" s="40" t="n"/>
+      <c r="J26" s="40" t="n"/>
+      <c r="K26" s="40" t="n"/>
+      <c r="L26" s="40" t="n"/>
+      <c r="M26" s="40" t="n"/>
+      <c r="N26" s="41" t="n"/>
       <c r="P26" s="34" t="inlineStr">
         <is>
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="Q26" s="35" t="n"/>
-      <c r="R26" s="35" t="n"/>
-      <c r="S26" s="35" t="n"/>
-      <c r="T26" s="35" t="n"/>
-      <c r="U26" s="35" t="n"/>
-      <c r="V26" s="35" t="n"/>
-      <c r="W26" s="35" t="n"/>
-      <c r="X26" s="35" t="n"/>
-      <c r="Y26" s="35" t="n"/>
-      <c r="Z26" s="35" t="n"/>
-      <c r="AA26" s="35" t="n"/>
-      <c r="AB26" s="35" t="n"/>
+      <c r="Q26" s="40" t="n"/>
+      <c r="R26" s="40" t="n"/>
+      <c r="S26" s="40" t="n"/>
+      <c r="T26" s="40" t="n"/>
+      <c r="U26" s="40" t="n"/>
+      <c r="V26" s="40" t="n"/>
+      <c r="W26" s="40" t="n"/>
+      <c r="X26" s="40" t="n"/>
+      <c r="Y26" s="40" t="n"/>
+      <c r="Z26" s="40" t="n"/>
+      <c r="AA26" s="40" t="n"/>
+      <c r="AB26" s="41" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="B27" s="35" t="n"/>
-      <c r="C27" s="35" t="n"/>
-      <c r="D27" s="35" t="n"/>
-      <c r="E27" s="35" t="n"/>
-      <c r="F27" s="35" t="n"/>
-      <c r="G27" s="35" t="n"/>
-      <c r="H27" s="35" t="n"/>
-      <c r="I27" s="35" t="n"/>
-      <c r="J27" s="35" t="n"/>
-      <c r="K27" s="35" t="n"/>
-      <c r="L27" s="35" t="n"/>
-      <c r="M27" s="35" t="n"/>
-      <c r="N27" s="35" t="n"/>
-      <c r="P27" s="35" t="n"/>
-      <c r="Q27" s="35" t="n"/>
-      <c r="R27" s="35" t="n"/>
-      <c r="S27" s="35" t="n"/>
-      <c r="T27" s="35" t="n"/>
-      <c r="U27" s="35" t="n"/>
-      <c r="V27" s="35" t="n"/>
-      <c r="W27" s="35" t="n"/>
-      <c r="X27" s="35" t="n"/>
-      <c r="Y27" s="35" t="n"/>
-      <c r="Z27" s="35" t="n"/>
-      <c r="AA27" s="35" t="n"/>
-      <c r="AB27" s="35" t="n"/>
+      <c r="B27" s="42" t="n"/>
+      <c r="N27" s="43" t="n"/>
+      <c r="P27" s="42" t="n"/>
+      <c r="AB27" s="43" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="35" t="n"/>
-      <c r="C28" s="35" t="n"/>
-      <c r="D28" s="35" t="n"/>
-      <c r="E28" s="35" t="n"/>
-      <c r="F28" s="35" t="n"/>
-      <c r="G28" s="35" t="n"/>
-      <c r="H28" s="35" t="n"/>
-      <c r="I28" s="35" t="n"/>
-      <c r="J28" s="35" t="n"/>
-      <c r="K28" s="35" t="n"/>
-      <c r="L28" s="35" t="n"/>
-      <c r="M28" s="35" t="n"/>
-      <c r="N28" s="35" t="n"/>
-      <c r="P28" s="35" t="n"/>
-      <c r="Q28" s="35" t="n"/>
-      <c r="R28" s="35" t="n"/>
-      <c r="S28" s="35" t="n"/>
-      <c r="T28" s="35" t="n"/>
-      <c r="U28" s="35" t="n"/>
-      <c r="V28" s="35" t="n"/>
-      <c r="W28" s="35" t="n"/>
-      <c r="X28" s="35" t="n"/>
-      <c r="Y28" s="35" t="n"/>
-      <c r="Z28" s="35" t="n"/>
-      <c r="AA28" s="35" t="n"/>
-      <c r="AB28" s="35" t="n"/>
+      <c r="B28" s="42" t="n"/>
+      <c r="N28" s="43" t="n"/>
+      <c r="P28" s="42" t="n"/>
+      <c r="AB28" s="43" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="B29" s="35" t="n"/>
-      <c r="C29" s="35" t="n"/>
-      <c r="D29" s="35" t="n"/>
-      <c r="E29" s="35" t="n"/>
-      <c r="F29" s="35" t="n"/>
-      <c r="G29" s="35" t="n"/>
-      <c r="H29" s="35" t="n"/>
-      <c r="I29" s="35" t="n"/>
-      <c r="J29" s="35" t="n"/>
-      <c r="K29" s="35" t="n"/>
-      <c r="L29" s="35" t="n"/>
-      <c r="M29" s="35" t="n"/>
-      <c r="N29" s="35" t="n"/>
-      <c r="P29" s="35" t="n"/>
-      <c r="Q29" s="35" t="n"/>
-      <c r="R29" s="35" t="n"/>
-      <c r="S29" s="35" t="n"/>
-      <c r="T29" s="35" t="n"/>
-      <c r="U29" s="35" t="n"/>
-      <c r="V29" s="35" t="n"/>
-      <c r="W29" s="35" t="n"/>
-      <c r="X29" s="35" t="n"/>
-      <c r="Y29" s="35" t="n"/>
-      <c r="Z29" s="35" t="n"/>
-      <c r="AA29" s="35" t="n"/>
-      <c r="AB29" s="35" t="n"/>
+      <c r="B29" s="42" t="n"/>
+      <c r="N29" s="43" t="n"/>
+      <c r="P29" s="42" t="n"/>
+      <c r="AB29" s="43" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="B30" s="35" t="n"/>
-      <c r="C30" s="35" t="n"/>
-      <c r="D30" s="35" t="n"/>
-      <c r="E30" s="35" t="n"/>
-      <c r="F30" s="35" t="n"/>
-      <c r="G30" s="35" t="n"/>
-      <c r="H30" s="35" t="n"/>
-      <c r="I30" s="35" t="n"/>
-      <c r="J30" s="35" t="n"/>
-      <c r="K30" s="35" t="n"/>
-      <c r="L30" s="35" t="n"/>
-      <c r="M30" s="35" t="n"/>
-      <c r="N30" s="35" t="n"/>
-      <c r="P30" s="35" t="n"/>
-      <c r="Q30" s="35" t="n"/>
-      <c r="R30" s="35" t="n"/>
-      <c r="S30" s="35" t="n"/>
-      <c r="T30" s="35" t="n"/>
-      <c r="U30" s="35" t="n"/>
-      <c r="V30" s="35" t="n"/>
-      <c r="W30" s="35" t="n"/>
-      <c r="X30" s="35" t="n"/>
-      <c r="Y30" s="35" t="n"/>
-      <c r="Z30" s="35" t="n"/>
-      <c r="AA30" s="35" t="n"/>
-      <c r="AB30" s="35" t="n"/>
+      <c r="B30" s="42" t="n"/>
+      <c r="N30" s="43" t="n"/>
+      <c r="P30" s="42" t="n"/>
+      <c r="AB30" s="43" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="B31" s="35" t="n"/>
-      <c r="C31" s="35" t="n"/>
-      <c r="D31" s="35" t="n"/>
-      <c r="E31" s="35" t="n"/>
-      <c r="F31" s="35" t="n"/>
-      <c r="G31" s="35" t="n"/>
-      <c r="H31" s="35" t="n"/>
-      <c r="I31" s="35" t="n"/>
-      <c r="J31" s="35" t="n"/>
-      <c r="K31" s="35" t="n"/>
-      <c r="L31" s="35" t="n"/>
-      <c r="M31" s="35" t="n"/>
-      <c r="N31" s="35" t="n"/>
-      <c r="P31" s="35" t="n"/>
-      <c r="Q31" s="35" t="n"/>
-      <c r="R31" s="35" t="n"/>
-      <c r="S31" s="35" t="n"/>
-      <c r="T31" s="35" t="n"/>
-      <c r="U31" s="35" t="n"/>
-      <c r="V31" s="35" t="n"/>
-      <c r="W31" s="35" t="n"/>
-      <c r="X31" s="35" t="n"/>
-      <c r="Y31" s="35" t="n"/>
-      <c r="Z31" s="35" t="n"/>
-      <c r="AA31" s="35" t="n"/>
-      <c r="AB31" s="35" t="n"/>
+      <c r="B31" s="42" t="n"/>
+      <c r="N31" s="43" t="n"/>
+      <c r="P31" s="42" t="n"/>
+      <c r="AB31" s="43" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="35" t="n"/>
-      <c r="C32" s="35" t="n"/>
-      <c r="D32" s="35" t="n"/>
-      <c r="E32" s="35" t="n"/>
-      <c r="F32" s="35" t="n"/>
-      <c r="G32" s="35" t="n"/>
-      <c r="H32" s="35" t="n"/>
-      <c r="I32" s="35" t="n"/>
-      <c r="J32" s="35" t="n"/>
-      <c r="K32" s="35" t="n"/>
-      <c r="L32" s="35" t="n"/>
-      <c r="M32" s="35" t="n"/>
-      <c r="N32" s="35" t="n"/>
-      <c r="P32" s="35" t="n"/>
-      <c r="Q32" s="35" t="n"/>
-      <c r="R32" s="35" t="n"/>
-      <c r="S32" s="35" t="n"/>
-      <c r="T32" s="35" t="n"/>
-      <c r="U32" s="35" t="n"/>
-      <c r="V32" s="35" t="n"/>
-      <c r="W32" s="35" t="n"/>
-      <c r="X32" s="35" t="n"/>
-      <c r="Y32" s="35" t="n"/>
-      <c r="Z32" s="35" t="n"/>
-      <c r="AA32" s="35" t="n"/>
-      <c r="AB32" s="35" t="n"/>
+      <c r="B32" s="42" t="n"/>
+      <c r="N32" s="43" t="n"/>
+      <c r="P32" s="42" t="n"/>
+      <c r="AB32" s="43" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="B33" s="35" t="n"/>
-      <c r="C33" s="35" t="n"/>
-      <c r="D33" s="35" t="n"/>
-      <c r="E33" s="35" t="n"/>
-      <c r="F33" s="35" t="n"/>
-      <c r="G33" s="35" t="n"/>
-      <c r="H33" s="35" t="n"/>
-      <c r="I33" s="35" t="n"/>
-      <c r="J33" s="35" t="n"/>
-      <c r="K33" s="35" t="n"/>
-      <c r="L33" s="35" t="n"/>
-      <c r="M33" s="35" t="n"/>
-      <c r="N33" s="35" t="n"/>
-      <c r="P33" s="35" t="n"/>
-      <c r="Q33" s="35" t="n"/>
-      <c r="R33" s="35" t="n"/>
-      <c r="S33" s="35" t="n"/>
-      <c r="T33" s="35" t="n"/>
-      <c r="U33" s="35" t="n"/>
-      <c r="V33" s="35" t="n"/>
-      <c r="W33" s="35" t="n"/>
-      <c r="X33" s="35" t="n"/>
-      <c r="Y33" s="35" t="n"/>
-      <c r="Z33" s="35" t="n"/>
-      <c r="AA33" s="35" t="n"/>
-      <c r="AB33" s="35" t="n"/>
+      <c r="B33" s="42" t="n"/>
+      <c r="N33" s="43" t="n"/>
+      <c r="P33" s="42" t="n"/>
+      <c r="AB33" s="43" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="B34" s="35" t="n"/>
-      <c r="C34" s="35" t="n"/>
-      <c r="D34" s="35" t="n"/>
-      <c r="E34" s="35" t="n"/>
-      <c r="F34" s="35" t="n"/>
-      <c r="G34" s="35" t="n"/>
-      <c r="H34" s="35" t="n"/>
-      <c r="I34" s="35" t="n"/>
-      <c r="J34" s="35" t="n"/>
-      <c r="K34" s="35" t="n"/>
-      <c r="L34" s="35" t="n"/>
-      <c r="M34" s="35" t="n"/>
-      <c r="N34" s="35" t="n"/>
-      <c r="P34" s="35" t="n"/>
-      <c r="Q34" s="35" t="n"/>
-      <c r="R34" s="35" t="n"/>
-      <c r="S34" s="35" t="n"/>
-      <c r="T34" s="35" t="n"/>
-      <c r="U34" s="35" t="n"/>
-      <c r="V34" s="35" t="n"/>
-      <c r="W34" s="35" t="n"/>
-      <c r="X34" s="35" t="n"/>
-      <c r="Y34" s="35" t="n"/>
-      <c r="Z34" s="35" t="n"/>
-      <c r="AA34" s="35" t="n"/>
-      <c r="AB34" s="35" t="n"/>
+      <c r="B34" s="42" t="n"/>
+      <c r="N34" s="43" t="n"/>
+      <c r="P34" s="42" t="n"/>
+      <c r="AB34" s="43" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="B35" s="35" t="n"/>
-      <c r="C35" s="35" t="n"/>
-      <c r="D35" s="35" t="n"/>
-      <c r="E35" s="35" t="n"/>
-      <c r="F35" s="35" t="n"/>
-      <c r="G35" s="35" t="n"/>
-      <c r="H35" s="35" t="n"/>
-      <c r="I35" s="35" t="n"/>
-      <c r="J35" s="35" t="n"/>
-      <c r="K35" s="35" t="n"/>
-      <c r="L35" s="35" t="n"/>
-      <c r="M35" s="35" t="n"/>
-      <c r="N35" s="35" t="n"/>
-      <c r="P35" s="35" t="n"/>
-      <c r="Q35" s="35" t="n"/>
-      <c r="R35" s="35" t="n"/>
-      <c r="S35" s="35" t="n"/>
-      <c r="T35" s="35" t="n"/>
-      <c r="U35" s="35" t="n"/>
-      <c r="V35" s="35" t="n"/>
-      <c r="W35" s="35" t="n"/>
-      <c r="X35" s="35" t="n"/>
-      <c r="Y35" s="35" t="n"/>
-      <c r="Z35" s="35" t="n"/>
-      <c r="AA35" s="35" t="n"/>
-      <c r="AB35" s="35" t="n"/>
+      <c r="B35" s="42" t="n"/>
+      <c r="N35" s="43" t="n"/>
+      <c r="P35" s="42" t="n"/>
+      <c r="AB35" s="43" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="B36" s="35" t="n"/>
-      <c r="C36" s="35" t="n"/>
-      <c r="D36" s="35" t="n"/>
-      <c r="E36" s="35" t="n"/>
-      <c r="F36" s="35" t="n"/>
-      <c r="G36" s="35" t="n"/>
-      <c r="H36" s="35" t="n"/>
-      <c r="I36" s="35" t="n"/>
-      <c r="J36" s="35" t="n"/>
-      <c r="K36" s="35" t="n"/>
-      <c r="L36" s="35" t="n"/>
-      <c r="M36" s="35" t="n"/>
-      <c r="N36" s="35" t="n"/>
-      <c r="P36" s="35" t="n"/>
-      <c r="Q36" s="35" t="n"/>
-      <c r="R36" s="35" t="n"/>
-      <c r="S36" s="35" t="n"/>
-      <c r="T36" s="35" t="n"/>
-      <c r="U36" s="35" t="n"/>
-      <c r="V36" s="35" t="n"/>
-      <c r="W36" s="35" t="n"/>
-      <c r="X36" s="35" t="n"/>
-      <c r="Y36" s="35" t="n"/>
-      <c r="Z36" s="35" t="n"/>
-      <c r="AA36" s="35" t="n"/>
-      <c r="AB36" s="35" t="n"/>
+      <c r="B36" s="44" t="n"/>
+      <c r="C36" s="45" t="n"/>
+      <c r="D36" s="45" t="n"/>
+      <c r="E36" s="45" t="n"/>
+      <c r="F36" s="45" t="n"/>
+      <c r="G36" s="45" t="n"/>
+      <c r="H36" s="45" t="n"/>
+      <c r="I36" s="45" t="n"/>
+      <c r="J36" s="45" t="n"/>
+      <c r="K36" s="45" t="n"/>
+      <c r="L36" s="45" t="n"/>
+      <c r="M36" s="45" t="n"/>
+      <c r="N36" s="46" t="n"/>
+      <c r="P36" s="44" t="n"/>
+      <c r="Q36" s="45" t="n"/>
+      <c r="R36" s="45" t="n"/>
+      <c r="S36" s="45" t="n"/>
+      <c r="T36" s="45" t="n"/>
+      <c r="U36" s="45" t="n"/>
+      <c r="V36" s="45" t="n"/>
+      <c r="W36" s="45" t="n"/>
+      <c r="X36" s="45" t="n"/>
+      <c r="Y36" s="45" t="n"/>
+      <c r="Z36" s="45" t="n"/>
+      <c r="AA36" s="45" t="n"/>
+      <c r="AB36" s="46" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="36" t="inlineStr">
@@ -3855,61 +3465,61 @@
           <t>조치내용</t>
         </is>
       </c>
-      <c r="C37" s="19" t="n"/>
+      <c r="C37" s="27" t="n"/>
       <c r="D37" s="51" t="inlineStr"/>
-      <c r="E37" s="7" t="n"/>
-      <c r="F37" s="7" t="n"/>
-      <c r="G37" s="7" t="n"/>
-      <c r="H37" s="7" t="n"/>
-      <c r="I37" s="7" t="n"/>
-      <c r="J37" s="7" t="n"/>
-      <c r="K37" s="7" t="n"/>
-      <c r="L37" s="7" t="n"/>
-      <c r="M37" s="7" t="n"/>
-      <c r="N37" s="7" t="n"/>
-      <c r="O37" s="7" t="n"/>
-      <c r="P37" s="7" t="n"/>
-      <c r="Q37" s="7" t="n"/>
-      <c r="R37" s="7" t="n"/>
-      <c r="S37" s="7" t="n"/>
-      <c r="T37" s="7" t="n"/>
-      <c r="U37" s="7" t="n"/>
-      <c r="V37" s="7" t="n"/>
-      <c r="W37" s="7" t="n"/>
-      <c r="X37" s="7" t="n"/>
-      <c r="Y37" s="7" t="n"/>
-      <c r="Z37" s="7" t="n"/>
-      <c r="AA37" s="7" t="n"/>
-      <c r="AB37" s="7" t="n"/>
+      <c r="E37" s="26" t="n"/>
+      <c r="F37" s="26" t="n"/>
+      <c r="G37" s="26" t="n"/>
+      <c r="H37" s="26" t="n"/>
+      <c r="I37" s="26" t="n"/>
+      <c r="J37" s="26" t="n"/>
+      <c r="K37" s="26" t="n"/>
+      <c r="L37" s="26" t="n"/>
+      <c r="M37" s="26" t="n"/>
+      <c r="N37" s="26" t="n"/>
+      <c r="O37" s="26" t="n"/>
+      <c r="P37" s="26" t="n"/>
+      <c r="Q37" s="26" t="n"/>
+      <c r="R37" s="26" t="n"/>
+      <c r="S37" s="26" t="n"/>
+      <c r="T37" s="26" t="n"/>
+      <c r="U37" s="26" t="n"/>
+      <c r="V37" s="26" t="n"/>
+      <c r="W37" s="26" t="n"/>
+      <c r="X37" s="26" t="n"/>
+      <c r="Y37" s="26" t="n"/>
+      <c r="Z37" s="26" t="n"/>
+      <c r="AA37" s="26" t="n"/>
+      <c r="AB37" s="27" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="B38" s="19" t="n"/>
-      <c r="C38" s="19" t="n"/>
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
-      <c r="F38" s="7" t="n"/>
-      <c r="G38" s="7" t="n"/>
-      <c r="H38" s="7" t="n"/>
-      <c r="I38" s="7" t="n"/>
-      <c r="J38" s="7" t="n"/>
-      <c r="K38" s="7" t="n"/>
-      <c r="L38" s="7" t="n"/>
-      <c r="M38" s="7" t="n"/>
-      <c r="N38" s="7" t="n"/>
-      <c r="O38" s="7" t="n"/>
-      <c r="P38" s="7" t="n"/>
-      <c r="Q38" s="7" t="n"/>
-      <c r="R38" s="7" t="n"/>
-      <c r="S38" s="7" t="n"/>
-      <c r="T38" s="7" t="n"/>
-      <c r="U38" s="7" t="n"/>
-      <c r="V38" s="7" t="n"/>
-      <c r="W38" s="7" t="n"/>
-      <c r="X38" s="7" t="n"/>
-      <c r="Y38" s="7" t="n"/>
-      <c r="Z38" s="7" t="n"/>
-      <c r="AA38" s="7" t="n"/>
-      <c r="AB38" s="7" t="n"/>
+      <c r="B38" s="30" t="n"/>
+      <c r="C38" s="32" t="n"/>
+      <c r="D38" s="30" t="n"/>
+      <c r="E38" s="31" t="n"/>
+      <c r="F38" s="31" t="n"/>
+      <c r="G38" s="31" t="n"/>
+      <c r="H38" s="31" t="n"/>
+      <c r="I38" s="31" t="n"/>
+      <c r="J38" s="31" t="n"/>
+      <c r="K38" s="31" t="n"/>
+      <c r="L38" s="31" t="n"/>
+      <c r="M38" s="31" t="n"/>
+      <c r="N38" s="31" t="n"/>
+      <c r="O38" s="31" t="n"/>
+      <c r="P38" s="31" t="n"/>
+      <c r="Q38" s="31" t="n"/>
+      <c r="R38" s="31" t="n"/>
+      <c r="S38" s="31" t="n"/>
+      <c r="T38" s="31" t="n"/>
+      <c r="U38" s="31" t="n"/>
+      <c r="V38" s="31" t="n"/>
+      <c r="W38" s="31" t="n"/>
+      <c r="X38" s="31" t="n"/>
+      <c r="Y38" s="31" t="n"/>
+      <c r="Z38" s="31" t="n"/>
+      <c r="AA38" s="31" t="n"/>
+      <c r="AB38" s="32" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="36" t="inlineStr">
@@ -3917,36 +3527,36 @@
           <t>조치일자</t>
         </is>
       </c>
-      <c r="C39" s="19" t="n"/>
+      <c r="C39" s="23" t="n"/>
       <c r="D39" s="12" t="inlineStr"/>
-      <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="n"/>
-      <c r="G39" s="7" t="n"/>
-      <c r="H39" s="7" t="n"/>
-      <c r="I39" s="7" t="n"/>
+      <c r="E39" s="22" t="n"/>
+      <c r="F39" s="22" t="n"/>
+      <c r="G39" s="22" t="n"/>
+      <c r="H39" s="22" t="n"/>
+      <c r="I39" s="23" t="n"/>
       <c r="J39" s="36" t="inlineStr">
         <is>
           <t>확인자</t>
         </is>
       </c>
-      <c r="K39" s="19" t="n"/>
-      <c r="L39" s="19" t="n"/>
+      <c r="K39" s="22" t="n"/>
+      <c r="L39" s="23" t="n"/>
       <c r="M39" s="12" t="inlineStr"/>
-      <c r="N39" s="7" t="n"/>
-      <c r="O39" s="7" t="n"/>
-      <c r="P39" s="7" t="n"/>
-      <c r="Q39" s="7" t="n"/>
-      <c r="R39" s="7" t="n"/>
-      <c r="S39" s="7" t="n"/>
-      <c r="T39" s="7" t="n"/>
-      <c r="U39" s="7" t="n"/>
-      <c r="V39" s="7" t="n"/>
-      <c r="W39" s="7" t="n"/>
-      <c r="X39" s="7" t="n"/>
-      <c r="Y39" s="7" t="n"/>
-      <c r="Z39" s="7" t="n"/>
-      <c r="AA39" s="7" t="n"/>
-      <c r="AB39" s="7" t="n"/>
+      <c r="N39" s="22" t="n"/>
+      <c r="O39" s="22" t="n"/>
+      <c r="P39" s="22" t="n"/>
+      <c r="Q39" s="22" t="n"/>
+      <c r="R39" s="22" t="n"/>
+      <c r="S39" s="22" t="n"/>
+      <c r="T39" s="22" t="n"/>
+      <c r="U39" s="22" t="n"/>
+      <c r="V39" s="22" t="n"/>
+      <c r="W39" s="22" t="n"/>
+      <c r="X39" s="22" t="n"/>
+      <c r="Y39" s="22" t="n"/>
+      <c r="Z39" s="22" t="n"/>
+      <c r="AA39" s="22" t="n"/>
+      <c r="AB39" s="23" t="n"/>
     </row>
     <row r="40" ht="14" customHeight="1"/>
     <row r="41" ht="20" customHeight="1">
@@ -3955,36 +3565,36 @@
           <t>No.3</t>
         </is>
       </c>
-      <c r="C41" s="10" t="n"/>
+      <c r="C41" s="23" t="n"/>
       <c r="D41" s="36" t="inlineStr">
         <is>
           <t>지적사항 내용</t>
         </is>
       </c>
-      <c r="E41" s="19" t="n"/>
-      <c r="F41" s="19" t="n"/>
-      <c r="G41" s="19" t="n"/>
-      <c r="H41" s="19" t="n"/>
+      <c r="E41" s="22" t="n"/>
+      <c r="F41" s="22" t="n"/>
+      <c r="G41" s="22" t="n"/>
+      <c r="H41" s="23" t="n"/>
       <c r="I41" s="48" t="inlineStr"/>
-      <c r="J41" s="7" t="n"/>
-      <c r="K41" s="7" t="n"/>
-      <c r="L41" s="7" t="n"/>
-      <c r="M41" s="7" t="n"/>
-      <c r="N41" s="7" t="n"/>
-      <c r="O41" s="7" t="n"/>
-      <c r="P41" s="7" t="n"/>
-      <c r="Q41" s="7" t="n"/>
-      <c r="R41" s="7" t="n"/>
-      <c r="S41" s="7" t="n"/>
-      <c r="T41" s="7" t="n"/>
-      <c r="U41" s="7" t="n"/>
-      <c r="V41" s="7" t="n"/>
-      <c r="W41" s="7" t="n"/>
-      <c r="X41" s="7" t="n"/>
-      <c r="Y41" s="7" t="n"/>
-      <c r="Z41" s="7" t="n"/>
-      <c r="AA41" s="7" t="n"/>
-      <c r="AB41" s="7" t="n"/>
+      <c r="J41" s="22" t="n"/>
+      <c r="K41" s="22" t="n"/>
+      <c r="L41" s="22" t="n"/>
+      <c r="M41" s="22" t="n"/>
+      <c r="N41" s="22" t="n"/>
+      <c r="O41" s="22" t="n"/>
+      <c r="P41" s="22" t="n"/>
+      <c r="Q41" s="22" t="n"/>
+      <c r="R41" s="22" t="n"/>
+      <c r="S41" s="22" t="n"/>
+      <c r="T41" s="22" t="n"/>
+      <c r="U41" s="22" t="n"/>
+      <c r="V41" s="22" t="n"/>
+      <c r="W41" s="22" t="n"/>
+      <c r="X41" s="22" t="n"/>
+      <c r="Y41" s="22" t="n"/>
+      <c r="Z41" s="22" t="n"/>
+      <c r="AA41" s="22" t="n"/>
+      <c r="AB41" s="23" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="49" t="inlineStr">
@@ -4004,315 +3614,117 @@
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="C43" s="35" t="n"/>
-      <c r="D43" s="35" t="n"/>
-      <c r="E43" s="35" t="n"/>
-      <c r="F43" s="35" t="n"/>
-      <c r="G43" s="35" t="n"/>
-      <c r="H43" s="35" t="n"/>
-      <c r="I43" s="35" t="n"/>
-      <c r="J43" s="35" t="n"/>
-      <c r="K43" s="35" t="n"/>
-      <c r="L43" s="35" t="n"/>
-      <c r="M43" s="35" t="n"/>
-      <c r="N43" s="35" t="n"/>
+      <c r="C43" s="40" t="n"/>
+      <c r="D43" s="40" t="n"/>
+      <c r="E43" s="40" t="n"/>
+      <c r="F43" s="40" t="n"/>
+      <c r="G43" s="40" t="n"/>
+      <c r="H43" s="40" t="n"/>
+      <c r="I43" s="40" t="n"/>
+      <c r="J43" s="40" t="n"/>
+      <c r="K43" s="40" t="n"/>
+      <c r="L43" s="40" t="n"/>
+      <c r="M43" s="40" t="n"/>
+      <c r="N43" s="41" t="n"/>
       <c r="P43" s="34" t="inlineStr">
         <is>
           <t>사진 삽입 영역</t>
         </is>
       </c>
-      <c r="Q43" s="35" t="n"/>
-      <c r="R43" s="35" t="n"/>
-      <c r="S43" s="35" t="n"/>
-      <c r="T43" s="35" t="n"/>
-      <c r="U43" s="35" t="n"/>
-      <c r="V43" s="35" t="n"/>
-      <c r="W43" s="35" t="n"/>
-      <c r="X43" s="35" t="n"/>
-      <c r="Y43" s="35" t="n"/>
-      <c r="Z43" s="35" t="n"/>
-      <c r="AA43" s="35" t="n"/>
-      <c r="AB43" s="35" t="n"/>
+      <c r="Q43" s="40" t="n"/>
+      <c r="R43" s="40" t="n"/>
+      <c r="S43" s="40" t="n"/>
+      <c r="T43" s="40" t="n"/>
+      <c r="U43" s="40" t="n"/>
+      <c r="V43" s="40" t="n"/>
+      <c r="W43" s="40" t="n"/>
+      <c r="X43" s="40" t="n"/>
+      <c r="Y43" s="40" t="n"/>
+      <c r="Z43" s="40" t="n"/>
+      <c r="AA43" s="40" t="n"/>
+      <c r="AB43" s="41" t="n"/>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="B44" s="35" t="n"/>
-      <c r="C44" s="35" t="n"/>
-      <c r="D44" s="35" t="n"/>
-      <c r="E44" s="35" t="n"/>
-      <c r="F44" s="35" t="n"/>
-      <c r="G44" s="35" t="n"/>
-      <c r="H44" s="35" t="n"/>
-      <c r="I44" s="35" t="n"/>
-      <c r="J44" s="35" t="n"/>
-      <c r="K44" s="35" t="n"/>
-      <c r="L44" s="35" t="n"/>
-      <c r="M44" s="35" t="n"/>
-      <c r="N44" s="35" t="n"/>
-      <c r="P44" s="35" t="n"/>
-      <c r="Q44" s="35" t="n"/>
-      <c r="R44" s="35" t="n"/>
-      <c r="S44" s="35" t="n"/>
-      <c r="T44" s="35" t="n"/>
-      <c r="U44" s="35" t="n"/>
-      <c r="V44" s="35" t="n"/>
-      <c r="W44" s="35" t="n"/>
-      <c r="X44" s="35" t="n"/>
-      <c r="Y44" s="35" t="n"/>
-      <c r="Z44" s="35" t="n"/>
-      <c r="AA44" s="35" t="n"/>
-      <c r="AB44" s="35" t="n"/>
+      <c r="B44" s="42" t="n"/>
+      <c r="N44" s="43" t="n"/>
+      <c r="P44" s="42" t="n"/>
+      <c r="AB44" s="43" t="n"/>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="B45" s="35" t="n"/>
-      <c r="C45" s="35" t="n"/>
-      <c r="D45" s="35" t="n"/>
-      <c r="E45" s="35" t="n"/>
-      <c r="F45" s="35" t="n"/>
-      <c r="G45" s="35" t="n"/>
-      <c r="H45" s="35" t="n"/>
-      <c r="I45" s="35" t="n"/>
-      <c r="J45" s="35" t="n"/>
-      <c r="K45" s="35" t="n"/>
-      <c r="L45" s="35" t="n"/>
-      <c r="M45" s="35" t="n"/>
-      <c r="N45" s="35" t="n"/>
-      <c r="P45" s="35" t="n"/>
-      <c r="Q45" s="35" t="n"/>
-      <c r="R45" s="35" t="n"/>
-      <c r="S45" s="35" t="n"/>
-      <c r="T45" s="35" t="n"/>
-      <c r="U45" s="35" t="n"/>
-      <c r="V45" s="35" t="n"/>
-      <c r="W45" s="35" t="n"/>
-      <c r="X45" s="35" t="n"/>
-      <c r="Y45" s="35" t="n"/>
-      <c r="Z45" s="35" t="n"/>
-      <c r="AA45" s="35" t="n"/>
-      <c r="AB45" s="35" t="n"/>
+      <c r="B45" s="42" t="n"/>
+      <c r="N45" s="43" t="n"/>
+      <c r="P45" s="42" t="n"/>
+      <c r="AB45" s="43" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="B46" s="35" t="n"/>
-      <c r="C46" s="35" t="n"/>
-      <c r="D46" s="35" t="n"/>
-      <c r="E46" s="35" t="n"/>
-      <c r="F46" s="35" t="n"/>
-      <c r="G46" s="35" t="n"/>
-      <c r="H46" s="35" t="n"/>
-      <c r="I46" s="35" t="n"/>
-      <c r="J46" s="35" t="n"/>
-      <c r="K46" s="35" t="n"/>
-      <c r="L46" s="35" t="n"/>
-      <c r="M46" s="35" t="n"/>
-      <c r="N46" s="35" t="n"/>
-      <c r="P46" s="35" t="n"/>
-      <c r="Q46" s="35" t="n"/>
-      <c r="R46" s="35" t="n"/>
-      <c r="S46" s="35" t="n"/>
-      <c r="T46" s="35" t="n"/>
-      <c r="U46" s="35" t="n"/>
-      <c r="V46" s="35" t="n"/>
-      <c r="W46" s="35" t="n"/>
-      <c r="X46" s="35" t="n"/>
-      <c r="Y46" s="35" t="n"/>
-      <c r="Z46" s="35" t="n"/>
-      <c r="AA46" s="35" t="n"/>
-      <c r="AB46" s="35" t="n"/>
+      <c r="B46" s="42" t="n"/>
+      <c r="N46" s="43" t="n"/>
+      <c r="P46" s="42" t="n"/>
+      <c r="AB46" s="43" t="n"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="B47" s="35" t="n"/>
-      <c r="C47" s="35" t="n"/>
-      <c r="D47" s="35" t="n"/>
-      <c r="E47" s="35" t="n"/>
-      <c r="F47" s="35" t="n"/>
-      <c r="G47" s="35" t="n"/>
-      <c r="H47" s="35" t="n"/>
-      <c r="I47" s="35" t="n"/>
-      <c r="J47" s="35" t="n"/>
-      <c r="K47" s="35" t="n"/>
-      <c r="L47" s="35" t="n"/>
-      <c r="M47" s="35" t="n"/>
-      <c r="N47" s="35" t="n"/>
-      <c r="P47" s="35" t="n"/>
-      <c r="Q47" s="35" t="n"/>
-      <c r="R47" s="35" t="n"/>
-      <c r="S47" s="35" t="n"/>
-      <c r="T47" s="35" t="n"/>
-      <c r="U47" s="35" t="n"/>
-      <c r="V47" s="35" t="n"/>
-      <c r="W47" s="35" t="n"/>
-      <c r="X47" s="35" t="n"/>
-      <c r="Y47" s="35" t="n"/>
-      <c r="Z47" s="35" t="n"/>
-      <c r="AA47" s="35" t="n"/>
-      <c r="AB47" s="35" t="n"/>
+      <c r="B47" s="42" t="n"/>
+      <c r="N47" s="43" t="n"/>
+      <c r="P47" s="42" t="n"/>
+      <c r="AB47" s="43" t="n"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="B48" s="35" t="n"/>
-      <c r="C48" s="35" t="n"/>
-      <c r="D48" s="35" t="n"/>
-      <c r="E48" s="35" t="n"/>
-      <c r="F48" s="35" t="n"/>
-      <c r="G48" s="35" t="n"/>
-      <c r="H48" s="35" t="n"/>
-      <c r="I48" s="35" t="n"/>
-      <c r="J48" s="35" t="n"/>
-      <c r="K48" s="35" t="n"/>
-      <c r="L48" s="35" t="n"/>
-      <c r="M48" s="35" t="n"/>
-      <c r="N48" s="35" t="n"/>
-      <c r="P48" s="35" t="n"/>
-      <c r="Q48" s="35" t="n"/>
-      <c r="R48" s="35" t="n"/>
-      <c r="S48" s="35" t="n"/>
-      <c r="T48" s="35" t="n"/>
-      <c r="U48" s="35" t="n"/>
-      <c r="V48" s="35" t="n"/>
-      <c r="W48" s="35" t="n"/>
-      <c r="X48" s="35" t="n"/>
-      <c r="Y48" s="35" t="n"/>
-      <c r="Z48" s="35" t="n"/>
-      <c r="AA48" s="35" t="n"/>
-      <c r="AB48" s="35" t="n"/>
+      <c r="B48" s="42" t="n"/>
+      <c r="N48" s="43" t="n"/>
+      <c r="P48" s="42" t="n"/>
+      <c r="AB48" s="43" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="B49" s="35" t="n"/>
-      <c r="C49" s="35" t="n"/>
-      <c r="D49" s="35" t="n"/>
-      <c r="E49" s="35" t="n"/>
-      <c r="F49" s="35" t="n"/>
-      <c r="G49" s="35" t="n"/>
-      <c r="H49" s="35" t="n"/>
-      <c r="I49" s="35" t="n"/>
-      <c r="J49" s="35" t="n"/>
-      <c r="K49" s="35" t="n"/>
-      <c r="L49" s="35" t="n"/>
-      <c r="M49" s="35" t="n"/>
-      <c r="N49" s="35" t="n"/>
-      <c r="P49" s="35" t="n"/>
-      <c r="Q49" s="35" t="n"/>
-      <c r="R49" s="35" t="n"/>
-      <c r="S49" s="35" t="n"/>
-      <c r="T49" s="35" t="n"/>
-      <c r="U49" s="35" t="n"/>
-      <c r="V49" s="35" t="n"/>
-      <c r="W49" s="35" t="n"/>
-      <c r="X49" s="35" t="n"/>
-      <c r="Y49" s="35" t="n"/>
-      <c r="Z49" s="35" t="n"/>
-      <c r="AA49" s="35" t="n"/>
-      <c r="AB49" s="35" t="n"/>
+      <c r="B49" s="42" t="n"/>
+      <c r="N49" s="43" t="n"/>
+      <c r="P49" s="42" t="n"/>
+      <c r="AB49" s="43" t="n"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="B50" s="35" t="n"/>
-      <c r="C50" s="35" t="n"/>
-      <c r="D50" s="35" t="n"/>
-      <c r="E50" s="35" t="n"/>
-      <c r="F50" s="35" t="n"/>
-      <c r="G50" s="35" t="n"/>
-      <c r="H50" s="35" t="n"/>
-      <c r="I50" s="35" t="n"/>
-      <c r="J50" s="35" t="n"/>
-      <c r="K50" s="35" t="n"/>
-      <c r="L50" s="35" t="n"/>
-      <c r="M50" s="35" t="n"/>
-      <c r="N50" s="35" t="n"/>
-      <c r="P50" s="35" t="n"/>
-      <c r="Q50" s="35" t="n"/>
-      <c r="R50" s="35" t="n"/>
-      <c r="S50" s="35" t="n"/>
-      <c r="T50" s="35" t="n"/>
-      <c r="U50" s="35" t="n"/>
-      <c r="V50" s="35" t="n"/>
-      <c r="W50" s="35" t="n"/>
-      <c r="X50" s="35" t="n"/>
-      <c r="Y50" s="35" t="n"/>
-      <c r="Z50" s="35" t="n"/>
-      <c r="AA50" s="35" t="n"/>
-      <c r="AB50" s="35" t="n"/>
+      <c r="B50" s="42" t="n"/>
+      <c r="N50" s="43" t="n"/>
+      <c r="P50" s="42" t="n"/>
+      <c r="AB50" s="43" t="n"/>
     </row>
     <row r="51" ht="16" customHeight="1">
-      <c r="B51" s="35" t="n"/>
-      <c r="C51" s="35" t="n"/>
-      <c r="D51" s="35" t="n"/>
-      <c r="E51" s="35" t="n"/>
-      <c r="F51" s="35" t="n"/>
-      <c r="G51" s="35" t="n"/>
-      <c r="H51" s="35" t="n"/>
-      <c r="I51" s="35" t="n"/>
-      <c r="J51" s="35" t="n"/>
-      <c r="K51" s="35" t="n"/>
-      <c r="L51" s="35" t="n"/>
-      <c r="M51" s="35" t="n"/>
-      <c r="N51" s="35" t="n"/>
-      <c r="P51" s="35" t="n"/>
-      <c r="Q51" s="35" t="n"/>
-      <c r="R51" s="35" t="n"/>
-      <c r="S51" s="35" t="n"/>
-      <c r="T51" s="35" t="n"/>
-      <c r="U51" s="35" t="n"/>
-      <c r="V51" s="35" t="n"/>
-      <c r="W51" s="35" t="n"/>
-      <c r="X51" s="35" t="n"/>
-      <c r="Y51" s="35" t="n"/>
-      <c r="Z51" s="35" t="n"/>
-      <c r="AA51" s="35" t="n"/>
-      <c r="AB51" s="35" t="n"/>
+      <c r="B51" s="42" t="n"/>
+      <c r="N51" s="43" t="n"/>
+      <c r="P51" s="42" t="n"/>
+      <c r="AB51" s="43" t="n"/>
     </row>
     <row r="52" ht="16" customHeight="1">
-      <c r="B52" s="35" t="n"/>
-      <c r="C52" s="35" t="n"/>
-      <c r="D52" s="35" t="n"/>
-      <c r="E52" s="35" t="n"/>
-      <c r="F52" s="35" t="n"/>
-      <c r="G52" s="35" t="n"/>
-      <c r="H52" s="35" t="n"/>
-      <c r="I52" s="35" t="n"/>
-      <c r="J52" s="35" t="n"/>
-      <c r="K52" s="35" t="n"/>
-      <c r="L52" s="35" t="n"/>
-      <c r="M52" s="35" t="n"/>
-      <c r="N52" s="35" t="n"/>
-      <c r="P52" s="35" t="n"/>
-      <c r="Q52" s="35" t="n"/>
-      <c r="R52" s="35" t="n"/>
-      <c r="S52" s="35" t="n"/>
-      <c r="T52" s="35" t="n"/>
-      <c r="U52" s="35" t="n"/>
-      <c r="V52" s="35" t="n"/>
-      <c r="W52" s="35" t="n"/>
-      <c r="X52" s="35" t="n"/>
-      <c r="Y52" s="35" t="n"/>
-      <c r="Z52" s="35" t="n"/>
-      <c r="AA52" s="35" t="n"/>
-      <c r="AB52" s="35" t="n"/>
+      <c r="B52" s="42" t="n"/>
+      <c r="N52" s="43" t="n"/>
+      <c r="P52" s="42" t="n"/>
+      <c r="AB52" s="43" t="n"/>
     </row>
     <row r="53" ht="16" customHeight="1">
-      <c r="B53" s="35" t="n"/>
-      <c r="C53" s="35" t="n"/>
-      <c r="D53" s="35" t="n"/>
-      <c r="E53" s="35" t="n"/>
-      <c r="F53" s="35" t="n"/>
-      <c r="G53" s="35" t="n"/>
-      <c r="H53" s="35" t="n"/>
-      <c r="I53" s="35" t="n"/>
-      <c r="J53" s="35" t="n"/>
-      <c r="K53" s="35" t="n"/>
-      <c r="L53" s="35" t="n"/>
-      <c r="M53" s="35" t="n"/>
-      <c r="N53" s="35" t="n"/>
-      <c r="P53" s="35" t="n"/>
-      <c r="Q53" s="35" t="n"/>
-      <c r="R53" s="35" t="n"/>
-      <c r="S53" s="35" t="n"/>
-      <c r="T53" s="35" t="n"/>
-      <c r="U53" s="35" t="n"/>
-      <c r="V53" s="35" t="n"/>
-      <c r="W53" s="35" t="n"/>
-      <c r="X53" s="35" t="n"/>
-      <c r="Y53" s="35" t="n"/>
-      <c r="Z53" s="35" t="n"/>
-      <c r="AA53" s="35" t="n"/>
-      <c r="AB53" s="35" t="n"/>
+      <c r="B53" s="44" t="n"/>
+      <c r="C53" s="45" t="n"/>
+      <c r="D53" s="45" t="n"/>
+      <c r="E53" s="45" t="n"/>
+      <c r="F53" s="45" t="n"/>
+      <c r="G53" s="45" t="n"/>
+      <c r="H53" s="45" t="n"/>
+      <c r="I53" s="45" t="n"/>
+      <c r="J53" s="45" t="n"/>
+      <c r="K53" s="45" t="n"/>
+      <c r="L53" s="45" t="n"/>
+      <c r="M53" s="45" t="n"/>
+      <c r="N53" s="46" t="n"/>
+      <c r="P53" s="44" t="n"/>
+      <c r="Q53" s="45" t="n"/>
+      <c r="R53" s="45" t="n"/>
+      <c r="S53" s="45" t="n"/>
+      <c r="T53" s="45" t="n"/>
+      <c r="U53" s="45" t="n"/>
+      <c r="V53" s="45" t="n"/>
+      <c r="W53" s="45" t="n"/>
+      <c r="X53" s="45" t="n"/>
+      <c r="Y53" s="45" t="n"/>
+      <c r="Z53" s="45" t="n"/>
+      <c r="AA53" s="45" t="n"/>
+      <c r="AB53" s="46" t="n"/>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="36" t="inlineStr">
@@ -4320,61 +3732,61 @@
           <t>조치내용</t>
         </is>
       </c>
-      <c r="C54" s="19" t="n"/>
+      <c r="C54" s="27" t="n"/>
       <c r="D54" s="51" t="inlineStr"/>
-      <c r="E54" s="7" t="n"/>
-      <c r="F54" s="7" t="n"/>
-      <c r="G54" s="7" t="n"/>
-      <c r="H54" s="7" t="n"/>
-      <c r="I54" s="7" t="n"/>
-      <c r="J54" s="7" t="n"/>
-      <c r="K54" s="7" t="n"/>
-      <c r="L54" s="7" t="n"/>
-      <c r="M54" s="7" t="n"/>
-      <c r="N54" s="7" t="n"/>
-      <c r="O54" s="7" t="n"/>
-      <c r="P54" s="7" t="n"/>
-      <c r="Q54" s="7" t="n"/>
-      <c r="R54" s="7" t="n"/>
-      <c r="S54" s="7" t="n"/>
-      <c r="T54" s="7" t="n"/>
-      <c r="U54" s="7" t="n"/>
-      <c r="V54" s="7" t="n"/>
-      <c r="W54" s="7" t="n"/>
-      <c r="X54" s="7" t="n"/>
-      <c r="Y54" s="7" t="n"/>
-      <c r="Z54" s="7" t="n"/>
-      <c r="AA54" s="7" t="n"/>
-      <c r="AB54" s="7" t="n"/>
+      <c r="E54" s="26" t="n"/>
+      <c r="F54" s="26" t="n"/>
+      <c r="G54" s="26" t="n"/>
+      <c r="H54" s="26" t="n"/>
+      <c r="I54" s="26" t="n"/>
+      <c r="J54" s="26" t="n"/>
+      <c r="K54" s="26" t="n"/>
+      <c r="L54" s="26" t="n"/>
+      <c r="M54" s="26" t="n"/>
+      <c r="N54" s="26" t="n"/>
+      <c r="O54" s="26" t="n"/>
+      <c r="P54" s="26" t="n"/>
+      <c r="Q54" s="26" t="n"/>
+      <c r="R54" s="26" t="n"/>
+      <c r="S54" s="26" t="n"/>
+      <c r="T54" s="26" t="n"/>
+      <c r="U54" s="26" t="n"/>
+      <c r="V54" s="26" t="n"/>
+      <c r="W54" s="26" t="n"/>
+      <c r="X54" s="26" t="n"/>
+      <c r="Y54" s="26" t="n"/>
+      <c r="Z54" s="26" t="n"/>
+      <c r="AA54" s="26" t="n"/>
+      <c r="AB54" s="27" t="n"/>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="B55" s="19" t="n"/>
-      <c r="C55" s="19" t="n"/>
-      <c r="D55" s="7" t="n"/>
-      <c r="E55" s="7" t="n"/>
-      <c r="F55" s="7" t="n"/>
-      <c r="G55" s="7" t="n"/>
-      <c r="H55" s="7" t="n"/>
-      <c r="I55" s="7" t="n"/>
-      <c r="J55" s="7" t="n"/>
-      <c r="K55" s="7" t="n"/>
-      <c r="L55" s="7" t="n"/>
-      <c r="M55" s="7" t="n"/>
-      <c r="N55" s="7" t="n"/>
-      <c r="O55" s="7" t="n"/>
-      <c r="P55" s="7" t="n"/>
-      <c r="Q55" s="7" t="n"/>
-      <c r="R55" s="7" t="n"/>
-      <c r="S55" s="7" t="n"/>
-      <c r="T55" s="7" t="n"/>
-      <c r="U55" s="7" t="n"/>
-      <c r="V55" s="7" t="n"/>
-      <c r="W55" s="7" t="n"/>
-      <c r="X55" s="7" t="n"/>
-      <c r="Y55" s="7" t="n"/>
-      <c r="Z55" s="7" t="n"/>
-      <c r="AA55" s="7" t="n"/>
-      <c r="AB55" s="7" t="n"/>
+      <c r="B55" s="30" t="n"/>
+      <c r="C55" s="32" t="n"/>
+      <c r="D55" s="30" t="n"/>
+      <c r="E55" s="31" t="n"/>
+      <c r="F55" s="31" t="n"/>
+      <c r="G55" s="31" t="n"/>
+      <c r="H55" s="31" t="n"/>
+      <c r="I55" s="31" t="n"/>
+      <c r="J55" s="31" t="n"/>
+      <c r="K55" s="31" t="n"/>
+      <c r="L55" s="31" t="n"/>
+      <c r="M55" s="31" t="n"/>
+      <c r="N55" s="31" t="n"/>
+      <c r="O55" s="31" t="n"/>
+      <c r="P55" s="31" t="n"/>
+      <c r="Q55" s="31" t="n"/>
+      <c r="R55" s="31" t="n"/>
+      <c r="S55" s="31" t="n"/>
+      <c r="T55" s="31" t="n"/>
+      <c r="U55" s="31" t="n"/>
+      <c r="V55" s="31" t="n"/>
+      <c r="W55" s="31" t="n"/>
+      <c r="X55" s="31" t="n"/>
+      <c r="Y55" s="31" t="n"/>
+      <c r="Z55" s="31" t="n"/>
+      <c r="AA55" s="31" t="n"/>
+      <c r="AB55" s="32" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="B56" s="36" t="inlineStr">
@@ -4382,36 +3794,36 @@
           <t>조치일자</t>
         </is>
       </c>
-      <c r="C56" s="19" t="n"/>
+      <c r="C56" s="23" t="n"/>
       <c r="D56" s="12" t="inlineStr"/>
-      <c r="E56" s="7" t="n"/>
-      <c r="F56" s="7" t="n"/>
-      <c r="G56" s="7" t="n"/>
-      <c r="H56" s="7" t="n"/>
-      <c r="I56" s="7" t="n"/>
+      <c r="E56" s="22" t="n"/>
+      <c r="F56" s="22" t="n"/>
+      <c r="G56" s="22" t="n"/>
+      <c r="H56" s="22" t="n"/>
+      <c r="I56" s="23" t="n"/>
       <c r="J56" s="36" t="inlineStr">
         <is>
           <t>확인자</t>
         </is>
       </c>
-      <c r="K56" s="19" t="n"/>
-      <c r="L56" s="19" t="n"/>
+      <c r="K56" s="22" t="n"/>
+      <c r="L56" s="23" t="n"/>
       <c r="M56" s="12" t="inlineStr"/>
-      <c r="N56" s="7" t="n"/>
-      <c r="O56" s="7" t="n"/>
-      <c r="P56" s="7" t="n"/>
-      <c r="Q56" s="7" t="n"/>
-      <c r="R56" s="7" t="n"/>
-      <c r="S56" s="7" t="n"/>
-      <c r="T56" s="7" t="n"/>
-      <c r="U56" s="7" t="n"/>
-      <c r="V56" s="7" t="n"/>
-      <c r="W56" s="7" t="n"/>
-      <c r="X56" s="7" t="n"/>
-      <c r="Y56" s="7" t="n"/>
-      <c r="Z56" s="7" t="n"/>
-      <c r="AA56" s="7" t="n"/>
-      <c r="AB56" s="7" t="n"/>
+      <c r="N56" s="22" t="n"/>
+      <c r="O56" s="22" t="n"/>
+      <c r="P56" s="22" t="n"/>
+      <c r="Q56" s="22" t="n"/>
+      <c r="R56" s="22" t="n"/>
+      <c r="S56" s="22" t="n"/>
+      <c r="T56" s="22" t="n"/>
+      <c r="U56" s="22" t="n"/>
+      <c r="V56" s="22" t="n"/>
+      <c r="W56" s="22" t="n"/>
+      <c r="X56" s="22" t="n"/>
+      <c r="Y56" s="22" t="n"/>
+      <c r="Z56" s="22" t="n"/>
+      <c r="AA56" s="22" t="n"/>
+      <c r="AB56" s="23" t="n"/>
     </row>
     <row r="57" ht="14" customHeight="1"/>
   </sheetData>
@@ -4432,8 +3844,8 @@
     <mergeCell ref="I7:AB7"/>
     <mergeCell ref="B54:C55"/>
     <mergeCell ref="B25:N25"/>
+    <mergeCell ref="J56:L56"/>
     <mergeCell ref="I41:AB41"/>
-    <mergeCell ref="J56:L56"/>
     <mergeCell ref="D39:I39"/>
     <mergeCell ref="D7:H7"/>
     <mergeCell ref="P25:AB25"/>
@@ -4462,4 +3874,1589 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF305496"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:AB33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4.6" customWidth="1" min="2" max="2"/>
+    <col width="4.6" customWidth="1" min="3" max="3"/>
+    <col width="4.6" customWidth="1" min="4" max="4"/>
+    <col width="4.6" customWidth="1" min="5" max="5"/>
+    <col width="4.6" customWidth="1" min="6" max="6"/>
+    <col width="4.6" customWidth="1" min="7" max="7"/>
+    <col width="4.6" customWidth="1" min="8" max="8"/>
+    <col width="4.6" customWidth="1" min="9" max="9"/>
+    <col width="4.6" customWidth="1" min="10" max="10"/>
+    <col width="4.6" customWidth="1" min="11" max="11"/>
+    <col width="4.6" customWidth="1" min="12" max="12"/>
+    <col width="4.6" customWidth="1" min="13" max="13"/>
+    <col width="4.6" customWidth="1" min="14" max="14"/>
+    <col width="4.6" customWidth="1" min="15" max="15"/>
+    <col width="4.6" customWidth="1" min="16" max="16"/>
+    <col width="4.6" customWidth="1" min="17" max="17"/>
+    <col width="4.6" customWidth="1" min="18" max="18"/>
+    <col width="4.6" customWidth="1" min="19" max="19"/>
+    <col width="4.6" customWidth="1" min="20" max="20"/>
+    <col width="4.6" customWidth="1" min="21" max="21"/>
+    <col width="4.6" customWidth="1" min="22" max="22"/>
+    <col width="4.6" customWidth="1" min="23" max="23"/>
+    <col width="4.6" customWidth="1" min="24" max="24"/>
+    <col width="4.6" customWidth="1" min="25" max="25"/>
+    <col width="4.6" customWidth="1" min="26" max="26"/>
+    <col width="4.6" customWidth="1" min="27" max="27"/>
+    <col width="4.6" customWidth="1" min="28" max="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="6" customHeight="1"/>
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>경영책임자 현장 순회점검 결과보고서</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+      <c r="Z2" s="2" t="n"/>
+      <c r="AA2" s="2" t="n"/>
+      <c r="AB2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>(중대재해처벌법 시행령 제4조 - 안전보건관리체계 구축·이행 점검 결과)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="8" customHeight="1"/>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>현장(사업장)명:</t>
+        </is>
+      </c>
+      <c r="D5" s="53">
+        <f>'현장순회점검표'!F6</f>
+        <v/>
+      </c>
+      <c r="N5" s="52" t="inlineStr">
+        <is>
+          <t>점검일시:</t>
+        </is>
+      </c>
+      <c r="P5" s="54">
+        <f>'현장순회점검표'!F7</f>
+        <v/>
+      </c>
+      <c r="W5" s="52" t="inlineStr">
+        <is>
+          <t>점검자:</t>
+        </is>
+      </c>
+      <c r="Y5" s="54">
+        <f>'현장순회점검표'!T7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="8" customHeight="1"/>
+    <row r="7" ht="20" customHeight="1">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>1. 점검결과 요약</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="5" t="n"/>
+      <c r="Q7" s="5" t="n"/>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="5" t="n"/>
+      <c r="T7" s="5" t="n"/>
+      <c r="U7" s="5" t="n"/>
+      <c r="V7" s="5" t="n"/>
+      <c r="W7" s="5" t="n"/>
+      <c r="X7" s="5" t="n"/>
+      <c r="Y7" s="5" t="n"/>
+      <c r="Z7" s="5" t="n"/>
+      <c r="AA7" s="5" t="n"/>
+      <c r="AB7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>점검항목수</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="n"/>
+      <c r="J8" s="10" t="n"/>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>양호</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="n"/>
+      <c r="M8" s="10" t="n"/>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>미흡</t>
+        </is>
+      </c>
+      <c r="O8" s="10" t="n"/>
+      <c r="P8" s="10" t="n"/>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="R8" s="10" t="n"/>
+      <c r="S8" s="10" t="n"/>
+      <c r="T8" s="9" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+      <c r="U8" s="10" t="n"/>
+      <c r="V8" s="10" t="n"/>
+      <c r="W8" s="10" t="n"/>
+      <c r="X8" s="10" t="n"/>
+      <c r="Y8" s="10" t="n"/>
+      <c r="Z8" s="10" t="n"/>
+      <c r="AA8" s="10" t="n"/>
+      <c r="AB8" s="10" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>안전보건관리체계</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="55" t="inlineStr"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="55" t="inlineStr"/>
+      <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="55" t="inlineStr"/>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="7" t="n"/>
+      <c r="Q9" s="55" t="inlineStr"/>
+      <c r="R9" s="7" t="n"/>
+      <c r="S9" s="7" t="n"/>
+      <c r="T9" s="14" t="inlineStr"/>
+      <c r="U9" s="7" t="n"/>
+      <c r="V9" s="7" t="n"/>
+      <c r="W9" s="7" t="n"/>
+      <c r="X9" s="7" t="n"/>
+      <c r="Y9" s="7" t="n"/>
+      <c r="Z9" s="7" t="n"/>
+      <c r="AA9" s="7" t="n"/>
+      <c r="AB9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>위험성평가</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="55" t="inlineStr"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="55" t="inlineStr"/>
+      <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="55" t="inlineStr"/>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="7" t="n"/>
+      <c r="Q10" s="55" t="inlineStr"/>
+      <c r="R10" s="7" t="n"/>
+      <c r="S10" s="7" t="n"/>
+      <c r="T10" s="14" t="inlineStr"/>
+      <c r="U10" s="7" t="n"/>
+      <c r="V10" s="7" t="n"/>
+      <c r="W10" s="7" t="n"/>
+      <c r="X10" s="7" t="n"/>
+      <c r="Y10" s="7" t="n"/>
+      <c r="Z10" s="7" t="n"/>
+      <c r="AA10" s="7" t="n"/>
+      <c r="AB10" s="7" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>안전교육</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="55" t="inlineStr"/>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="55" t="inlineStr"/>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7" t="n"/>
+      <c r="N11" s="55" t="inlineStr"/>
+      <c r="O11" s="7" t="n"/>
+      <c r="P11" s="7" t="n"/>
+      <c r="Q11" s="55" t="inlineStr"/>
+      <c r="R11" s="7" t="n"/>
+      <c r="S11" s="7" t="n"/>
+      <c r="T11" s="14" t="inlineStr"/>
+      <c r="U11" s="7" t="n"/>
+      <c r="V11" s="7" t="n"/>
+      <c r="W11" s="7" t="n"/>
+      <c r="X11" s="7" t="n"/>
+      <c r="Y11" s="7" t="n"/>
+      <c r="Z11" s="7" t="n"/>
+      <c r="AA11" s="7" t="n"/>
+      <c r="AB11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>현장 안전시설·보호구</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="55" t="inlineStr"/>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="55" t="inlineStr"/>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="55" t="inlineStr"/>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="7" t="n"/>
+      <c r="Q12" s="55" t="inlineStr"/>
+      <c r="R12" s="7" t="n"/>
+      <c r="S12" s="7" t="n"/>
+      <c r="T12" s="14" t="inlineStr"/>
+      <c r="U12" s="7" t="n"/>
+      <c r="V12" s="7" t="n"/>
+      <c r="W12" s="7" t="n"/>
+      <c r="X12" s="7" t="n"/>
+      <c r="Y12" s="7" t="n"/>
+      <c r="Z12" s="7" t="n"/>
+      <c r="AA12" s="7" t="n"/>
+      <c r="AB12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>협력업체(수급인) 관리</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="55" t="inlineStr"/>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="55" t="inlineStr"/>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="55" t="inlineStr"/>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="7" t="n"/>
+      <c r="Q13" s="55" t="inlineStr"/>
+      <c r="R13" s="7" t="n"/>
+      <c r="S13" s="7" t="n"/>
+      <c r="T13" s="14" t="inlineStr"/>
+      <c r="U13" s="7" t="n"/>
+      <c r="V13" s="7" t="n"/>
+      <c r="W13" s="7" t="n"/>
+      <c r="X13" s="7" t="n"/>
+      <c r="Y13" s="7" t="n"/>
+      <c r="Z13" s="7" t="n"/>
+      <c r="AA13" s="7" t="n"/>
+      <c r="AB13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>근로자 의견청취 및 개선</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="55" t="inlineStr"/>
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="55" t="inlineStr"/>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="55" t="inlineStr"/>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="7" t="n"/>
+      <c r="Q14" s="55" t="inlineStr"/>
+      <c r="R14" s="7" t="n"/>
+      <c r="S14" s="7" t="n"/>
+      <c r="T14" s="14" t="inlineStr"/>
+      <c r="U14" s="7" t="n"/>
+      <c r="V14" s="7" t="n"/>
+      <c r="W14" s="7" t="n"/>
+      <c r="X14" s="7" t="n"/>
+      <c r="Y14" s="7" t="n"/>
+      <c r="Z14" s="7" t="n"/>
+      <c r="AA14" s="7" t="n"/>
+      <c r="AB14" s="7" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="17" t="n"/>
+      <c r="H15" s="56">
+        <f>SUM(H9:H14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="17" t="n"/>
+      <c r="J15" s="17" t="n"/>
+      <c r="K15" s="56">
+        <f>SUM(K9:K14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="17" t="n"/>
+      <c r="M15" s="17" t="n"/>
+      <c r="N15" s="56">
+        <f>SUM(N9:N14)</f>
+        <v/>
+      </c>
+      <c r="O15" s="17" t="n"/>
+      <c r="P15" s="17" t="n"/>
+      <c r="Q15" s="56">
+        <f>SUM(Q9:Q14)</f>
+        <v/>
+      </c>
+      <c r="R15" s="17" t="n"/>
+      <c r="S15" s="17" t="n"/>
+      <c r="T15" s="14" t="inlineStr"/>
+      <c r="U15" s="7" t="n"/>
+      <c r="V15" s="7" t="n"/>
+      <c r="W15" s="7" t="n"/>
+      <c r="X15" s="7" t="n"/>
+      <c r="Y15" s="7" t="n"/>
+      <c r="Z15" s="7" t="n"/>
+      <c r="AA15" s="7" t="n"/>
+      <c r="AB15" s="7" t="n"/>
+    </row>
+    <row r="16" ht="8" customHeight="1"/>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>2. 주요 지적사항 목록</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
+      <c r="K17" s="5" t="n"/>
+      <c r="L17" s="5" t="n"/>
+      <c r="M17" s="5" t="n"/>
+      <c r="N17" s="5" t="n"/>
+      <c r="O17" s="5" t="n"/>
+      <c r="P17" s="5" t="n"/>
+      <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="5" t="n"/>
+      <c r="S17" s="5" t="n"/>
+      <c r="T17" s="5" t="n"/>
+      <c r="U17" s="5" t="n"/>
+      <c r="V17" s="5" t="n"/>
+      <c r="W17" s="5" t="n"/>
+      <c r="X17" s="5" t="n"/>
+      <c r="Y17" s="5" t="n"/>
+      <c r="Z17" s="5" t="n"/>
+      <c r="AA17" s="5" t="n"/>
+      <c r="AB17" s="5" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>지적사항 내용</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="n"/>
+      <c r="K18" s="10" t="n"/>
+      <c r="L18" s="10" t="n"/>
+      <c r="M18" s="10" t="n"/>
+      <c r="N18" s="10" t="n"/>
+      <c r="O18" s="10" t="n"/>
+      <c r="P18" s="10" t="n"/>
+      <c r="Q18" s="10" t="n"/>
+      <c r="R18" s="10" t="n"/>
+      <c r="S18" s="10" t="n"/>
+      <c r="T18" s="9" t="inlineStr">
+        <is>
+          <t>위험도
+(상/중/하)</t>
+        </is>
+      </c>
+      <c r="U18" s="10" t="n"/>
+      <c r="V18" s="10" t="n"/>
+      <c r="W18" s="9" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+      <c r="X18" s="10" t="n"/>
+      <c r="Y18" s="10" t="n"/>
+      <c r="Z18" s="10" t="n"/>
+      <c r="AA18" s="10" t="n"/>
+      <c r="AB18" s="10" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="14" t="inlineStr"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="14" t="inlineStr"/>
+      <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="n"/>
+      <c r="N19" s="7" t="n"/>
+      <c r="O19" s="7" t="n"/>
+      <c r="P19" s="7" t="n"/>
+      <c r="Q19" s="7" t="n"/>
+      <c r="R19" s="7" t="n"/>
+      <c r="S19" s="7" t="n"/>
+      <c r="T19" s="55" t="inlineStr"/>
+      <c r="U19" s="7" t="n"/>
+      <c r="V19" s="7" t="n"/>
+      <c r="W19" s="14" t="inlineStr"/>
+      <c r="X19" s="7" t="n"/>
+      <c r="Y19" s="7" t="n"/>
+      <c r="Z19" s="7" t="n"/>
+      <c r="AA19" s="7" t="n"/>
+      <c r="AB19" s="7" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="14" t="inlineStr"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="14" t="inlineStr"/>
+      <c r="J20" s="7" t="n"/>
+      <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
+      <c r="N20" s="7" t="n"/>
+      <c r="O20" s="7" t="n"/>
+      <c r="P20" s="7" t="n"/>
+      <c r="Q20" s="7" t="n"/>
+      <c r="R20" s="7" t="n"/>
+      <c r="S20" s="7" t="n"/>
+      <c r="T20" s="55" t="inlineStr"/>
+      <c r="U20" s="7" t="n"/>
+      <c r="V20" s="7" t="n"/>
+      <c r="W20" s="14" t="inlineStr"/>
+      <c r="X20" s="7" t="n"/>
+      <c r="Y20" s="7" t="n"/>
+      <c r="Z20" s="7" t="n"/>
+      <c r="AA20" s="7" t="n"/>
+      <c r="AB20" s="7" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="14" t="inlineStr"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="14" t="inlineStr"/>
+      <c r="J21" s="7" t="n"/>
+      <c r="K21" s="7" t="n"/>
+      <c r="L21" s="7" t="n"/>
+      <c r="M21" s="7" t="n"/>
+      <c r="N21" s="7" t="n"/>
+      <c r="O21" s="7" t="n"/>
+      <c r="P21" s="7" t="n"/>
+      <c r="Q21" s="7" t="n"/>
+      <c r="R21" s="7" t="n"/>
+      <c r="S21" s="7" t="n"/>
+      <c r="T21" s="55" t="inlineStr"/>
+      <c r="U21" s="7" t="n"/>
+      <c r="V21" s="7" t="n"/>
+      <c r="W21" s="14" t="inlineStr"/>
+      <c r="X21" s="7" t="n"/>
+      <c r="Y21" s="7" t="n"/>
+      <c r="Z21" s="7" t="n"/>
+      <c r="AA21" s="7" t="n"/>
+      <c r="AB21" s="7" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="14" t="inlineStr"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="14" t="inlineStr"/>
+      <c r="J22" s="7" t="n"/>
+      <c r="K22" s="7" t="n"/>
+      <c r="L22" s="7" t="n"/>
+      <c r="M22" s="7" t="n"/>
+      <c r="N22" s="7" t="n"/>
+      <c r="O22" s="7" t="n"/>
+      <c r="P22" s="7" t="n"/>
+      <c r="Q22" s="7" t="n"/>
+      <c r="R22" s="7" t="n"/>
+      <c r="S22" s="7" t="n"/>
+      <c r="T22" s="55" t="inlineStr"/>
+      <c r="U22" s="7" t="n"/>
+      <c r="V22" s="7" t="n"/>
+      <c r="W22" s="14" t="inlineStr"/>
+      <c r="X22" s="7" t="n"/>
+      <c r="Y22" s="7" t="n"/>
+      <c r="Z22" s="7" t="n"/>
+      <c r="AA22" s="7" t="n"/>
+      <c r="AB22" s="7" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="55" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="14" t="inlineStr"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="14" t="inlineStr"/>
+      <c r="J23" s="7" t="n"/>
+      <c r="K23" s="7" t="n"/>
+      <c r="L23" s="7" t="n"/>
+      <c r="M23" s="7" t="n"/>
+      <c r="N23" s="7" t="n"/>
+      <c r="O23" s="7" t="n"/>
+      <c r="P23" s="7" t="n"/>
+      <c r="Q23" s="7" t="n"/>
+      <c r="R23" s="7" t="n"/>
+      <c r="S23" s="7" t="n"/>
+      <c r="T23" s="55" t="inlineStr"/>
+      <c r="U23" s="7" t="n"/>
+      <c r="V23" s="7" t="n"/>
+      <c r="W23" s="14" t="inlineStr"/>
+      <c r="X23" s="7" t="n"/>
+      <c r="Y23" s="7" t="n"/>
+      <c r="Z23" s="7" t="n"/>
+      <c r="AA23" s="7" t="n"/>
+      <c r="AB23" s="7" t="n"/>
+    </row>
+    <row r="24" ht="8" customHeight="1"/>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>3. 종합의견</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="n"/>
+      <c r="I25" s="5" t="n"/>
+      <c r="J25" s="5" t="n"/>
+      <c r="K25" s="5" t="n"/>
+      <c r="L25" s="5" t="n"/>
+      <c r="M25" s="5" t="n"/>
+      <c r="N25" s="5" t="n"/>
+      <c r="O25" s="5" t="n"/>
+      <c r="P25" s="5" t="n"/>
+      <c r="Q25" s="5" t="n"/>
+      <c r="R25" s="5" t="n"/>
+      <c r="S25" s="5" t="n"/>
+      <c r="T25" s="5" t="n"/>
+      <c r="U25" s="5" t="n"/>
+      <c r="V25" s="5" t="n"/>
+      <c r="W25" s="5" t="n"/>
+      <c r="X25" s="5" t="n"/>
+      <c r="Y25" s="5" t="n"/>
+      <c r="Z25" s="5" t="n"/>
+      <c r="AA25" s="5" t="n"/>
+      <c r="AB25" s="5" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="57" t="inlineStr"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="7" t="n"/>
+      <c r="J26" s="7" t="n"/>
+      <c r="K26" s="7" t="n"/>
+      <c r="L26" s="7" t="n"/>
+      <c r="M26" s="7" t="n"/>
+      <c r="N26" s="7" t="n"/>
+      <c r="O26" s="7" t="n"/>
+      <c r="P26" s="7" t="n"/>
+      <c r="Q26" s="7" t="n"/>
+      <c r="R26" s="7" t="n"/>
+      <c r="S26" s="7" t="n"/>
+      <c r="T26" s="7" t="n"/>
+      <c r="U26" s="7" t="n"/>
+      <c r="V26" s="7" t="n"/>
+      <c r="W26" s="7" t="n"/>
+      <c r="X26" s="7" t="n"/>
+      <c r="Y26" s="7" t="n"/>
+      <c r="Z26" s="7" t="n"/>
+      <c r="AA26" s="7" t="n"/>
+      <c r="AB26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="n"/>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="7" t="n"/>
+      <c r="J27" s="7" t="n"/>
+      <c r="K27" s="7" t="n"/>
+      <c r="L27" s="7" t="n"/>
+      <c r="M27" s="7" t="n"/>
+      <c r="N27" s="7" t="n"/>
+      <c r="O27" s="7" t="n"/>
+      <c r="P27" s="7" t="n"/>
+      <c r="Q27" s="7" t="n"/>
+      <c r="R27" s="7" t="n"/>
+      <c r="S27" s="7" t="n"/>
+      <c r="T27" s="7" t="n"/>
+      <c r="U27" s="7" t="n"/>
+      <c r="V27" s="7" t="n"/>
+      <c r="W27" s="7" t="n"/>
+      <c r="X27" s="7" t="n"/>
+      <c r="Y27" s="7" t="n"/>
+      <c r="Z27" s="7" t="n"/>
+      <c r="AA27" s="7" t="n"/>
+      <c r="AB27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+      <c r="H28" s="7" t="n"/>
+      <c r="I28" s="7" t="n"/>
+      <c r="J28" s="7" t="n"/>
+      <c r="K28" s="7" t="n"/>
+      <c r="L28" s="7" t="n"/>
+      <c r="M28" s="7" t="n"/>
+      <c r="N28" s="7" t="n"/>
+      <c r="O28" s="7" t="n"/>
+      <c r="P28" s="7" t="n"/>
+      <c r="Q28" s="7" t="n"/>
+      <c r="R28" s="7" t="n"/>
+      <c r="S28" s="7" t="n"/>
+      <c r="T28" s="7" t="n"/>
+      <c r="U28" s="7" t="n"/>
+      <c r="V28" s="7" t="n"/>
+      <c r="W28" s="7" t="n"/>
+      <c r="X28" s="7" t="n"/>
+      <c r="Y28" s="7" t="n"/>
+      <c r="Z28" s="7" t="n"/>
+      <c r="AA28" s="7" t="n"/>
+      <c r="AB28" s="7" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="7" t="n"/>
+      <c r="J29" s="7" t="n"/>
+      <c r="K29" s="7" t="n"/>
+      <c r="L29" s="7" t="n"/>
+      <c r="M29" s="7" t="n"/>
+      <c r="N29" s="7" t="n"/>
+      <c r="O29" s="7" t="n"/>
+      <c r="P29" s="7" t="n"/>
+      <c r="Q29" s="7" t="n"/>
+      <c r="R29" s="7" t="n"/>
+      <c r="S29" s="7" t="n"/>
+      <c r="T29" s="7" t="n"/>
+      <c r="U29" s="7" t="n"/>
+      <c r="V29" s="7" t="n"/>
+      <c r="W29" s="7" t="n"/>
+      <c r="X29" s="7" t="n"/>
+      <c r="Y29" s="7" t="n"/>
+      <c r="Z29" s="7" t="n"/>
+      <c r="AA29" s="7" t="n"/>
+      <c r="AB29" s="7" t="n"/>
+    </row>
+    <row r="30" ht="8" customHeight="1"/>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>4. 보고 및 결재</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
+      <c r="K31" s="5" t="n"/>
+      <c r="L31" s="5" t="n"/>
+      <c r="M31" s="5" t="n"/>
+      <c r="N31" s="5" t="n"/>
+      <c r="O31" s="5" t="n"/>
+      <c r="P31" s="5" t="n"/>
+      <c r="Q31" s="5" t="n"/>
+      <c r="R31" s="5" t="n"/>
+      <c r="S31" s="5" t="n"/>
+      <c r="T31" s="5" t="n"/>
+      <c r="U31" s="5" t="n"/>
+      <c r="V31" s="5" t="n"/>
+      <c r="W31" s="5" t="n"/>
+      <c r="X31" s="5" t="n"/>
+      <c r="Y31" s="5" t="n"/>
+      <c r="Z31" s="5" t="n"/>
+      <c r="AA31" s="5" t="n"/>
+      <c r="AB31" s="5" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>경영책임자</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="n"/>
+      <c r="D32" s="17" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="17" t="n"/>
+      <c r="H32" s="17" t="n"/>
+      <c r="I32" s="17" t="n"/>
+      <c r="J32" s="17" t="n"/>
+      <c r="K32" s="13" t="inlineStr">
+        <is>
+          <t>현장소장
+(안전보건관리책임자)</t>
+        </is>
+      </c>
+      <c r="L32" s="17" t="n"/>
+      <c r="M32" s="17" t="n"/>
+      <c r="N32" s="17" t="n"/>
+      <c r="O32" s="17" t="n"/>
+      <c r="P32" s="17" t="n"/>
+      <c r="Q32" s="17" t="n"/>
+      <c r="R32" s="17" t="n"/>
+      <c r="S32" s="17" t="n"/>
+      <c r="T32" s="13" t="inlineStr">
+        <is>
+          <t>안전관리자</t>
+        </is>
+      </c>
+      <c r="U32" s="17" t="n"/>
+      <c r="V32" s="17" t="n"/>
+      <c r="W32" s="17" t="n"/>
+      <c r="X32" s="17" t="n"/>
+      <c r="Y32" s="17" t="n"/>
+      <c r="Z32" s="17" t="n"/>
+      <c r="AA32" s="17" t="n"/>
+      <c r="AB32" s="17" t="n"/>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="B33" s="55" t="inlineStr">
+        <is>
+          <t>(서명)</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="n"/>
+      <c r="H33" s="7" t="n"/>
+      <c r="I33" s="7" t="n"/>
+      <c r="J33" s="7" t="n"/>
+      <c r="K33" s="55" t="inlineStr">
+        <is>
+          <t>(서명)</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="n"/>
+      <c r="M33" s="7" t="n"/>
+      <c r="N33" s="7" t="n"/>
+      <c r="O33" s="7" t="n"/>
+      <c r="P33" s="7" t="n"/>
+      <c r="Q33" s="7" t="n"/>
+      <c r="R33" s="7" t="n"/>
+      <c r="S33" s="7" t="n"/>
+      <c r="T33" s="55" t="inlineStr">
+        <is>
+          <t>(서명)</t>
+        </is>
+      </c>
+      <c r="U33" s="7" t="n"/>
+      <c r="V33" s="7" t="n"/>
+      <c r="W33" s="7" t="n"/>
+      <c r="X33" s="7" t="n"/>
+      <c r="Y33" s="7" t="n"/>
+      <c r="Z33" s="7" t="n"/>
+      <c r="AA33" s="7" t="n"/>
+      <c r="AB33" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="97">
+    <mergeCell ref="Q14:S14"/>
+    <mergeCell ref="W20:AB20"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="W22:AB22"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="T12:AB12"/>
+    <mergeCell ref="Q15:S15"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="T22:V22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N5:O5"/>
+    <mergeCell ref="I18:S18"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="W23:AB23"/>
+    <mergeCell ref="B32:J32"/>
+    <mergeCell ref="T20:V20"/>
+    <mergeCell ref="T33:AB33"/>
+    <mergeCell ref="K9:M9"/>
+    <mergeCell ref="I20:S20"/>
+    <mergeCell ref="B25:AB25"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="T10:AB10"/>
+    <mergeCell ref="K32:S32"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="T9:AB9"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="K8:M8"/>
+    <mergeCell ref="T11:AB11"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="T19:V19"/>
+    <mergeCell ref="Q13:S13"/>
+    <mergeCell ref="T15:AB15"/>
+    <mergeCell ref="B7:AB7"/>
+    <mergeCell ref="I19:S19"/>
+    <mergeCell ref="B3:AB3"/>
+    <mergeCell ref="Q8:S8"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="Q10:S10"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="B2:AB2"/>
+    <mergeCell ref="T21:V21"/>
+    <mergeCell ref="W5:X5"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="T23:V23"/>
+    <mergeCell ref="W18:AB18"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="D5:L5"/>
+    <mergeCell ref="K13:M13"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="T18:V18"/>
+    <mergeCell ref="W19:AB19"/>
+    <mergeCell ref="I23:S23"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="Q12:S12"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="T32:AB32"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="T14:AB14"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="B17:AB17"/>
+    <mergeCell ref="W21:AB21"/>
+    <mergeCell ref="B26:AB29"/>
+    <mergeCell ref="N13:P13"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="Q9:S9"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="T13:AB13"/>
+    <mergeCell ref="T8:AB8"/>
+    <mergeCell ref="I22:S22"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="Q11:S11"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="I21:S21"/>
+    <mergeCell ref="P5:U5"/>
+    <mergeCell ref="Y5:AB5"/>
+    <mergeCell ref="K33:S33"/>
+    <mergeCell ref="B31:AB31"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF305496"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:AB18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4.6" customWidth="1" min="2" max="2"/>
+    <col width="4.6" customWidth="1" min="3" max="3"/>
+    <col width="4.6" customWidth="1" min="4" max="4"/>
+    <col width="4.6" customWidth="1" min="5" max="5"/>
+    <col width="4.6" customWidth="1" min="6" max="6"/>
+    <col width="4.6" customWidth="1" min="7" max="7"/>
+    <col width="4.6" customWidth="1" min="8" max="8"/>
+    <col width="4.6" customWidth="1" min="9" max="9"/>
+    <col width="4.6" customWidth="1" min="10" max="10"/>
+    <col width="4.6" customWidth="1" min="11" max="11"/>
+    <col width="4.6" customWidth="1" min="12" max="12"/>
+    <col width="4.6" customWidth="1" min="13" max="13"/>
+    <col width="4.6" customWidth="1" min="14" max="14"/>
+    <col width="4.6" customWidth="1" min="15" max="15"/>
+    <col width="4.6" customWidth="1" min="16" max="16"/>
+    <col width="4.6" customWidth="1" min="17" max="17"/>
+    <col width="4.6" customWidth="1" min="18" max="18"/>
+    <col width="4.6" customWidth="1" min="19" max="19"/>
+    <col width="4.6" customWidth="1" min="20" max="20"/>
+    <col width="4.6" customWidth="1" min="21" max="21"/>
+    <col width="4.6" customWidth="1" min="22" max="22"/>
+    <col width="4.6" customWidth="1" min="23" max="23"/>
+    <col width="4.6" customWidth="1" min="24" max="24"/>
+    <col width="4.6" customWidth="1" min="25" max="25"/>
+    <col width="4.6" customWidth="1" min="26" max="26"/>
+    <col width="4.6" customWidth="1" min="27" max="27"/>
+    <col width="4.6" customWidth="1" min="28" max="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="6" customHeight="1"/>
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>지적사항 조치계획서</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+      <c r="Z2" s="2" t="n"/>
+      <c r="AA2" s="2" t="n"/>
+      <c r="AB2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>(경영책임자 현장 순회점검 지적사항에 대한 원인분석 및 개선조치 계획)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="8" customHeight="1"/>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>현장(사업장)명:</t>
+        </is>
+      </c>
+      <c r="D5" s="54">
+        <f>'현장순회점검표'!F6</f>
+        <v/>
+      </c>
+      <c r="N5" s="52" t="inlineStr">
+        <is>
+          <t>작성일자:</t>
+        </is>
+      </c>
+      <c r="P5" s="53" t="inlineStr"/>
+    </row>
+    <row r="6" ht="8" customHeight="1"/>
+    <row r="7" ht="28" customHeight="1">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>지적사항</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>원인분석</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="n"/>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="10" t="n"/>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>개선대책
+(조치계획)</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="n"/>
+      <c r="N7" s="10" t="n"/>
+      <c r="O7" s="10" t="n"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>담당부서
+/담당자</t>
+        </is>
+      </c>
+      <c r="Q7" s="10" t="n"/>
+      <c r="R7" s="10" t="n"/>
+      <c r="S7" s="9" t="inlineStr">
+        <is>
+          <t>조치예정일</t>
+        </is>
+      </c>
+      <c r="T7" s="10" t="n"/>
+      <c r="U7" s="10" t="n"/>
+      <c r="V7" s="9" t="inlineStr">
+        <is>
+          <t>소요예산
+(원)</t>
+        </is>
+      </c>
+      <c r="W7" s="10" t="n"/>
+      <c r="X7" s="9" t="inlineStr">
+        <is>
+          <t>진행상태</t>
+        </is>
+      </c>
+      <c r="Y7" s="10" t="n"/>
+      <c r="Z7" s="9" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="AA7" s="10" t="n"/>
+      <c r="AB7" s="9" t="inlineStr">
+        <is>
+          <t>확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="B8" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="14" t="inlineStr"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="14" t="inlineStr"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="14" t="inlineStr"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="14" t="inlineStr"/>
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="55" t="inlineStr"/>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="55" t="inlineStr"/>
+      <c r="W8" s="7" t="n"/>
+      <c r="X8" s="55" t="inlineStr"/>
+      <c r="Y8" s="7" t="n"/>
+      <c r="Z8" s="55" t="inlineStr"/>
+      <c r="AA8" s="7" t="n"/>
+      <c r="AB8" s="55" t="inlineStr"/>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="B9" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="14" t="inlineStr"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="14" t="inlineStr"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="14" t="inlineStr"/>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="7" t="n"/>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="14" t="inlineStr"/>
+      <c r="Q9" s="7" t="n"/>
+      <c r="R9" s="7" t="n"/>
+      <c r="S9" s="55" t="inlineStr"/>
+      <c r="T9" s="7" t="n"/>
+      <c r="U9" s="7" t="n"/>
+      <c r="V9" s="55" t="inlineStr"/>
+      <c r="W9" s="7" t="n"/>
+      <c r="X9" s="55" t="inlineStr"/>
+      <c r="Y9" s="7" t="n"/>
+      <c r="Z9" s="55" t="inlineStr"/>
+      <c r="AA9" s="7" t="n"/>
+      <c r="AB9" s="55" t="inlineStr"/>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="B10" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="14" t="inlineStr"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="14" t="inlineStr"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
+      <c r="L10" s="14" t="inlineStr"/>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="7" t="n"/>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="14" t="inlineStr"/>
+      <c r="Q10" s="7" t="n"/>
+      <c r="R10" s="7" t="n"/>
+      <c r="S10" s="55" t="inlineStr"/>
+      <c r="T10" s="7" t="n"/>
+      <c r="U10" s="7" t="n"/>
+      <c r="V10" s="55" t="inlineStr"/>
+      <c r="W10" s="7" t="n"/>
+      <c r="X10" s="55" t="inlineStr"/>
+      <c r="Y10" s="7" t="n"/>
+      <c r="Z10" s="55" t="inlineStr"/>
+      <c r="AA10" s="7" t="n"/>
+      <c r="AB10" s="55" t="inlineStr"/>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="B11" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="14" t="inlineStr"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="14" t="inlineStr"/>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="7" t="n"/>
+      <c r="L11" s="14" t="inlineStr"/>
+      <c r="M11" s="7" t="n"/>
+      <c r="N11" s="7" t="n"/>
+      <c r="O11" s="7" t="n"/>
+      <c r="P11" s="14" t="inlineStr"/>
+      <c r="Q11" s="7" t="n"/>
+      <c r="R11" s="7" t="n"/>
+      <c r="S11" s="55" t="inlineStr"/>
+      <c r="T11" s="7" t="n"/>
+      <c r="U11" s="7" t="n"/>
+      <c r="V11" s="55" t="inlineStr"/>
+      <c r="W11" s="7" t="n"/>
+      <c r="X11" s="55" t="inlineStr"/>
+      <c r="Y11" s="7" t="n"/>
+      <c r="Z11" s="55" t="inlineStr"/>
+      <c r="AA11" s="7" t="n"/>
+      <c r="AB11" s="55" t="inlineStr"/>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="B12" s="55" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="14" t="inlineStr"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="14" t="inlineStr"/>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="7" t="n"/>
+      <c r="L12" s="14" t="inlineStr"/>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="7" t="n"/>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="14" t="inlineStr"/>
+      <c r="Q12" s="7" t="n"/>
+      <c r="R12" s="7" t="n"/>
+      <c r="S12" s="55" t="inlineStr"/>
+      <c r="T12" s="7" t="n"/>
+      <c r="U12" s="7" t="n"/>
+      <c r="V12" s="55" t="inlineStr"/>
+      <c r="W12" s="7" t="n"/>
+      <c r="X12" s="55" t="inlineStr"/>
+      <c r="Y12" s="7" t="n"/>
+      <c r="Z12" s="55" t="inlineStr"/>
+      <c r="AA12" s="7" t="n"/>
+      <c r="AB12" s="55" t="inlineStr"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="B13" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="14" t="inlineStr"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
+      <c r="L13" s="14" t="inlineStr"/>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="n"/>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="14" t="inlineStr"/>
+      <c r="Q13" s="7" t="n"/>
+      <c r="R13" s="7" t="n"/>
+      <c r="S13" s="55" t="inlineStr"/>
+      <c r="T13" s="7" t="n"/>
+      <c r="U13" s="7" t="n"/>
+      <c r="V13" s="55" t="inlineStr"/>
+      <c r="W13" s="7" t="n"/>
+      <c r="X13" s="55" t="inlineStr"/>
+      <c r="Y13" s="7" t="n"/>
+      <c r="Z13" s="55" t="inlineStr"/>
+      <c r="AA13" s="7" t="n"/>
+      <c r="AB13" s="55" t="inlineStr"/>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="B14" s="55" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="14" t="inlineStr"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="14" t="inlineStr"/>
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="n"/>
+      <c r="L14" s="14" t="inlineStr"/>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="7" t="n"/>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="14" t="inlineStr"/>
+      <c r="Q14" s="7" t="n"/>
+      <c r="R14" s="7" t="n"/>
+      <c r="S14" s="55" t="inlineStr"/>
+      <c r="T14" s="7" t="n"/>
+      <c r="U14" s="7" t="n"/>
+      <c r="V14" s="55" t="inlineStr"/>
+      <c r="W14" s="7" t="n"/>
+      <c r="X14" s="55" t="inlineStr"/>
+      <c r="Y14" s="7" t="n"/>
+      <c r="Z14" s="55" t="inlineStr"/>
+      <c r="AA14" s="7" t="n"/>
+      <c r="AB14" s="55" t="inlineStr"/>
+    </row>
+    <row r="15" ht="8" customHeight="1"/>
+    <row r="16" ht="16" customHeight="1">
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>※ 진행상태는 '예정 / 진행중 / 완료' 중 기재하며, 완료 시 완료일과 확인자 서명을 기입한다. 미조치 지적사항은 다음 순회점검 시 재확인한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="8" customHeight="1"/>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>작성자</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="55" t="inlineStr"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="7" t="n"/>
+      <c r="P18" s="13" t="inlineStr">
+        <is>
+          <t>승인(결재)자</t>
+        </is>
+      </c>
+      <c r="Q18" s="17" t="n"/>
+      <c r="R18" s="17" t="n"/>
+      <c r="S18" s="17" t="n"/>
+      <c r="T18" s="55" t="inlineStr"/>
+      <c r="U18" s="7" t="n"/>
+      <c r="V18" s="7" t="n"/>
+      <c r="W18" s="7" t="n"/>
+      <c r="X18" s="7" t="n"/>
+      <c r="Y18" s="7" t="n"/>
+      <c r="Z18" s="7" t="n"/>
+      <c r="AA18" s="7" t="n"/>
+      <c r="AB18" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="91">
+    <mergeCell ref="S14:U14"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="P18:S18"/>
+    <mergeCell ref="X11:Y11"/>
+    <mergeCell ref="Z11:AA11"/>
+    <mergeCell ref="S13:U13"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="N5:O5"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="P14:R14"/>
+    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="Z13:AA13"/>
+    <mergeCell ref="L14:O14"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="V8:W8"/>
+    <mergeCell ref="X8:Y8"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="V10:W10"/>
+    <mergeCell ref="V9:W9"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="AB14"/>
+    <mergeCell ref="Z12:AA12"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="V11:W11"/>
+    <mergeCell ref="X14:Y14"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="Z14:AA14"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="B16:AB16"/>
+    <mergeCell ref="B3:AB3"/>
+    <mergeCell ref="S8:U8"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="P8:R8"/>
+    <mergeCell ref="AB8"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="B2:AB2"/>
+    <mergeCell ref="F18:N18"/>
+    <mergeCell ref="V13:W13"/>
+    <mergeCell ref="AB10"/>
+    <mergeCell ref="X13:Y13"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="X7:Y7"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="Z7:AA7"/>
+    <mergeCell ref="L7:O7"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="Z8:AA8"/>
+    <mergeCell ref="D5:L5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="S12:U12"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="AB12"/>
+    <mergeCell ref="P9:R9"/>
+    <mergeCell ref="L10:O10"/>
+    <mergeCell ref="V12:W12"/>
+    <mergeCell ref="S7:U7"/>
+    <mergeCell ref="X12:Y12"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="AB13"/>
+    <mergeCell ref="AB7"/>
+    <mergeCell ref="V14:W14"/>
+    <mergeCell ref="L11:O11"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="P5:AB5"/>
+    <mergeCell ref="P13:R13"/>
+    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="T18:AB18"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="AB9"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="X10:Y10"/>
+    <mergeCell ref="Z10:AA10"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="AB11"/>
+    <mergeCell ref="X9:Y9"/>
+    <mergeCell ref="Z9:AA9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add corrective action completion report sheet
Adds 지적사항_조치결과보고서 to 경영책임자_현장순회점검표.xlsx, distinct
from 조치계획서 (the plan): confirms actual implementation results per
finding (completion status, action taken, completion date, evidence
photo check, confirmer), an overall completion tally, and a final
sign-off block. Cross-references the 지적사항_조치전후사진대지 sheet as
the photo evidence source for completed items.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SqkinqfGqqfBrcHRBkScVm
</commit_message>
<xml_diff>
--- a/templates/경영책임자_현장순회점검표.xlsx
+++ b/templates/경영책임자_현장순회점검표.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="지적사항_조치전후사진대지" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="결과보고서" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="조치계획서" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="지적사항_조치결과보고서" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'현장순회점검표'!$A$1:$AB$42</definedName>
@@ -19,6 +20,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="2">'지적사항_조치전후사진대지'!$A$1:$AB$58</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'결과보고서'!$A$1:$AB$34</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'조치계획서'!$A$1:$AB$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'지적사항_조치결과보고서'!$A$1:$AB$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -169,6 +171,17 @@
     <font>
       <name val="맑은 고딕"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9.300000000000001"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="FF000000"/>
+      <sz val="9.199999999999999"/>
     </font>
   </fonts>
   <fills count="7">
@@ -430,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -551,6 +564,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -3923,32 +3948,6 @@
           <t>경영책임자 현장 순회점검 결과보고서</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
-      <c r="V2" s="2" t="n"/>
-      <c r="W2" s="2" t="n"/>
-      <c r="X2" s="2" t="n"/>
-      <c r="Y2" s="2" t="n"/>
-      <c r="Z2" s="2" t="n"/>
-      <c r="AA2" s="2" t="n"/>
-      <c r="AB2" s="2" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
@@ -3994,32 +3993,6 @@
           <t>1. 점검결과 요약</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
-      <c r="P7" s="5" t="n"/>
-      <c r="Q7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
-      <c r="S7" s="5" t="n"/>
-      <c r="T7" s="5" t="n"/>
-      <c r="U7" s="5" t="n"/>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="5" t="n"/>
-      <c r="X7" s="5" t="n"/>
-      <c r="Y7" s="5" t="n"/>
-      <c r="Z7" s="5" t="n"/>
-      <c r="AA7" s="5" t="n"/>
-      <c r="AB7" s="5" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="9" t="inlineStr">
@@ -4027,52 +4000,52 @@
           <t>구분</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="22" t="n"/>
+      <c r="F8" s="22" t="n"/>
+      <c r="G8" s="23" t="n"/>
       <c r="H8" s="9" t="inlineStr">
         <is>
           <t>점검항목수</t>
         </is>
       </c>
-      <c r="I8" s="10" t="n"/>
-      <c r="J8" s="10" t="n"/>
+      <c r="I8" s="22" t="n"/>
+      <c r="J8" s="23" t="n"/>
       <c r="K8" s="9" t="inlineStr">
         <is>
           <t>양호</t>
         </is>
       </c>
-      <c r="L8" s="10" t="n"/>
-      <c r="M8" s="10" t="n"/>
+      <c r="L8" s="22" t="n"/>
+      <c r="M8" s="23" t="n"/>
       <c r="N8" s="9" t="inlineStr">
         <is>
           <t>미흡</t>
         </is>
       </c>
-      <c r="O8" s="10" t="n"/>
-      <c r="P8" s="10" t="n"/>
+      <c r="O8" s="22" t="n"/>
+      <c r="P8" s="23" t="n"/>
       <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="R8" s="10" t="n"/>
-      <c r="S8" s="10" t="n"/>
+      <c r="R8" s="22" t="n"/>
+      <c r="S8" s="23" t="n"/>
       <c r="T8" s="9" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-      <c r="U8" s="10" t="n"/>
-      <c r="V8" s="10" t="n"/>
-      <c r="W8" s="10" t="n"/>
-      <c r="X8" s="10" t="n"/>
-      <c r="Y8" s="10" t="n"/>
-      <c r="Z8" s="10" t="n"/>
-      <c r="AA8" s="10" t="n"/>
-      <c r="AB8" s="10" t="n"/>
+      <c r="U8" s="22" t="n"/>
+      <c r="V8" s="22" t="n"/>
+      <c r="W8" s="22" t="n"/>
+      <c r="X8" s="22" t="n"/>
+      <c r="Y8" s="22" t="n"/>
+      <c r="Z8" s="22" t="n"/>
+      <c r="AA8" s="22" t="n"/>
+      <c r="AB8" s="23" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="14" t="inlineStr">
@@ -4080,32 +4053,32 @@
           <t>안전보건관리체계</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="23" t="n"/>
       <c r="H9" s="55" t="inlineStr"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="23" t="n"/>
       <c r="K9" s="55" t="inlineStr"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
+      <c r="L9" s="22" t="n"/>
+      <c r="M9" s="23" t="n"/>
       <c r="N9" s="55" t="inlineStr"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="7" t="n"/>
+      <c r="O9" s="22" t="n"/>
+      <c r="P9" s="23" t="n"/>
       <c r="Q9" s="55" t="inlineStr"/>
-      <c r="R9" s="7" t="n"/>
-      <c r="S9" s="7" t="n"/>
+      <c r="R9" s="22" t="n"/>
+      <c r="S9" s="23" t="n"/>
       <c r="T9" s="14" t="inlineStr"/>
-      <c r="U9" s="7" t="n"/>
-      <c r="V9" s="7" t="n"/>
-      <c r="W9" s="7" t="n"/>
-      <c r="X9" s="7" t="n"/>
-      <c r="Y9" s="7" t="n"/>
-      <c r="Z9" s="7" t="n"/>
-      <c r="AA9" s="7" t="n"/>
-      <c r="AB9" s="7" t="n"/>
+      <c r="U9" s="22" t="n"/>
+      <c r="V9" s="22" t="n"/>
+      <c r="W9" s="22" t="n"/>
+      <c r="X9" s="22" t="n"/>
+      <c r="Y9" s="22" t="n"/>
+      <c r="Z9" s="22" t="n"/>
+      <c r="AA9" s="22" t="n"/>
+      <c r="AB9" s="23" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="14" t="inlineStr">
@@ -4113,32 +4086,32 @@
           <t>위험성평가</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="22" t="n"/>
+      <c r="G10" s="23" t="n"/>
       <c r="H10" s="55" t="inlineStr"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
+      <c r="I10" s="22" t="n"/>
+      <c r="J10" s="23" t="n"/>
       <c r="K10" s="55" t="inlineStr"/>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
+      <c r="L10" s="22" t="n"/>
+      <c r="M10" s="23" t="n"/>
       <c r="N10" s="55" t="inlineStr"/>
-      <c r="O10" s="7" t="n"/>
-      <c r="P10" s="7" t="n"/>
+      <c r="O10" s="22" t="n"/>
+      <c r="P10" s="23" t="n"/>
       <c r="Q10" s="55" t="inlineStr"/>
-      <c r="R10" s="7" t="n"/>
-      <c r="S10" s="7" t="n"/>
+      <c r="R10" s="22" t="n"/>
+      <c r="S10" s="23" t="n"/>
       <c r="T10" s="14" t="inlineStr"/>
-      <c r="U10" s="7" t="n"/>
-      <c r="V10" s="7" t="n"/>
-      <c r="W10" s="7" t="n"/>
-      <c r="X10" s="7" t="n"/>
-      <c r="Y10" s="7" t="n"/>
-      <c r="Z10" s="7" t="n"/>
-      <c r="AA10" s="7" t="n"/>
-      <c r="AB10" s="7" t="n"/>
+      <c r="U10" s="22" t="n"/>
+      <c r="V10" s="22" t="n"/>
+      <c r="W10" s="22" t="n"/>
+      <c r="X10" s="22" t="n"/>
+      <c r="Y10" s="22" t="n"/>
+      <c r="Z10" s="22" t="n"/>
+      <c r="AA10" s="22" t="n"/>
+      <c r="AB10" s="23" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="14" t="inlineStr">
@@ -4146,32 +4119,32 @@
           <t>안전교육</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
+      <c r="F11" s="22" t="n"/>
+      <c r="G11" s="23" t="n"/>
       <c r="H11" s="55" t="inlineStr"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
+      <c r="I11" s="22" t="n"/>
+      <c r="J11" s="23" t="n"/>
       <c r="K11" s="55" t="inlineStr"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
+      <c r="L11" s="22" t="n"/>
+      <c r="M11" s="23" t="n"/>
       <c r="N11" s="55" t="inlineStr"/>
-      <c r="O11" s="7" t="n"/>
-      <c r="P11" s="7" t="n"/>
+      <c r="O11" s="22" t="n"/>
+      <c r="P11" s="23" t="n"/>
       <c r="Q11" s="55" t="inlineStr"/>
-      <c r="R11" s="7" t="n"/>
-      <c r="S11" s="7" t="n"/>
+      <c r="R11" s="22" t="n"/>
+      <c r="S11" s="23" t="n"/>
       <c r="T11" s="14" t="inlineStr"/>
-      <c r="U11" s="7" t="n"/>
-      <c r="V11" s="7" t="n"/>
-      <c r="W11" s="7" t="n"/>
-      <c r="X11" s="7" t="n"/>
-      <c r="Y11" s="7" t="n"/>
-      <c r="Z11" s="7" t="n"/>
-      <c r="AA11" s="7" t="n"/>
-      <c r="AB11" s="7" t="n"/>
+      <c r="U11" s="22" t="n"/>
+      <c r="V11" s="22" t="n"/>
+      <c r="W11" s="22" t="n"/>
+      <c r="X11" s="22" t="n"/>
+      <c r="Y11" s="22" t="n"/>
+      <c r="Z11" s="22" t="n"/>
+      <c r="AA11" s="22" t="n"/>
+      <c r="AB11" s="23" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="14" t="inlineStr">
@@ -4179,32 +4152,32 @@
           <t>현장 안전시설·보호구</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="22" t="n"/>
+      <c r="F12" s="22" t="n"/>
+      <c r="G12" s="23" t="n"/>
       <c r="H12" s="55" t="inlineStr"/>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
+      <c r="I12" s="22" t="n"/>
+      <c r="J12" s="23" t="n"/>
       <c r="K12" s="55" t="inlineStr"/>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="n"/>
+      <c r="L12" s="22" t="n"/>
+      <c r="M12" s="23" t="n"/>
       <c r="N12" s="55" t="inlineStr"/>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="7" t="n"/>
+      <c r="O12" s="22" t="n"/>
+      <c r="P12" s="23" t="n"/>
       <c r="Q12" s="55" t="inlineStr"/>
-      <c r="R12" s="7" t="n"/>
-      <c r="S12" s="7" t="n"/>
+      <c r="R12" s="22" t="n"/>
+      <c r="S12" s="23" t="n"/>
       <c r="T12" s="14" t="inlineStr"/>
-      <c r="U12" s="7" t="n"/>
-      <c r="V12" s="7" t="n"/>
-      <c r="W12" s="7" t="n"/>
-      <c r="X12" s="7" t="n"/>
-      <c r="Y12" s="7" t="n"/>
-      <c r="Z12" s="7" t="n"/>
-      <c r="AA12" s="7" t="n"/>
-      <c r="AB12" s="7" t="n"/>
+      <c r="U12" s="22" t="n"/>
+      <c r="V12" s="22" t="n"/>
+      <c r="W12" s="22" t="n"/>
+      <c r="X12" s="22" t="n"/>
+      <c r="Y12" s="22" t="n"/>
+      <c r="Z12" s="22" t="n"/>
+      <c r="AA12" s="22" t="n"/>
+      <c r="AB12" s="23" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="14" t="inlineStr">
@@ -4212,32 +4185,32 @@
           <t>협력업체(수급인) 관리</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
+      <c r="C13" s="22" t="n"/>
+      <c r="D13" s="22" t="n"/>
+      <c r="E13" s="22" t="n"/>
+      <c r="F13" s="22" t="n"/>
+      <c r="G13" s="23" t="n"/>
       <c r="H13" s="55" t="inlineStr"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
+      <c r="I13" s="22" t="n"/>
+      <c r="J13" s="23" t="n"/>
       <c r="K13" s="55" t="inlineStr"/>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
+      <c r="L13" s="22" t="n"/>
+      <c r="M13" s="23" t="n"/>
       <c r="N13" s="55" t="inlineStr"/>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="7" t="n"/>
+      <c r="O13" s="22" t="n"/>
+      <c r="P13" s="23" t="n"/>
       <c r="Q13" s="55" t="inlineStr"/>
-      <c r="R13" s="7" t="n"/>
-      <c r="S13" s="7" t="n"/>
+      <c r="R13" s="22" t="n"/>
+      <c r="S13" s="23" t="n"/>
       <c r="T13" s="14" t="inlineStr"/>
-      <c r="U13" s="7" t="n"/>
-      <c r="V13" s="7" t="n"/>
-      <c r="W13" s="7" t="n"/>
-      <c r="X13" s="7" t="n"/>
-      <c r="Y13" s="7" t="n"/>
-      <c r="Z13" s="7" t="n"/>
-      <c r="AA13" s="7" t="n"/>
-      <c r="AB13" s="7" t="n"/>
+      <c r="U13" s="22" t="n"/>
+      <c r="V13" s="22" t="n"/>
+      <c r="W13" s="22" t="n"/>
+      <c r="X13" s="22" t="n"/>
+      <c r="Y13" s="22" t="n"/>
+      <c r="Z13" s="22" t="n"/>
+      <c r="AA13" s="22" t="n"/>
+      <c r="AB13" s="23" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="B14" s="14" t="inlineStr">
@@ -4245,32 +4218,32 @@
           <t>근로자 의견청취 및 개선</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
+      <c r="C14" s="22" t="n"/>
+      <c r="D14" s="22" t="n"/>
+      <c r="E14" s="22" t="n"/>
+      <c r="F14" s="22" t="n"/>
+      <c r="G14" s="23" t="n"/>
       <c r="H14" s="55" t="inlineStr"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="n"/>
+      <c r="I14" s="22" t="n"/>
+      <c r="J14" s="23" t="n"/>
       <c r="K14" s="55" t="inlineStr"/>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7" t="n"/>
+      <c r="L14" s="22" t="n"/>
+      <c r="M14" s="23" t="n"/>
       <c r="N14" s="55" t="inlineStr"/>
-      <c r="O14" s="7" t="n"/>
-      <c r="P14" s="7" t="n"/>
+      <c r="O14" s="22" t="n"/>
+      <c r="P14" s="23" t="n"/>
       <c r="Q14" s="55" t="inlineStr"/>
-      <c r="R14" s="7" t="n"/>
-      <c r="S14" s="7" t="n"/>
+      <c r="R14" s="22" t="n"/>
+      <c r="S14" s="23" t="n"/>
       <c r="T14" s="14" t="inlineStr"/>
-      <c r="U14" s="7" t="n"/>
-      <c r="V14" s="7" t="n"/>
-      <c r="W14" s="7" t="n"/>
-      <c r="X14" s="7" t="n"/>
-      <c r="Y14" s="7" t="n"/>
-      <c r="Z14" s="7" t="n"/>
-      <c r="AA14" s="7" t="n"/>
-      <c r="AB14" s="7" t="n"/>
+      <c r="U14" s="22" t="n"/>
+      <c r="V14" s="22" t="n"/>
+      <c r="W14" s="22" t="n"/>
+      <c r="X14" s="22" t="n"/>
+      <c r="Y14" s="22" t="n"/>
+      <c r="Z14" s="22" t="n"/>
+      <c r="AA14" s="22" t="n"/>
+      <c r="AB14" s="23" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="13" t="inlineStr">
@@ -4278,44 +4251,44 @@
           <t>합계</t>
         </is>
       </c>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n"/>
-      <c r="G15" s="17" t="n"/>
+      <c r="C15" s="22" t="n"/>
+      <c r="D15" s="22" t="n"/>
+      <c r="E15" s="22" t="n"/>
+      <c r="F15" s="22" t="n"/>
+      <c r="G15" s="23" t="n"/>
       <c r="H15" s="56">
         <f>SUM(H9:H14)</f>
         <v/>
       </c>
-      <c r="I15" s="17" t="n"/>
-      <c r="J15" s="17" t="n"/>
+      <c r="I15" s="22" t="n"/>
+      <c r="J15" s="23" t="n"/>
       <c r="K15" s="56">
         <f>SUM(K9:K14)</f>
         <v/>
       </c>
-      <c r="L15" s="17" t="n"/>
-      <c r="M15" s="17" t="n"/>
+      <c r="L15" s="22" t="n"/>
+      <c r="M15" s="23" t="n"/>
       <c r="N15" s="56">
         <f>SUM(N9:N14)</f>
         <v/>
       </c>
-      <c r="O15" s="17" t="n"/>
-      <c r="P15" s="17" t="n"/>
+      <c r="O15" s="22" t="n"/>
+      <c r="P15" s="23" t="n"/>
       <c r="Q15" s="56">
         <f>SUM(Q9:Q14)</f>
         <v/>
       </c>
-      <c r="R15" s="17" t="n"/>
-      <c r="S15" s="17" t="n"/>
+      <c r="R15" s="22" t="n"/>
+      <c r="S15" s="23" t="n"/>
       <c r="T15" s="14" t="inlineStr"/>
-      <c r="U15" s="7" t="n"/>
-      <c r="V15" s="7" t="n"/>
-      <c r="W15" s="7" t="n"/>
-      <c r="X15" s="7" t="n"/>
-      <c r="Y15" s="7" t="n"/>
-      <c r="Z15" s="7" t="n"/>
-      <c r="AA15" s="7" t="n"/>
-      <c r="AB15" s="7" t="n"/>
+      <c r="U15" s="22" t="n"/>
+      <c r="V15" s="22" t="n"/>
+      <c r="W15" s="22" t="n"/>
+      <c r="X15" s="22" t="n"/>
+      <c r="Y15" s="22" t="n"/>
+      <c r="Z15" s="22" t="n"/>
+      <c r="AA15" s="22" t="n"/>
+      <c r="AB15" s="23" t="n"/>
     </row>
     <row r="16" ht="8" customHeight="1"/>
     <row r="17" ht="20" customHeight="1">
@@ -4324,32 +4297,6 @@
           <t>2. 주요 지적사항 목록</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
-      <c r="L17" s="5" t="n"/>
-      <c r="M17" s="5" t="n"/>
-      <c r="N17" s="5" t="n"/>
-      <c r="O17" s="5" t="n"/>
-      <c r="P17" s="5" t="n"/>
-      <c r="Q17" s="5" t="n"/>
-      <c r="R17" s="5" t="n"/>
-      <c r="S17" s="5" t="n"/>
-      <c r="T17" s="5" t="n"/>
-      <c r="U17" s="5" t="n"/>
-      <c r="V17" s="5" t="n"/>
-      <c r="W17" s="5" t="n"/>
-      <c r="X17" s="5" t="n"/>
-      <c r="Y17" s="5" t="n"/>
-      <c r="Z17" s="5" t="n"/>
-      <c r="AA17" s="5" t="n"/>
-      <c r="AB17" s="5" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="B18" s="9" t="inlineStr">
@@ -4357,204 +4304,204 @@
           <t>No</t>
         </is>
       </c>
-      <c r="C18" s="10" t="n"/>
+      <c r="C18" s="23" t="n"/>
       <c r="D18" s="9" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="10" t="n"/>
+      <c r="E18" s="22" t="n"/>
+      <c r="F18" s="22" t="n"/>
+      <c r="G18" s="22" t="n"/>
+      <c r="H18" s="23" t="n"/>
       <c r="I18" s="9" t="inlineStr">
         <is>
           <t>지적사항 내용</t>
         </is>
       </c>
-      <c r="J18" s="10" t="n"/>
-      <c r="K18" s="10" t="n"/>
-      <c r="L18" s="10" t="n"/>
-      <c r="M18" s="10" t="n"/>
-      <c r="N18" s="10" t="n"/>
-      <c r="O18" s="10" t="n"/>
-      <c r="P18" s="10" t="n"/>
-      <c r="Q18" s="10" t="n"/>
-      <c r="R18" s="10" t="n"/>
-      <c r="S18" s="10" t="n"/>
+      <c r="J18" s="22" t="n"/>
+      <c r="K18" s="22" t="n"/>
+      <c r="L18" s="22" t="n"/>
+      <c r="M18" s="22" t="n"/>
+      <c r="N18" s="22" t="n"/>
+      <c r="O18" s="22" t="n"/>
+      <c r="P18" s="22" t="n"/>
+      <c r="Q18" s="22" t="n"/>
+      <c r="R18" s="22" t="n"/>
+      <c r="S18" s="23" t="n"/>
       <c r="T18" s="9" t="inlineStr">
         <is>
           <t>위험도
 (상/중/하)</t>
         </is>
       </c>
-      <c r="U18" s="10" t="n"/>
-      <c r="V18" s="10" t="n"/>
+      <c r="U18" s="22" t="n"/>
+      <c r="V18" s="23" t="n"/>
       <c r="W18" s="9" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-      <c r="X18" s="10" t="n"/>
-      <c r="Y18" s="10" t="n"/>
-      <c r="Z18" s="10" t="n"/>
-      <c r="AA18" s="10" t="n"/>
-      <c r="AB18" s="10" t="n"/>
+      <c r="X18" s="22" t="n"/>
+      <c r="Y18" s="22" t="n"/>
+      <c r="Z18" s="22" t="n"/>
+      <c r="AA18" s="22" t="n"/>
+      <c r="AB18" s="23" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="7" t="n"/>
+      <c r="C19" s="23" t="n"/>
       <c r="D19" s="14" t="inlineStr"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
+      <c r="E19" s="22" t="n"/>
+      <c r="F19" s="22" t="n"/>
+      <c r="G19" s="22" t="n"/>
+      <c r="H19" s="23" t="n"/>
       <c r="I19" s="14" t="inlineStr"/>
-      <c r="J19" s="7" t="n"/>
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
-      <c r="N19" s="7" t="n"/>
-      <c r="O19" s="7" t="n"/>
-      <c r="P19" s="7" t="n"/>
-      <c r="Q19" s="7" t="n"/>
-      <c r="R19" s="7" t="n"/>
-      <c r="S19" s="7" t="n"/>
+      <c r="J19" s="22" t="n"/>
+      <c r="K19" s="22" t="n"/>
+      <c r="L19" s="22" t="n"/>
+      <c r="M19" s="22" t="n"/>
+      <c r="N19" s="22" t="n"/>
+      <c r="O19" s="22" t="n"/>
+      <c r="P19" s="22" t="n"/>
+      <c r="Q19" s="22" t="n"/>
+      <c r="R19" s="22" t="n"/>
+      <c r="S19" s="23" t="n"/>
       <c r="T19" s="55" t="inlineStr"/>
-      <c r="U19" s="7" t="n"/>
-      <c r="V19" s="7" t="n"/>
+      <c r="U19" s="22" t="n"/>
+      <c r="V19" s="23" t="n"/>
       <c r="W19" s="14" t="inlineStr"/>
-      <c r="X19" s="7" t="n"/>
-      <c r="Y19" s="7" t="n"/>
-      <c r="Z19" s="7" t="n"/>
-      <c r="AA19" s="7" t="n"/>
-      <c r="AB19" s="7" t="n"/>
+      <c r="X19" s="22" t="n"/>
+      <c r="Y19" s="22" t="n"/>
+      <c r="Z19" s="22" t="n"/>
+      <c r="AA19" s="22" t="n"/>
+      <c r="AB19" s="23" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="C20" s="7" t="n"/>
+      <c r="C20" s="23" t="n"/>
       <c r="D20" s="14" t="inlineStr"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
+      <c r="E20" s="22" t="n"/>
+      <c r="F20" s="22" t="n"/>
+      <c r="G20" s="22" t="n"/>
+      <c r="H20" s="23" t="n"/>
       <c r="I20" s="14" t="inlineStr"/>
-      <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
-      <c r="O20" s="7" t="n"/>
-      <c r="P20" s="7" t="n"/>
-      <c r="Q20" s="7" t="n"/>
-      <c r="R20" s="7" t="n"/>
-      <c r="S20" s="7" t="n"/>
+      <c r="J20" s="22" t="n"/>
+      <c r="K20" s="22" t="n"/>
+      <c r="L20" s="22" t="n"/>
+      <c r="M20" s="22" t="n"/>
+      <c r="N20" s="22" t="n"/>
+      <c r="O20" s="22" t="n"/>
+      <c r="P20" s="22" t="n"/>
+      <c r="Q20" s="22" t="n"/>
+      <c r="R20" s="22" t="n"/>
+      <c r="S20" s="23" t="n"/>
       <c r="T20" s="55" t="inlineStr"/>
-      <c r="U20" s="7" t="n"/>
-      <c r="V20" s="7" t="n"/>
+      <c r="U20" s="22" t="n"/>
+      <c r="V20" s="23" t="n"/>
       <c r="W20" s="14" t="inlineStr"/>
-      <c r="X20" s="7" t="n"/>
-      <c r="Y20" s="7" t="n"/>
-      <c r="Z20" s="7" t="n"/>
-      <c r="AA20" s="7" t="n"/>
-      <c r="AB20" s="7" t="n"/>
+      <c r="X20" s="22" t="n"/>
+      <c r="Y20" s="22" t="n"/>
+      <c r="Z20" s="22" t="n"/>
+      <c r="AA20" s="22" t="n"/>
+      <c r="AB20" s="23" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="55" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="7" t="n"/>
+      <c r="C21" s="23" t="n"/>
       <c r="D21" s="14" t="inlineStr"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
+      <c r="E21" s="22" t="n"/>
+      <c r="F21" s="22" t="n"/>
+      <c r="G21" s="22" t="n"/>
+      <c r="H21" s="23" t="n"/>
       <c r="I21" s="14" t="inlineStr"/>
-      <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
-      <c r="P21" s="7" t="n"/>
-      <c r="Q21" s="7" t="n"/>
-      <c r="R21" s="7" t="n"/>
-      <c r="S21" s="7" t="n"/>
+      <c r="J21" s="22" t="n"/>
+      <c r="K21" s="22" t="n"/>
+      <c r="L21" s="22" t="n"/>
+      <c r="M21" s="22" t="n"/>
+      <c r="N21" s="22" t="n"/>
+      <c r="O21" s="22" t="n"/>
+      <c r="P21" s="22" t="n"/>
+      <c r="Q21" s="22" t="n"/>
+      <c r="R21" s="22" t="n"/>
+      <c r="S21" s="23" t="n"/>
       <c r="T21" s="55" t="inlineStr"/>
-      <c r="U21" s="7" t="n"/>
-      <c r="V21" s="7" t="n"/>
+      <c r="U21" s="22" t="n"/>
+      <c r="V21" s="23" t="n"/>
       <c r="W21" s="14" t="inlineStr"/>
-      <c r="X21" s="7" t="n"/>
-      <c r="Y21" s="7" t="n"/>
-      <c r="Z21" s="7" t="n"/>
-      <c r="AA21" s="7" t="n"/>
-      <c r="AB21" s="7" t="n"/>
+      <c r="X21" s="22" t="n"/>
+      <c r="Y21" s="22" t="n"/>
+      <c r="Z21" s="22" t="n"/>
+      <c r="AA21" s="22" t="n"/>
+      <c r="AB21" s="23" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="55" t="n">
         <v>4</v>
       </c>
-      <c r="C22" s="7" t="n"/>
+      <c r="C22" s="23" t="n"/>
       <c r="D22" s="14" t="inlineStr"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
+      <c r="E22" s="22" t="n"/>
+      <c r="F22" s="22" t="n"/>
+      <c r="G22" s="22" t="n"/>
+      <c r="H22" s="23" t="n"/>
       <c r="I22" s="14" t="inlineStr"/>
-      <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="7" t="n"/>
-      <c r="Q22" s="7" t="n"/>
-      <c r="R22" s="7" t="n"/>
-      <c r="S22" s="7" t="n"/>
+      <c r="J22" s="22" t="n"/>
+      <c r="K22" s="22" t="n"/>
+      <c r="L22" s="22" t="n"/>
+      <c r="M22" s="22" t="n"/>
+      <c r="N22" s="22" t="n"/>
+      <c r="O22" s="22" t="n"/>
+      <c r="P22" s="22" t="n"/>
+      <c r="Q22" s="22" t="n"/>
+      <c r="R22" s="22" t="n"/>
+      <c r="S22" s="23" t="n"/>
       <c r="T22" s="55" t="inlineStr"/>
-      <c r="U22" s="7" t="n"/>
-      <c r="V22" s="7" t="n"/>
+      <c r="U22" s="22" t="n"/>
+      <c r="V22" s="23" t="n"/>
       <c r="W22" s="14" t="inlineStr"/>
-      <c r="X22" s="7" t="n"/>
-      <c r="Y22" s="7" t="n"/>
-      <c r="Z22" s="7" t="n"/>
-      <c r="AA22" s="7" t="n"/>
-      <c r="AB22" s="7" t="n"/>
+      <c r="X22" s="22" t="n"/>
+      <c r="Y22" s="22" t="n"/>
+      <c r="Z22" s="22" t="n"/>
+      <c r="AA22" s="22" t="n"/>
+      <c r="AB22" s="23" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="55" t="n">
         <v>5</v>
       </c>
-      <c r="C23" s="7" t="n"/>
+      <c r="C23" s="23" t="n"/>
       <c r="D23" s="14" t="inlineStr"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="7" t="n"/>
+      <c r="E23" s="22" t="n"/>
+      <c r="F23" s="22" t="n"/>
+      <c r="G23" s="22" t="n"/>
+      <c r="H23" s="23" t="n"/>
       <c r="I23" s="14" t="inlineStr"/>
-      <c r="J23" s="7" t="n"/>
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="n"/>
-      <c r="N23" s="7" t="n"/>
-      <c r="O23" s="7" t="n"/>
-      <c r="P23" s="7" t="n"/>
-      <c r="Q23" s="7" t="n"/>
-      <c r="R23" s="7" t="n"/>
-      <c r="S23" s="7" t="n"/>
+      <c r="J23" s="22" t="n"/>
+      <c r="K23" s="22" t="n"/>
+      <c r="L23" s="22" t="n"/>
+      <c r="M23" s="22" t="n"/>
+      <c r="N23" s="22" t="n"/>
+      <c r="O23" s="22" t="n"/>
+      <c r="P23" s="22" t="n"/>
+      <c r="Q23" s="22" t="n"/>
+      <c r="R23" s="22" t="n"/>
+      <c r="S23" s="23" t="n"/>
       <c r="T23" s="55" t="inlineStr"/>
-      <c r="U23" s="7" t="n"/>
-      <c r="V23" s="7" t="n"/>
+      <c r="U23" s="22" t="n"/>
+      <c r="V23" s="23" t="n"/>
       <c r="W23" s="14" t="inlineStr"/>
-      <c r="X23" s="7" t="n"/>
-      <c r="Y23" s="7" t="n"/>
-      <c r="Z23" s="7" t="n"/>
-      <c r="AA23" s="7" t="n"/>
-      <c r="AB23" s="7" t="n"/>
+      <c r="X23" s="22" t="n"/>
+      <c r="Y23" s="22" t="n"/>
+      <c r="Z23" s="22" t="n"/>
+      <c r="AA23" s="22" t="n"/>
+      <c r="AB23" s="23" t="n"/>
     </row>
     <row r="24" ht="8" customHeight="1"/>
     <row r="25" ht="20" customHeight="1">
@@ -4563,148 +4510,72 @@
           <t>3. 종합의견</t>
         </is>
       </c>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="5" t="n"/>
-      <c r="K25" s="5" t="n"/>
-      <c r="L25" s="5" t="n"/>
-      <c r="M25" s="5" t="n"/>
-      <c r="N25" s="5" t="n"/>
-      <c r="O25" s="5" t="n"/>
-      <c r="P25" s="5" t="n"/>
-      <c r="Q25" s="5" t="n"/>
-      <c r="R25" s="5" t="n"/>
-      <c r="S25" s="5" t="n"/>
-      <c r="T25" s="5" t="n"/>
-      <c r="U25" s="5" t="n"/>
-      <c r="V25" s="5" t="n"/>
-      <c r="W25" s="5" t="n"/>
-      <c r="X25" s="5" t="n"/>
-      <c r="Y25" s="5" t="n"/>
-      <c r="Z25" s="5" t="n"/>
-      <c r="AA25" s="5" t="n"/>
-      <c r="AB25" s="5" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="B26" s="57" t="inlineStr"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
-      <c r="F26" s="7" t="n"/>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="7" t="n"/>
-      <c r="I26" s="7" t="n"/>
-      <c r="J26" s="7" t="n"/>
-      <c r="K26" s="7" t="n"/>
-      <c r="L26" s="7" t="n"/>
-      <c r="M26" s="7" t="n"/>
-      <c r="N26" s="7" t="n"/>
-      <c r="O26" s="7" t="n"/>
-      <c r="P26" s="7" t="n"/>
-      <c r="Q26" s="7" t="n"/>
-      <c r="R26" s="7" t="n"/>
-      <c r="S26" s="7" t="n"/>
-      <c r="T26" s="7" t="n"/>
-      <c r="U26" s="7" t="n"/>
-      <c r="V26" s="7" t="n"/>
-      <c r="W26" s="7" t="n"/>
-      <c r="X26" s="7" t="n"/>
-      <c r="Y26" s="7" t="n"/>
-      <c r="Z26" s="7" t="n"/>
-      <c r="AA26" s="7" t="n"/>
-      <c r="AB26" s="7" t="n"/>
+      <c r="C26" s="26" t="n"/>
+      <c r="D26" s="26" t="n"/>
+      <c r="E26" s="26" t="n"/>
+      <c r="F26" s="26" t="n"/>
+      <c r="G26" s="26" t="n"/>
+      <c r="H26" s="26" t="n"/>
+      <c r="I26" s="26" t="n"/>
+      <c r="J26" s="26" t="n"/>
+      <c r="K26" s="26" t="n"/>
+      <c r="L26" s="26" t="n"/>
+      <c r="M26" s="26" t="n"/>
+      <c r="N26" s="26" t="n"/>
+      <c r="O26" s="26" t="n"/>
+      <c r="P26" s="26" t="n"/>
+      <c r="Q26" s="26" t="n"/>
+      <c r="R26" s="26" t="n"/>
+      <c r="S26" s="26" t="n"/>
+      <c r="T26" s="26" t="n"/>
+      <c r="U26" s="26" t="n"/>
+      <c r="V26" s="26" t="n"/>
+      <c r="W26" s="26" t="n"/>
+      <c r="X26" s="26" t="n"/>
+      <c r="Y26" s="26" t="n"/>
+      <c r="Z26" s="26" t="n"/>
+      <c r="AA26" s="26" t="n"/>
+      <c r="AB26" s="27" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
-      <c r="F27" s="7" t="n"/>
-      <c r="G27" s="7" t="n"/>
-      <c r="H27" s="7" t="n"/>
-      <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="n"/>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
-      <c r="N27" s="7" t="n"/>
-      <c r="O27" s="7" t="n"/>
-      <c r="P27" s="7" t="n"/>
-      <c r="Q27" s="7" t="n"/>
-      <c r="R27" s="7" t="n"/>
-      <c r="S27" s="7" t="n"/>
-      <c r="T27" s="7" t="n"/>
-      <c r="U27" s="7" t="n"/>
-      <c r="V27" s="7" t="n"/>
-      <c r="W27" s="7" t="n"/>
-      <c r="X27" s="7" t="n"/>
-      <c r="Y27" s="7" t="n"/>
-      <c r="Z27" s="7" t="n"/>
-      <c r="AA27" s="7" t="n"/>
-      <c r="AB27" s="7" t="n"/>
+      <c r="B27" s="28" t="n"/>
+      <c r="AB27" s="29" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
-      <c r="F28" s="7" t="n"/>
-      <c r="G28" s="7" t="n"/>
-      <c r="H28" s="7" t="n"/>
-      <c r="I28" s="7" t="n"/>
-      <c r="J28" s="7" t="n"/>
-      <c r="K28" s="7" t="n"/>
-      <c r="L28" s="7" t="n"/>
-      <c r="M28" s="7" t="n"/>
-      <c r="N28" s="7" t="n"/>
-      <c r="O28" s="7" t="n"/>
-      <c r="P28" s="7" t="n"/>
-      <c r="Q28" s="7" t="n"/>
-      <c r="R28" s="7" t="n"/>
-      <c r="S28" s="7" t="n"/>
-      <c r="T28" s="7" t="n"/>
-      <c r="U28" s="7" t="n"/>
-      <c r="V28" s="7" t="n"/>
-      <c r="W28" s="7" t="n"/>
-      <c r="X28" s="7" t="n"/>
-      <c r="Y28" s="7" t="n"/>
-      <c r="Z28" s="7" t="n"/>
-      <c r="AA28" s="7" t="n"/>
-      <c r="AB28" s="7" t="n"/>
+      <c r="B28" s="28" t="n"/>
+      <c r="AB28" s="29" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
-      <c r="F29" s="7" t="n"/>
-      <c r="G29" s="7" t="n"/>
-      <c r="H29" s="7" t="n"/>
-      <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="n"/>
-      <c r="K29" s="7" t="n"/>
-      <c r="L29" s="7" t="n"/>
-      <c r="M29" s="7" t="n"/>
-      <c r="N29" s="7" t="n"/>
-      <c r="O29" s="7" t="n"/>
-      <c r="P29" s="7" t="n"/>
-      <c r="Q29" s="7" t="n"/>
-      <c r="R29" s="7" t="n"/>
-      <c r="S29" s="7" t="n"/>
-      <c r="T29" s="7" t="n"/>
-      <c r="U29" s="7" t="n"/>
-      <c r="V29" s="7" t="n"/>
-      <c r="W29" s="7" t="n"/>
-      <c r="X29" s="7" t="n"/>
-      <c r="Y29" s="7" t="n"/>
-      <c r="Z29" s="7" t="n"/>
-      <c r="AA29" s="7" t="n"/>
-      <c r="AB29" s="7" t="n"/>
+      <c r="B29" s="30" t="n"/>
+      <c r="C29" s="31" t="n"/>
+      <c r="D29" s="31" t="n"/>
+      <c r="E29" s="31" t="n"/>
+      <c r="F29" s="31" t="n"/>
+      <c r="G29" s="31" t="n"/>
+      <c r="H29" s="31" t="n"/>
+      <c r="I29" s="31" t="n"/>
+      <c r="J29" s="31" t="n"/>
+      <c r="K29" s="31" t="n"/>
+      <c r="L29" s="31" t="n"/>
+      <c r="M29" s="31" t="n"/>
+      <c r="N29" s="31" t="n"/>
+      <c r="O29" s="31" t="n"/>
+      <c r="P29" s="31" t="n"/>
+      <c r="Q29" s="31" t="n"/>
+      <c r="R29" s="31" t="n"/>
+      <c r="S29" s="31" t="n"/>
+      <c r="T29" s="31" t="n"/>
+      <c r="U29" s="31" t="n"/>
+      <c r="V29" s="31" t="n"/>
+      <c r="W29" s="31" t="n"/>
+      <c r="X29" s="31" t="n"/>
+      <c r="Y29" s="31" t="n"/>
+      <c r="Z29" s="31" t="n"/>
+      <c r="AA29" s="31" t="n"/>
+      <c r="AB29" s="32" t="n"/>
     </row>
     <row r="30" ht="8" customHeight="1"/>
     <row r="31" ht="20" customHeight="1">
@@ -4713,32 +4584,6 @@
           <t>4. 보고 및 결재</t>
         </is>
       </c>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="n"/>
-      <c r="K31" s="5" t="n"/>
-      <c r="L31" s="5" t="n"/>
-      <c r="M31" s="5" t="n"/>
-      <c r="N31" s="5" t="n"/>
-      <c r="O31" s="5" t="n"/>
-      <c r="P31" s="5" t="n"/>
-      <c r="Q31" s="5" t="n"/>
-      <c r="R31" s="5" t="n"/>
-      <c r="S31" s="5" t="n"/>
-      <c r="T31" s="5" t="n"/>
-      <c r="U31" s="5" t="n"/>
-      <c r="V31" s="5" t="n"/>
-      <c r="W31" s="5" t="n"/>
-      <c r="X31" s="5" t="n"/>
-      <c r="Y31" s="5" t="n"/>
-      <c r="Z31" s="5" t="n"/>
-      <c r="AA31" s="5" t="n"/>
-      <c r="AB31" s="5" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="B32" s="13" t="inlineStr">
@@ -4746,41 +4591,41 @@
           <t>경영책임자</t>
         </is>
       </c>
-      <c r="C32" s="17" t="n"/>
-      <c r="D32" s="17" t="n"/>
-      <c r="E32" s="17" t="n"/>
-      <c r="F32" s="17" t="n"/>
-      <c r="G32" s="17" t="n"/>
-      <c r="H32" s="17" t="n"/>
-      <c r="I32" s="17" t="n"/>
-      <c r="J32" s="17" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="22" t="n"/>
+      <c r="F32" s="22" t="n"/>
+      <c r="G32" s="22" t="n"/>
+      <c r="H32" s="22" t="n"/>
+      <c r="I32" s="22" t="n"/>
+      <c r="J32" s="23" t="n"/>
       <c r="K32" s="13" t="inlineStr">
         <is>
           <t>현장소장
 (안전보건관리책임자)</t>
         </is>
       </c>
-      <c r="L32" s="17" t="n"/>
-      <c r="M32" s="17" t="n"/>
-      <c r="N32" s="17" t="n"/>
-      <c r="O32" s="17" t="n"/>
-      <c r="P32" s="17" t="n"/>
-      <c r="Q32" s="17" t="n"/>
-      <c r="R32" s="17" t="n"/>
-      <c r="S32" s="17" t="n"/>
+      <c r="L32" s="22" t="n"/>
+      <c r="M32" s="22" t="n"/>
+      <c r="N32" s="22" t="n"/>
+      <c r="O32" s="22" t="n"/>
+      <c r="P32" s="22" t="n"/>
+      <c r="Q32" s="22" t="n"/>
+      <c r="R32" s="22" t="n"/>
+      <c r="S32" s="23" t="n"/>
       <c r="T32" s="13" t="inlineStr">
         <is>
           <t>안전관리자</t>
         </is>
       </c>
-      <c r="U32" s="17" t="n"/>
-      <c r="V32" s="17" t="n"/>
-      <c r="W32" s="17" t="n"/>
-      <c r="X32" s="17" t="n"/>
-      <c r="Y32" s="17" t="n"/>
-      <c r="Z32" s="17" t="n"/>
-      <c r="AA32" s="17" t="n"/>
-      <c r="AB32" s="17" t="n"/>
+      <c r="U32" s="22" t="n"/>
+      <c r="V32" s="22" t="n"/>
+      <c r="W32" s="22" t="n"/>
+      <c r="X32" s="22" t="n"/>
+      <c r="Y32" s="22" t="n"/>
+      <c r="Z32" s="22" t="n"/>
+      <c r="AA32" s="22" t="n"/>
+      <c r="AB32" s="23" t="n"/>
     </row>
     <row r="33" ht="34" customHeight="1">
       <c r="B33" s="55" t="inlineStr">
@@ -4788,40 +4633,40 @@
           <t>(서명)</t>
         </is>
       </c>
-      <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="7" t="n"/>
-      <c r="G33" s="7" t="n"/>
-      <c r="H33" s="7" t="n"/>
-      <c r="I33" s="7" t="n"/>
-      <c r="J33" s="7" t="n"/>
+      <c r="C33" s="22" t="n"/>
+      <c r="D33" s="22" t="n"/>
+      <c r="E33" s="22" t="n"/>
+      <c r="F33" s="22" t="n"/>
+      <c r="G33" s="22" t="n"/>
+      <c r="H33" s="22" t="n"/>
+      <c r="I33" s="22" t="n"/>
+      <c r="J33" s="23" t="n"/>
       <c r="K33" s="55" t="inlineStr">
         <is>
           <t>(서명)</t>
         </is>
       </c>
-      <c r="L33" s="7" t="n"/>
-      <c r="M33" s="7" t="n"/>
-      <c r="N33" s="7" t="n"/>
-      <c r="O33" s="7" t="n"/>
-      <c r="P33" s="7" t="n"/>
-      <c r="Q33" s="7" t="n"/>
-      <c r="R33" s="7" t="n"/>
-      <c r="S33" s="7" t="n"/>
+      <c r="L33" s="22" t="n"/>
+      <c r="M33" s="22" t="n"/>
+      <c r="N33" s="22" t="n"/>
+      <c r="O33" s="22" t="n"/>
+      <c r="P33" s="22" t="n"/>
+      <c r="Q33" s="22" t="n"/>
+      <c r="R33" s="22" t="n"/>
+      <c r="S33" s="23" t="n"/>
       <c r="T33" s="55" t="inlineStr">
         <is>
           <t>(서명)</t>
         </is>
       </c>
-      <c r="U33" s="7" t="n"/>
-      <c r="V33" s="7" t="n"/>
-      <c r="W33" s="7" t="n"/>
-      <c r="X33" s="7" t="n"/>
-      <c r="Y33" s="7" t="n"/>
-      <c r="Z33" s="7" t="n"/>
-      <c r="AA33" s="7" t="n"/>
-      <c r="AB33" s="7" t="n"/>
+      <c r="U33" s="22" t="n"/>
+      <c r="V33" s="22" t="n"/>
+      <c r="W33" s="22" t="n"/>
+      <c r="X33" s="22" t="n"/>
+      <c r="Y33" s="22" t="n"/>
+      <c r="Z33" s="22" t="n"/>
+      <c r="AA33" s="22" t="n"/>
+      <c r="AB33" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="97">
@@ -4975,32 +4820,6 @@
           <t>지적사항 조치계획서</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
-      <c r="V2" s="2" t="n"/>
-      <c r="W2" s="2" t="n"/>
-      <c r="X2" s="2" t="n"/>
-      <c r="Y2" s="2" t="n"/>
-      <c r="Z2" s="2" t="n"/>
-      <c r="AA2" s="2" t="n"/>
-      <c r="AB2" s="2" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
@@ -5034,66 +4853,66 @@
           <t>No</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n"/>
+      <c r="C7" s="23" t="n"/>
       <c r="D7" s="9" t="inlineStr">
         <is>
           <t>지적사항</t>
         </is>
       </c>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="23" t="n"/>
       <c r="H7" s="9" t="inlineStr">
         <is>
           <t>원인분석</t>
         </is>
       </c>
-      <c r="I7" s="10" t="n"/>
-      <c r="J7" s="10" t="n"/>
-      <c r="K7" s="10" t="n"/>
+      <c r="I7" s="22" t="n"/>
+      <c r="J7" s="22" t="n"/>
+      <c r="K7" s="23" t="n"/>
       <c r="L7" s="9" t="inlineStr">
         <is>
           <t>개선대책
 (조치계획)</t>
         </is>
       </c>
-      <c r="M7" s="10" t="n"/>
-      <c r="N7" s="10" t="n"/>
-      <c r="O7" s="10" t="n"/>
+      <c r="M7" s="22" t="n"/>
+      <c r="N7" s="22" t="n"/>
+      <c r="O7" s="23" t="n"/>
       <c r="P7" s="9" t="inlineStr">
         <is>
           <t>담당부서
 /담당자</t>
         </is>
       </c>
-      <c r="Q7" s="10" t="n"/>
-      <c r="R7" s="10" t="n"/>
+      <c r="Q7" s="22" t="n"/>
+      <c r="R7" s="23" t="n"/>
       <c r="S7" s="9" t="inlineStr">
         <is>
           <t>조치예정일</t>
         </is>
       </c>
-      <c r="T7" s="10" t="n"/>
-      <c r="U7" s="10" t="n"/>
+      <c r="T7" s="22" t="n"/>
+      <c r="U7" s="23" t="n"/>
       <c r="V7" s="9" t="inlineStr">
         <is>
           <t>소요예산
 (원)</t>
         </is>
       </c>
-      <c r="W7" s="10" t="n"/>
+      <c r="W7" s="23" t="n"/>
       <c r="X7" s="9" t="inlineStr">
         <is>
           <t>진행상태</t>
         </is>
       </c>
-      <c r="Y7" s="10" t="n"/>
+      <c r="Y7" s="23" t="n"/>
       <c r="Z7" s="9" t="inlineStr">
         <is>
           <t>완료일</t>
         </is>
       </c>
-      <c r="AA7" s="10" t="n"/>
+      <c r="AA7" s="23" t="n"/>
       <c r="AB7" s="9" t="inlineStr">
         <is>
           <t>확인</t>
@@ -5104,217 +4923,217 @@
       <c r="B8" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="7" t="n"/>
+      <c r="C8" s="23" t="n"/>
       <c r="D8" s="14" t="inlineStr"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
+      <c r="E8" s="22" t="n"/>
+      <c r="F8" s="22" t="n"/>
+      <c r="G8" s="23" t="n"/>
       <c r="H8" s="14" t="inlineStr"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
+      <c r="I8" s="22" t="n"/>
+      <c r="J8" s="22" t="n"/>
+      <c r="K8" s="23" t="n"/>
       <c r="L8" s="14" t="inlineStr"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
+      <c r="M8" s="22" t="n"/>
+      <c r="N8" s="22" t="n"/>
+      <c r="O8" s="23" t="n"/>
       <c r="P8" s="14" t="inlineStr"/>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
+      <c r="Q8" s="22" t="n"/>
+      <c r="R8" s="23" t="n"/>
       <c r="S8" s="55" t="inlineStr"/>
-      <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="n"/>
+      <c r="T8" s="22" t="n"/>
+      <c r="U8" s="23" t="n"/>
       <c r="V8" s="55" t="inlineStr"/>
-      <c r="W8" s="7" t="n"/>
+      <c r="W8" s="23" t="n"/>
       <c r="X8" s="55" t="inlineStr"/>
-      <c r="Y8" s="7" t="n"/>
+      <c r="Y8" s="23" t="n"/>
       <c r="Z8" s="55" t="inlineStr"/>
-      <c r="AA8" s="7" t="n"/>
+      <c r="AA8" s="23" t="n"/>
       <c r="AB8" s="55" t="inlineStr"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="B9" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="7" t="n"/>
+      <c r="C9" s="23" t="n"/>
       <c r="D9" s="14" t="inlineStr"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="23" t="n"/>
       <c r="H9" s="14" t="inlineStr"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="22" t="n"/>
+      <c r="K9" s="23" t="n"/>
       <c r="L9" s="14" t="inlineStr"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="7" t="n"/>
+      <c r="M9" s="22" t="n"/>
+      <c r="N9" s="22" t="n"/>
+      <c r="O9" s="23" t="n"/>
       <c r="P9" s="14" t="inlineStr"/>
-      <c r="Q9" s="7" t="n"/>
-      <c r="R9" s="7" t="n"/>
+      <c r="Q9" s="22" t="n"/>
+      <c r="R9" s="23" t="n"/>
       <c r="S9" s="55" t="inlineStr"/>
-      <c r="T9" s="7" t="n"/>
-      <c r="U9" s="7" t="n"/>
+      <c r="T9" s="22" t="n"/>
+      <c r="U9" s="23" t="n"/>
       <c r="V9" s="55" t="inlineStr"/>
-      <c r="W9" s="7" t="n"/>
+      <c r="W9" s="23" t="n"/>
       <c r="X9" s="55" t="inlineStr"/>
-      <c r="Y9" s="7" t="n"/>
+      <c r="Y9" s="23" t="n"/>
       <c r="Z9" s="55" t="inlineStr"/>
-      <c r="AA9" s="7" t="n"/>
+      <c r="AA9" s="23" t="n"/>
       <c r="AB9" s="55" t="inlineStr"/>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="B10" s="55" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="7" t="n"/>
+      <c r="C10" s="23" t="n"/>
       <c r="D10" s="14" t="inlineStr"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="22" t="n"/>
+      <c r="G10" s="23" t="n"/>
       <c r="H10" s="14" t="inlineStr"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
+      <c r="I10" s="22" t="n"/>
+      <c r="J10" s="22" t="n"/>
+      <c r="K10" s="23" t="n"/>
       <c r="L10" s="14" t="inlineStr"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
-      <c r="O10" s="7" t="n"/>
+      <c r="M10" s="22" t="n"/>
+      <c r="N10" s="22" t="n"/>
+      <c r="O10" s="23" t="n"/>
       <c r="P10" s="14" t="inlineStr"/>
-      <c r="Q10" s="7" t="n"/>
-      <c r="R10" s="7" t="n"/>
+      <c r="Q10" s="22" t="n"/>
+      <c r="R10" s="23" t="n"/>
       <c r="S10" s="55" t="inlineStr"/>
-      <c r="T10" s="7" t="n"/>
-      <c r="U10" s="7" t="n"/>
+      <c r="T10" s="22" t="n"/>
+      <c r="U10" s="23" t="n"/>
       <c r="V10" s="55" t="inlineStr"/>
-      <c r="W10" s="7" t="n"/>
+      <c r="W10" s="23" t="n"/>
       <c r="X10" s="55" t="inlineStr"/>
-      <c r="Y10" s="7" t="n"/>
+      <c r="Y10" s="23" t="n"/>
       <c r="Z10" s="55" t="inlineStr"/>
-      <c r="AA10" s="7" t="n"/>
+      <c r="AA10" s="23" t="n"/>
       <c r="AB10" s="55" t="inlineStr"/>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="B11" s="55" t="n">
         <v>4</v>
       </c>
-      <c r="C11" s="7" t="n"/>
+      <c r="C11" s="23" t="n"/>
       <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
+      <c r="E11" s="22" t="n"/>
+      <c r="F11" s="22" t="n"/>
+      <c r="G11" s="23" t="n"/>
       <c r="H11" s="14" t="inlineStr"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
+      <c r="I11" s="22" t="n"/>
+      <c r="J11" s="22" t="n"/>
+      <c r="K11" s="23" t="n"/>
       <c r="L11" s="14" t="inlineStr"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
-      <c r="O11" s="7" t="n"/>
+      <c r="M11" s="22" t="n"/>
+      <c r="N11" s="22" t="n"/>
+      <c r="O11" s="23" t="n"/>
       <c r="P11" s="14" t="inlineStr"/>
-      <c r="Q11" s="7" t="n"/>
-      <c r="R11" s="7" t="n"/>
+      <c r="Q11" s="22" t="n"/>
+      <c r="R11" s="23" t="n"/>
       <c r="S11" s="55" t="inlineStr"/>
-      <c r="T11" s="7" t="n"/>
-      <c r="U11" s="7" t="n"/>
+      <c r="T11" s="22" t="n"/>
+      <c r="U11" s="23" t="n"/>
       <c r="V11" s="55" t="inlineStr"/>
-      <c r="W11" s="7" t="n"/>
+      <c r="W11" s="23" t="n"/>
       <c r="X11" s="55" t="inlineStr"/>
-      <c r="Y11" s="7" t="n"/>
+      <c r="Y11" s="23" t="n"/>
       <c r="Z11" s="55" t="inlineStr"/>
-      <c r="AA11" s="7" t="n"/>
+      <c r="AA11" s="23" t="n"/>
       <c r="AB11" s="55" t="inlineStr"/>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="B12" s="55" t="n">
         <v>5</v>
       </c>
-      <c r="C12" s="7" t="n"/>
+      <c r="C12" s="23" t="n"/>
       <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
+      <c r="E12" s="22" t="n"/>
+      <c r="F12" s="22" t="n"/>
+      <c r="G12" s="23" t="n"/>
       <c r="H12" s="14" t="inlineStr"/>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
-      <c r="K12" s="7" t="n"/>
+      <c r="I12" s="22" t="n"/>
+      <c r="J12" s="22" t="n"/>
+      <c r="K12" s="23" t="n"/>
       <c r="L12" s="14" t="inlineStr"/>
-      <c r="M12" s="7" t="n"/>
-      <c r="N12" s="7" t="n"/>
-      <c r="O12" s="7" t="n"/>
+      <c r="M12" s="22" t="n"/>
+      <c r="N12" s="22" t="n"/>
+      <c r="O12" s="23" t="n"/>
       <c r="P12" s="14" t="inlineStr"/>
-      <c r="Q12" s="7" t="n"/>
-      <c r="R12" s="7" t="n"/>
+      <c r="Q12" s="22" t="n"/>
+      <c r="R12" s="23" t="n"/>
       <c r="S12" s="55" t="inlineStr"/>
-      <c r="T12" s="7" t="n"/>
-      <c r="U12" s="7" t="n"/>
+      <c r="T12" s="22" t="n"/>
+      <c r="U12" s="23" t="n"/>
       <c r="V12" s="55" t="inlineStr"/>
-      <c r="W12" s="7" t="n"/>
+      <c r="W12" s="23" t="n"/>
       <c r="X12" s="55" t="inlineStr"/>
-      <c r="Y12" s="7" t="n"/>
+      <c r="Y12" s="23" t="n"/>
       <c r="Z12" s="55" t="inlineStr"/>
-      <c r="AA12" s="7" t="n"/>
+      <c r="AA12" s="23" t="n"/>
       <c r="AB12" s="55" t="inlineStr"/>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="B13" s="55" t="n">
         <v>6</v>
       </c>
-      <c r="C13" s="7" t="n"/>
+      <c r="C13" s="23" t="n"/>
       <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
+      <c r="E13" s="22" t="n"/>
+      <c r="F13" s="22" t="n"/>
+      <c r="G13" s="23" t="n"/>
       <c r="H13" s="14" t="inlineStr"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
-      <c r="K13" s="7" t="n"/>
+      <c r="I13" s="22" t="n"/>
+      <c r="J13" s="22" t="n"/>
+      <c r="K13" s="23" t="n"/>
       <c r="L13" s="14" t="inlineStr"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="n"/>
+      <c r="M13" s="22" t="n"/>
+      <c r="N13" s="22" t="n"/>
+      <c r="O13" s="23" t="n"/>
       <c r="P13" s="14" t="inlineStr"/>
-      <c r="Q13" s="7" t="n"/>
-      <c r="R13" s="7" t="n"/>
+      <c r="Q13" s="22" t="n"/>
+      <c r="R13" s="23" t="n"/>
       <c r="S13" s="55" t="inlineStr"/>
-      <c r="T13" s="7" t="n"/>
-      <c r="U13" s="7" t="n"/>
+      <c r="T13" s="22" t="n"/>
+      <c r="U13" s="23" t="n"/>
       <c r="V13" s="55" t="inlineStr"/>
-      <c r="W13" s="7" t="n"/>
+      <c r="W13" s="23" t="n"/>
       <c r="X13" s="55" t="inlineStr"/>
-      <c r="Y13" s="7" t="n"/>
+      <c r="Y13" s="23" t="n"/>
       <c r="Z13" s="55" t="inlineStr"/>
-      <c r="AA13" s="7" t="n"/>
+      <c r="AA13" s="23" t="n"/>
       <c r="AB13" s="55" t="inlineStr"/>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="B14" s="55" t="n">
         <v>7</v>
       </c>
-      <c r="C14" s="7" t="n"/>
+      <c r="C14" s="23" t="n"/>
       <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
+      <c r="E14" s="22" t="n"/>
+      <c r="F14" s="22" t="n"/>
+      <c r="G14" s="23" t="n"/>
       <c r="H14" s="14" t="inlineStr"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="n"/>
-      <c r="K14" s="7" t="n"/>
+      <c r="I14" s="22" t="n"/>
+      <c r="J14" s="22" t="n"/>
+      <c r="K14" s="23" t="n"/>
       <c r="L14" s="14" t="inlineStr"/>
-      <c r="M14" s="7" t="n"/>
-      <c r="N14" s="7" t="n"/>
-      <c r="O14" s="7" t="n"/>
+      <c r="M14" s="22" t="n"/>
+      <c r="N14" s="22" t="n"/>
+      <c r="O14" s="23" t="n"/>
       <c r="P14" s="14" t="inlineStr"/>
-      <c r="Q14" s="7" t="n"/>
-      <c r="R14" s="7" t="n"/>
+      <c r="Q14" s="22" t="n"/>
+      <c r="R14" s="23" t="n"/>
       <c r="S14" s="55" t="inlineStr"/>
-      <c r="T14" s="7" t="n"/>
-      <c r="U14" s="7" t="n"/>
+      <c r="T14" s="22" t="n"/>
+      <c r="U14" s="23" t="n"/>
       <c r="V14" s="55" t="inlineStr"/>
-      <c r="W14" s="7" t="n"/>
+      <c r="W14" s="23" t="n"/>
       <c r="X14" s="55" t="inlineStr"/>
-      <c r="Y14" s="7" t="n"/>
+      <c r="Y14" s="23" t="n"/>
       <c r="Z14" s="55" t="inlineStr"/>
-      <c r="AA14" s="7" t="n"/>
+      <c r="AA14" s="23" t="n"/>
       <c r="AB14" s="55" t="inlineStr"/>
     </row>
     <row r="15" ht="8" customHeight="1"/>
@@ -5332,35 +5151,35 @@
           <t>작성자</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n"/>
-      <c r="D18" s="17" t="n"/>
-      <c r="E18" s="17" t="n"/>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="22" t="n"/>
+      <c r="E18" s="23" t="n"/>
       <c r="F18" s="55" t="inlineStr"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="n"/>
-      <c r="N18" s="7" t="n"/>
+      <c r="G18" s="22" t="n"/>
+      <c r="H18" s="22" t="n"/>
+      <c r="I18" s="22" t="n"/>
+      <c r="J18" s="22" t="n"/>
+      <c r="K18" s="22" t="n"/>
+      <c r="L18" s="22" t="n"/>
+      <c r="M18" s="22" t="n"/>
+      <c r="N18" s="23" t="n"/>
       <c r="P18" s="13" t="inlineStr">
         <is>
           <t>승인(결재)자</t>
         </is>
       </c>
-      <c r="Q18" s="17" t="n"/>
-      <c r="R18" s="17" t="n"/>
-      <c r="S18" s="17" t="n"/>
+      <c r="Q18" s="22" t="n"/>
+      <c r="R18" s="22" t="n"/>
+      <c r="S18" s="23" t="n"/>
       <c r="T18" s="55" t="inlineStr"/>
-      <c r="U18" s="7" t="n"/>
-      <c r="V18" s="7" t="n"/>
-      <c r="W18" s="7" t="n"/>
-      <c r="X18" s="7" t="n"/>
-      <c r="Y18" s="7" t="n"/>
-      <c r="Z18" s="7" t="n"/>
-      <c r="AA18" s="7" t="n"/>
-      <c r="AB18" s="7" t="n"/>
+      <c r="U18" s="22" t="n"/>
+      <c r="V18" s="22" t="n"/>
+      <c r="W18" s="22" t="n"/>
+      <c r="X18" s="22" t="n"/>
+      <c r="Y18" s="22" t="n"/>
+      <c r="Z18" s="22" t="n"/>
+      <c r="AA18" s="22" t="n"/>
+      <c r="AB18" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="91">
@@ -5431,8 +5250,8 @@
     <mergeCell ref="S7:U7"/>
     <mergeCell ref="X12:Y12"/>
     <mergeCell ref="P11:R11"/>
+    <mergeCell ref="D12:G12"/>
     <mergeCell ref="L9:O9"/>
-    <mergeCell ref="D12:G12"/>
     <mergeCell ref="AB13"/>
     <mergeCell ref="AB7"/>
     <mergeCell ref="V14:W14"/>
@@ -5459,4 +5278,878 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF305496"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:AB30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4.6" customWidth="1" min="2" max="2"/>
+    <col width="4.6" customWidth="1" min="3" max="3"/>
+    <col width="4.6" customWidth="1" min="4" max="4"/>
+    <col width="4.6" customWidth="1" min="5" max="5"/>
+    <col width="4.6" customWidth="1" min="6" max="6"/>
+    <col width="4.6" customWidth="1" min="7" max="7"/>
+    <col width="4.6" customWidth="1" min="8" max="8"/>
+    <col width="4.6" customWidth="1" min="9" max="9"/>
+    <col width="4.6" customWidth="1" min="10" max="10"/>
+    <col width="4.6" customWidth="1" min="11" max="11"/>
+    <col width="4.6" customWidth="1" min="12" max="12"/>
+    <col width="4.6" customWidth="1" min="13" max="13"/>
+    <col width="4.6" customWidth="1" min="14" max="14"/>
+    <col width="4.6" customWidth="1" min="15" max="15"/>
+    <col width="4.6" customWidth="1" min="16" max="16"/>
+    <col width="4.6" customWidth="1" min="17" max="17"/>
+    <col width="4.6" customWidth="1" min="18" max="18"/>
+    <col width="4.6" customWidth="1" min="19" max="19"/>
+    <col width="4.6" customWidth="1" min="20" max="20"/>
+    <col width="4.6" customWidth="1" min="21" max="21"/>
+    <col width="4.6" customWidth="1" min="22" max="22"/>
+    <col width="4.6" customWidth="1" min="23" max="23"/>
+    <col width="4.6" customWidth="1" min="24" max="24"/>
+    <col width="4.6" customWidth="1" min="25" max="25"/>
+    <col width="4.6" customWidth="1" min="26" max="26"/>
+    <col width="4.6" customWidth="1" min="27" max="27"/>
+    <col width="4.6" customWidth="1" min="28" max="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="6" customHeight="1"/>
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>지적사항 조치 결과보고서</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+      <c r="Z2" s="2" t="n"/>
+      <c r="AA2" s="2" t="n"/>
+      <c r="AB2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>(조치계획서에 따른 지적사항별 이행결과 확인 - 완료 여부, 조치내용, 증빙사진 확인)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="8" customHeight="1"/>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>현장(사업장)명:</t>
+        </is>
+      </c>
+      <c r="D5" s="54">
+        <f>'현장순회점검표'!F6</f>
+        <v/>
+      </c>
+      <c r="N5" s="52" t="inlineStr">
+        <is>
+          <t>확인일자:</t>
+        </is>
+      </c>
+      <c r="P5" s="53" t="inlineStr"/>
+      <c r="W5" s="52" t="inlineStr">
+        <is>
+          <t>확인자:</t>
+        </is>
+      </c>
+      <c r="Y5" s="53" t="inlineStr"/>
+    </row>
+    <row r="6" ht="8" customHeight="1"/>
+    <row r="7" ht="20" customHeight="1">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>1. 조치 이행결과 총괄</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="5" t="n"/>
+      <c r="Q7" s="5" t="n"/>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="5" t="n"/>
+      <c r="T7" s="5" t="n"/>
+      <c r="U7" s="5" t="n"/>
+      <c r="V7" s="5" t="n"/>
+      <c r="W7" s="5" t="n"/>
+      <c r="X7" s="5" t="n"/>
+      <c r="Y7" s="5" t="n"/>
+      <c r="Z7" s="5" t="n"/>
+      <c r="AA7" s="5" t="n"/>
+      <c r="AB7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="58" t="inlineStr">
+        <is>
+          <t>지적사항 총 건수</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
+      <c r="H8" s="10" t="n"/>
+      <c r="I8" s="10" t="n"/>
+      <c r="J8" s="58" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="n"/>
+      <c r="L8" s="10" t="n"/>
+      <c r="M8" s="10" t="n"/>
+      <c r="N8" s="10" t="n"/>
+      <c r="O8" s="10" t="n"/>
+      <c r="P8" s="58" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="Q8" s="10" t="n"/>
+      <c r="R8" s="10" t="n"/>
+      <c r="S8" s="10" t="n"/>
+      <c r="T8" s="10" t="n"/>
+      <c r="U8" s="10" t="n"/>
+      <c r="V8" s="58" t="inlineStr">
+        <is>
+          <t>미완료(보류)</t>
+        </is>
+      </c>
+      <c r="W8" s="10" t="n"/>
+      <c r="X8" s="10" t="n"/>
+      <c r="Y8" s="10" t="n"/>
+      <c r="Z8" s="10" t="n"/>
+      <c r="AA8" s="10" t="n"/>
+      <c r="AB8" s="10" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="59" t="inlineStr"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="59" t="inlineStr"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="7" t="n"/>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="59" t="inlineStr"/>
+      <c r="Q9" s="7" t="n"/>
+      <c r="R9" s="7" t="n"/>
+      <c r="S9" s="7" t="n"/>
+      <c r="T9" s="7" t="n"/>
+      <c r="U9" s="7" t="n"/>
+      <c r="V9" s="59" t="inlineStr"/>
+      <c r="W9" s="7" t="n"/>
+      <c r="X9" s="7" t="n"/>
+      <c r="Y9" s="7" t="n"/>
+      <c r="Z9" s="7" t="n"/>
+      <c r="AA9" s="7" t="n"/>
+      <c r="AB9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="8" customHeight="1"/>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>2. 지적사항별 조치 결과</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="5" t="n"/>
+      <c r="O11" s="5" t="n"/>
+      <c r="P11" s="5" t="n"/>
+      <c r="Q11" s="5" t="n"/>
+      <c r="R11" s="5" t="n"/>
+      <c r="S11" s="5" t="n"/>
+      <c r="T11" s="5" t="n"/>
+      <c r="U11" s="5" t="n"/>
+      <c r="V11" s="5" t="n"/>
+      <c r="W11" s="5" t="n"/>
+      <c r="X11" s="5" t="n"/>
+      <c r="Y11" s="5" t="n"/>
+      <c r="Z11" s="5" t="n"/>
+      <c r="AA11" s="5" t="n"/>
+      <c r="AB11" s="5" t="n"/>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="B12" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="58" t="inlineStr">
+        <is>
+          <t>지적사항</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
+      <c r="H12" s="10" t="n"/>
+      <c r="I12" s="58" t="inlineStr">
+        <is>
+          <t>조치계획
+(요약)</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="n"/>
+      <c r="K12" s="10" t="n"/>
+      <c r="L12" s="10" t="n"/>
+      <c r="M12" s="10" t="n"/>
+      <c r="N12" s="58" t="inlineStr">
+        <is>
+          <t>조치결과 내용</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="n"/>
+      <c r="P12" s="10" t="n"/>
+      <c r="Q12" s="10" t="n"/>
+      <c r="R12" s="58" t="inlineStr">
+        <is>
+          <t>완료여부
+(완료/진행중/보류)</t>
+        </is>
+      </c>
+      <c r="S12" s="10" t="n"/>
+      <c r="T12" s="10" t="n"/>
+      <c r="U12" s="58" t="inlineStr">
+        <is>
+          <t>완료일</t>
+        </is>
+      </c>
+      <c r="V12" s="10" t="n"/>
+      <c r="W12" s="58" t="inlineStr">
+        <is>
+          <t>증빙사진
+(첨부 여부)</t>
+        </is>
+      </c>
+      <c r="X12" s="10" t="n"/>
+      <c r="Y12" s="10" t="n"/>
+      <c r="Z12" s="58" t="inlineStr">
+        <is>
+          <t>확인자</t>
+        </is>
+      </c>
+      <c r="AA12" s="10" t="n"/>
+      <c r="AB12" s="10" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="B13" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="60" t="inlineStr"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="60" t="inlineStr"/>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="60" t="inlineStr"/>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="7" t="n"/>
+      <c r="Q13" s="7" t="n"/>
+      <c r="R13" s="59" t="inlineStr"/>
+      <c r="S13" s="7" t="n"/>
+      <c r="T13" s="7" t="n"/>
+      <c r="U13" s="59" t="inlineStr"/>
+      <c r="V13" s="7" t="n"/>
+      <c r="W13" s="59" t="inlineStr"/>
+      <c r="X13" s="7" t="n"/>
+      <c r="Y13" s="7" t="n"/>
+      <c r="Z13" s="59" t="inlineStr"/>
+      <c r="AA13" s="7" t="n"/>
+      <c r="AB13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="B14" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="60" t="inlineStr"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="60" t="inlineStr"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="n"/>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="60" t="inlineStr"/>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="7" t="n"/>
+      <c r="Q14" s="7" t="n"/>
+      <c r="R14" s="59" t="inlineStr"/>
+      <c r="S14" s="7" t="n"/>
+      <c r="T14" s="7" t="n"/>
+      <c r="U14" s="59" t="inlineStr"/>
+      <c r="V14" s="7" t="n"/>
+      <c r="W14" s="59" t="inlineStr"/>
+      <c r="X14" s="7" t="n"/>
+      <c r="Y14" s="7" t="n"/>
+      <c r="Z14" s="59" t="inlineStr"/>
+      <c r="AA14" s="7" t="n"/>
+      <c r="AB14" s="7" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="B15" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="60" t="inlineStr"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="60" t="inlineStr"/>
+      <c r="J15" s="7" t="n"/>
+      <c r="K15" s="7" t="n"/>
+      <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="60" t="inlineStr"/>
+      <c r="O15" s="7" t="n"/>
+      <c r="P15" s="7" t="n"/>
+      <c r="Q15" s="7" t="n"/>
+      <c r="R15" s="59" t="inlineStr"/>
+      <c r="S15" s="7" t="n"/>
+      <c r="T15" s="7" t="n"/>
+      <c r="U15" s="59" t="inlineStr"/>
+      <c r="V15" s="7" t="n"/>
+      <c r="W15" s="59" t="inlineStr"/>
+      <c r="X15" s="7" t="n"/>
+      <c r="Y15" s="7" t="n"/>
+      <c r="Z15" s="59" t="inlineStr"/>
+      <c r="AA15" s="7" t="n"/>
+      <c r="AB15" s="7" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="B16" s="59" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="60" t="inlineStr"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="60" t="inlineStr"/>
+      <c r="J16" s="7" t="n"/>
+      <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n"/>
+      <c r="M16" s="7" t="n"/>
+      <c r="N16" s="60" t="inlineStr"/>
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" s="7" t="n"/>
+      <c r="Q16" s="7" t="n"/>
+      <c r="R16" s="59" t="inlineStr"/>
+      <c r="S16" s="7" t="n"/>
+      <c r="T16" s="7" t="n"/>
+      <c r="U16" s="59" t="inlineStr"/>
+      <c r="V16" s="7" t="n"/>
+      <c r="W16" s="59" t="inlineStr"/>
+      <c r="X16" s="7" t="n"/>
+      <c r="Y16" s="7" t="n"/>
+      <c r="Z16" s="59" t="inlineStr"/>
+      <c r="AA16" s="7" t="n"/>
+      <c r="AB16" s="7" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="B17" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="60" t="inlineStr"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="60" t="inlineStr"/>
+      <c r="J17" s="7" t="n"/>
+      <c r="K17" s="7" t="n"/>
+      <c r="L17" s="7" t="n"/>
+      <c r="M17" s="7" t="n"/>
+      <c r="N17" s="60" t="inlineStr"/>
+      <c r="O17" s="7" t="n"/>
+      <c r="P17" s="7" t="n"/>
+      <c r="Q17" s="7" t="n"/>
+      <c r="R17" s="59" t="inlineStr"/>
+      <c r="S17" s="7" t="n"/>
+      <c r="T17" s="7" t="n"/>
+      <c r="U17" s="59" t="inlineStr"/>
+      <c r="V17" s="7" t="n"/>
+      <c r="W17" s="59" t="inlineStr"/>
+      <c r="X17" s="7" t="n"/>
+      <c r="Y17" s="7" t="n"/>
+      <c r="Z17" s="59" t="inlineStr"/>
+      <c r="AA17" s="7" t="n"/>
+      <c r="AB17" s="7" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="B18" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="60" t="inlineStr"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="60" t="inlineStr"/>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="60" t="inlineStr"/>
+      <c r="O18" s="7" t="n"/>
+      <c r="P18" s="7" t="n"/>
+      <c r="Q18" s="7" t="n"/>
+      <c r="R18" s="59" t="inlineStr"/>
+      <c r="S18" s="7" t="n"/>
+      <c r="T18" s="7" t="n"/>
+      <c r="U18" s="59" t="inlineStr"/>
+      <c r="V18" s="7" t="n"/>
+      <c r="W18" s="59" t="inlineStr"/>
+      <c r="X18" s="7" t="n"/>
+      <c r="Y18" s="7" t="n"/>
+      <c r="Z18" s="59" t="inlineStr"/>
+      <c r="AA18" s="7" t="n"/>
+      <c r="AB18" s="7" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="B19" s="59" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="60" t="inlineStr"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="60" t="inlineStr"/>
+      <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="n"/>
+      <c r="N19" s="60" t="inlineStr"/>
+      <c r="O19" s="7" t="n"/>
+      <c r="P19" s="7" t="n"/>
+      <c r="Q19" s="7" t="n"/>
+      <c r="R19" s="59" t="inlineStr"/>
+      <c r="S19" s="7" t="n"/>
+      <c r="T19" s="7" t="n"/>
+      <c r="U19" s="59" t="inlineStr"/>
+      <c r="V19" s="7" t="n"/>
+      <c r="W19" s="59" t="inlineStr"/>
+      <c r="X19" s="7" t="n"/>
+      <c r="Y19" s="7" t="n"/>
+      <c r="Z19" s="59" t="inlineStr"/>
+      <c r="AA19" s="7" t="n"/>
+      <c r="AB19" s="7" t="n"/>
+    </row>
+    <row r="20" ht="8" customHeight="1"/>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>3. 종합의견 및 향후계획</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="5" t="n"/>
+      <c r="I21" s="5" t="n"/>
+      <c r="J21" s="5" t="n"/>
+      <c r="K21" s="5" t="n"/>
+      <c r="L21" s="5" t="n"/>
+      <c r="M21" s="5" t="n"/>
+      <c r="N21" s="5" t="n"/>
+      <c r="O21" s="5" t="n"/>
+      <c r="P21" s="5" t="n"/>
+      <c r="Q21" s="5" t="n"/>
+      <c r="R21" s="5" t="n"/>
+      <c r="S21" s="5" t="n"/>
+      <c r="T21" s="5" t="n"/>
+      <c r="U21" s="5" t="n"/>
+      <c r="V21" s="5" t="n"/>
+      <c r="W21" s="5" t="n"/>
+      <c r="X21" s="5" t="n"/>
+      <c r="Y21" s="5" t="n"/>
+      <c r="Z21" s="5" t="n"/>
+      <c r="AA21" s="5" t="n"/>
+      <c r="AB21" s="5" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="61" t="inlineStr"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="7" t="n"/>
+      <c r="K22" s="7" t="n"/>
+      <c r="L22" s="7" t="n"/>
+      <c r="M22" s="7" t="n"/>
+      <c r="N22" s="7" t="n"/>
+      <c r="O22" s="7" t="n"/>
+      <c r="P22" s="7" t="n"/>
+      <c r="Q22" s="7" t="n"/>
+      <c r="R22" s="7" t="n"/>
+      <c r="S22" s="7" t="n"/>
+      <c r="T22" s="7" t="n"/>
+      <c r="U22" s="7" t="n"/>
+      <c r="V22" s="7" t="n"/>
+      <c r="W22" s="7" t="n"/>
+      <c r="X22" s="7" t="n"/>
+      <c r="Y22" s="7" t="n"/>
+      <c r="Z22" s="7" t="n"/>
+      <c r="AA22" s="7" t="n"/>
+      <c r="AB22" s="7" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="7" t="n"/>
+      <c r="K23" s="7" t="n"/>
+      <c r="L23" s="7" t="n"/>
+      <c r="M23" s="7" t="n"/>
+      <c r="N23" s="7" t="n"/>
+      <c r="O23" s="7" t="n"/>
+      <c r="P23" s="7" t="n"/>
+      <c r="Q23" s="7" t="n"/>
+      <c r="R23" s="7" t="n"/>
+      <c r="S23" s="7" t="n"/>
+      <c r="T23" s="7" t="n"/>
+      <c r="U23" s="7" t="n"/>
+      <c r="V23" s="7" t="n"/>
+      <c r="W23" s="7" t="n"/>
+      <c r="X23" s="7" t="n"/>
+      <c r="Y23" s="7" t="n"/>
+      <c r="Z23" s="7" t="n"/>
+      <c r="AA23" s="7" t="n"/>
+      <c r="AB23" s="7" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="7" t="n"/>
+      <c r="I24" s="7" t="n"/>
+      <c r="J24" s="7" t="n"/>
+      <c r="K24" s="7" t="n"/>
+      <c r="L24" s="7" t="n"/>
+      <c r="M24" s="7" t="n"/>
+      <c r="N24" s="7" t="n"/>
+      <c r="O24" s="7" t="n"/>
+      <c r="P24" s="7" t="n"/>
+      <c r="Q24" s="7" t="n"/>
+      <c r="R24" s="7" t="n"/>
+      <c r="S24" s="7" t="n"/>
+      <c r="T24" s="7" t="n"/>
+      <c r="U24" s="7" t="n"/>
+      <c r="V24" s="7" t="n"/>
+      <c r="W24" s="7" t="n"/>
+      <c r="X24" s="7" t="n"/>
+      <c r="Y24" s="7" t="n"/>
+      <c r="Z24" s="7" t="n"/>
+      <c r="AA24" s="7" t="n"/>
+      <c r="AB24" s="7" t="n"/>
+    </row>
+    <row r="25" ht="8" customHeight="1"/>
+    <row r="26" ht="16" customHeight="1">
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>※ '완료' 처리 항목은 지적사항_조치전후사진대지 시트에 조치 전(Before)/조치 후(After) 사진을 첨부하여 근거로 보관한다. '보류' 항목은 사유를 종합의견에 기재하고 다음 순회점검 시 재확인한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="8" customHeight="1"/>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>4. 최종 확인</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="5" t="n"/>
+      <c r="I28" s="5" t="n"/>
+      <c r="J28" s="5" t="n"/>
+      <c r="K28" s="5" t="n"/>
+      <c r="L28" s="5" t="n"/>
+      <c r="M28" s="5" t="n"/>
+      <c r="N28" s="5" t="n"/>
+      <c r="O28" s="5" t="n"/>
+      <c r="P28" s="5" t="n"/>
+      <c r="Q28" s="5" t="n"/>
+      <c r="R28" s="5" t="n"/>
+      <c r="S28" s="5" t="n"/>
+      <c r="T28" s="5" t="n"/>
+      <c r="U28" s="5" t="n"/>
+      <c r="V28" s="5" t="n"/>
+      <c r="W28" s="5" t="n"/>
+      <c r="X28" s="5" t="n"/>
+      <c r="Y28" s="5" t="n"/>
+      <c r="Z28" s="5" t="n"/>
+      <c r="AA28" s="5" t="n"/>
+      <c r="AB28" s="5" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>경영책임자</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="n"/>
+      <c r="D29" s="17" t="n"/>
+      <c r="E29" s="17" t="n"/>
+      <c r="F29" s="17" t="n"/>
+      <c r="G29" s="17" t="n"/>
+      <c r="H29" s="17" t="n"/>
+      <c r="I29" s="17" t="n"/>
+      <c r="J29" s="17" t="n"/>
+      <c r="K29" s="13" t="inlineStr">
+        <is>
+          <t>현장소장
+(안전보건관리책임자)</t>
+        </is>
+      </c>
+      <c r="L29" s="17" t="n"/>
+      <c r="M29" s="17" t="n"/>
+      <c r="N29" s="17" t="n"/>
+      <c r="O29" s="17" t="n"/>
+      <c r="P29" s="17" t="n"/>
+      <c r="Q29" s="17" t="n"/>
+      <c r="R29" s="17" t="n"/>
+      <c r="S29" s="17" t="n"/>
+      <c r="T29" s="13" t="inlineStr">
+        <is>
+          <t>안전관리자</t>
+        </is>
+      </c>
+      <c r="U29" s="17" t="n"/>
+      <c r="V29" s="17" t="n"/>
+      <c r="W29" s="17" t="n"/>
+      <c r="X29" s="17" t="n"/>
+      <c r="Y29" s="17" t="n"/>
+      <c r="Z29" s="17" t="n"/>
+      <c r="AA29" s="17" t="n"/>
+      <c r="AB29" s="17" t="n"/>
+    </row>
+    <row r="30" ht="34" customHeight="1">
+      <c r="B30" s="59" t="inlineStr">
+        <is>
+          <t>(서명)</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="n"/>
+      <c r="H30" s="7" t="n"/>
+      <c r="I30" s="7" t="n"/>
+      <c r="J30" s="7" t="n"/>
+      <c r="K30" s="59" t="inlineStr">
+        <is>
+          <t>(서명)</t>
+        </is>
+      </c>
+      <c r="L30" s="7" t="n"/>
+      <c r="M30" s="7" t="n"/>
+      <c r="N30" s="7" t="n"/>
+      <c r="O30" s="7" t="n"/>
+      <c r="P30" s="7" t="n"/>
+      <c r="Q30" s="7" t="n"/>
+      <c r="R30" s="7" t="n"/>
+      <c r="S30" s="7" t="n"/>
+      <c r="T30" s="59" t="inlineStr">
+        <is>
+          <t>(서명)</t>
+        </is>
+      </c>
+      <c r="U30" s="7" t="n"/>
+      <c r="V30" s="7" t="n"/>
+      <c r="W30" s="7" t="n"/>
+      <c r="X30" s="7" t="n"/>
+      <c r="Y30" s="7" t="n"/>
+      <c r="Z30" s="7" t="n"/>
+      <c r="AA30" s="7" t="n"/>
+      <c r="AB30" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="92">
+    <mergeCell ref="P8:U8"/>
+    <mergeCell ref="B21:AB21"/>
+    <mergeCell ref="U15:V15"/>
+    <mergeCell ref="Z18:AB18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="Z17:AB17"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="W16:Y16"/>
+    <mergeCell ref="U16:V16"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="W18:Y18"/>
+    <mergeCell ref="N5:O5"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="V8:AB8"/>
+    <mergeCell ref="R14:T14"/>
+    <mergeCell ref="N12:Q12"/>
+    <mergeCell ref="K30:S30"/>
+    <mergeCell ref="I17:M17"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="N14:Q14"/>
+    <mergeCell ref="V9:AB9"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="I19:M19"/>
+    <mergeCell ref="J9:O9"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B11:AB11"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B29:J29"/>
+    <mergeCell ref="W12:Y12"/>
+    <mergeCell ref="R17:T17"/>
+    <mergeCell ref="N16:Q16"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="I12:M12"/>
+    <mergeCell ref="Z19:AB19"/>
+    <mergeCell ref="I14:M14"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="U18:V18"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="B26:AB26"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="T29:AB29"/>
+    <mergeCell ref="B7:AB7"/>
+    <mergeCell ref="R13:T13"/>
+    <mergeCell ref="B3:AB3"/>
+    <mergeCell ref="P9:U9"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="U19:V19"/>
+    <mergeCell ref="K29:S29"/>
+    <mergeCell ref="R15:T15"/>
+    <mergeCell ref="N13:Q13"/>
+    <mergeCell ref="B2:AB2"/>
+    <mergeCell ref="R12:T12"/>
+    <mergeCell ref="N15:Q15"/>
+    <mergeCell ref="W5:X5"/>
+    <mergeCell ref="B28:AB28"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="U12:V12"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="D5:L5"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="N18:Q18"/>
+    <mergeCell ref="T30:AB30"/>
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="R19:T19"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="N17:Q17"/>
+    <mergeCell ref="I13:M13"/>
+    <mergeCell ref="B22:AB24"/>
+    <mergeCell ref="N19:Q19"/>
+    <mergeCell ref="I15:M15"/>
+    <mergeCell ref="Z12:AB12"/>
+    <mergeCell ref="U17:V17"/>
+    <mergeCell ref="Z14:AB14"/>
+    <mergeCell ref="I16:M16"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="Z13:AB13"/>
+    <mergeCell ref="W17:Y17"/>
+    <mergeCell ref="I18:M18"/>
+    <mergeCell ref="Z15:AB15"/>
+    <mergeCell ref="P5:U5"/>
+    <mergeCell ref="R18:T18"/>
+    <mergeCell ref="W19:Y19"/>
+    <mergeCell ref="Y5:AB5"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="Z16:AB16"/>
+    <mergeCell ref="R16:T16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>